<commit_message>
Resultados con 35 nodos y beam search =7 con gap estocastico de 3.1% y det 7.7%
</commit_message>
<xml_diff>
--- a/results_35nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_35nodes/DRL_Routing_Summary_AM.xlsx
@@ -11,7 +11,6 @@
     <sheet name="Per Node Results" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Stochastic Descriptive Stats" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Wilcoxon Significance" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="PPO Convergence" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,12 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00&quot;%&quot;"/>
-    <numFmt numFmtId="165" formatCode="0.000000"/>
-    <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,27 +43,8 @@
     <font>
       <b val="1"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <color rgb="00000000"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00548235"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00548235"/>
-      <sz val="12"/>
-    </font>
   </fonts>
-  <fills count="16">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -111,36 +89,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C55A11"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00595959"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00404040"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00833C00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -190,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -254,56 +202,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -724,7 +622,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>33.2845097496396</v>
+        <v>32.4363594963437</v>
       </c>
     </row>
     <row r="4">
@@ -734,13 +632,13 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>3931.723809523809</v>
+        <v>4183.628571428571</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>12.9201028037663</v>
+        <v>7.699473677278425</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>117.5538880484445</v>
+        <v>559.4056061335972</v>
       </c>
     </row>
     <row r="5">
@@ -756,7 +654,7 @@
         <v>0.7830855557137725</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>13201.29866600037</v>
+        <v>12493.53005999611</v>
       </c>
     </row>
     <row r="6">
@@ -772,7 +670,7 @@
         <v>13.09578163496531</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>5.09979384286063</v>
+        <v>4.917651131039573</v>
       </c>
     </row>
     <row r="7">
@@ -788,7 +686,7 @@
         <v>52.95029311789443</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.499150866553897</v>
+        <v>0.4690283820742653</v>
       </c>
     </row>
     <row r="9">
@@ -836,7 +734,7 @@
         <v>0</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>90.77652976626442</v>
+        <v>93.94339606875465</v>
       </c>
     </row>
     <row r="12">
@@ -846,13 +744,13 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>4001.780952380952</v>
+        <v>4408.571428571428</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>10.95925841763052</v>
+        <v>3.146613048719591</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>117.5538880484445</v>
+        <v>559.4056061335972</v>
       </c>
     </row>
     <row r="13">
@@ -868,7 +766,7 @@
         <v>11.87591998359568</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>13.24944723220099</v>
+        <v>13.07282447814941</v>
       </c>
     </row>
     <row r="14">
@@ -898,7 +796,7 @@
         <v>14.13950847586963</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>10.93339692978632</v>
+        <v>10.56132089524042</v>
       </c>
     </row>
     <row r="17">
@@ -928,7 +826,7 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>1443.609605550766</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -938,7 +836,7 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>117.5538880484445</v>
+        <v>559.4056061335972</v>
       </c>
     </row>
     <row r="21">
@@ -948,7 +846,7 @@
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>13201.29866600037</v>
+        <v>12493.53005999611</v>
       </c>
     </row>
     <row r="22">
@@ -958,7 +856,7 @@
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>33.2845097496396</v>
+        <v>32.4363594963437</v>
       </c>
     </row>
     <row r="23">
@@ -968,7 +866,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>0.499150866553897</v>
+        <v>0.4690283820742653</v>
       </c>
     </row>
     <row r="24">
@@ -978,7 +876,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>5.09979384286063</v>
+        <v>4.917651131039573</v>
       </c>
     </row>
     <row r="25">
@@ -988,7 +886,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>13.24944723220099</v>
+        <v>13.07282447814941</v>
       </c>
     </row>
     <row r="26">
@@ -998,7 +896,7 @@
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>10.93339692978632</v>
+        <v>10.56132089524042</v>
       </c>
     </row>
     <row r="27">
@@ -1008,7 +906,7 @@
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>90.77652976626442</v>
+        <v>93.94339606875465</v>
       </c>
     </row>
   </sheetData>
@@ -1585,14 +1483,14 @@
       </c>
       <c r="I4" s="15" t="inlineStr">
         <is>
-          <t>[0, 15, 24, 6, 30, 0]</t>
+          <t>[0, 32, 23, 13, 30, 0]</t>
         </is>
       </c>
       <c r="J4" s="16" t="n">
-        <v>3710</v>
+        <v>4586</v>
       </c>
       <c r="K4" s="17" t="n">
-        <v>68.69978393103956</v>
+        <v>76.99346174245754</v>
       </c>
       <c r="L4" s="15" t="b">
         <v>1</v>
@@ -1648,7 +1546,7 @@
         <v>0</v>
       </c>
       <c r="AA4" s="5" t="n">
-        <v>26.25720532697277</v>
+        <v>8.845160007950707</v>
       </c>
       <c r="AB4" s="5" t="n">
         <v>0</v>
@@ -1680,14 +1578,14 @@
       </c>
       <c r="AJ4" s="18" t="inlineStr">
         <is>
-          <t>[0, 15, 24, 6, 30, 0]</t>
+          <t>[0, 27, 30, 32, 28, 15, 0]</t>
         </is>
       </c>
       <c r="AK4" s="19" t="n">
-        <v>3710</v>
+        <v>4724</v>
       </c>
       <c r="AL4" s="20" t="n">
-        <v>68.69978393103956</v>
+        <v>72.72308136763814</v>
       </c>
       <c r="AM4" s="18" t="b">
         <v>1</v>
@@ -1738,7 +1636,7 @@
         <v>0</v>
       </c>
       <c r="BA4" s="5" t="n">
-        <v>26.25720532697277</v>
+        <v>6.102166567282846</v>
       </c>
       <c r="BB4" s="5" t="n">
         <v>1.649771417213278</v>
@@ -1781,14 +1679,14 @@
       </c>
       <c r="I5" s="15" t="inlineStr">
         <is>
-          <t>[0, 15, 24, 6, 30, 0]</t>
+          <t>[0, 32, 23, 11, 28, 15, 30, 0]</t>
         </is>
       </c>
       <c r="J5" s="16" t="n">
-        <v>3587</v>
+        <v>4915</v>
       </c>
       <c r="K5" s="17" t="n">
-        <v>68.69978393103956</v>
+        <v>72.3529809644612</v>
       </c>
       <c r="L5" s="15" t="b">
         <v>1</v>
@@ -1844,7 +1742,7 @@
         <v>0</v>
       </c>
       <c r="AA5" s="5" t="n">
-        <v>35.3227551388388</v>
+        <v>11.37756941940137</v>
       </c>
       <c r="AB5" s="5" t="n">
         <v>0</v>
@@ -1876,14 +1774,14 @@
       </c>
       <c r="AJ5" s="18" t="inlineStr">
         <is>
-          <t>[0, 32, 28, 30, 27, 0]</t>
+          <t>[0, 32, 23, 1, 15, 30, 0]</t>
         </is>
       </c>
       <c r="AK5" s="19" t="n">
-        <v>4731</v>
+        <v>4840</v>
       </c>
       <c r="AL5" s="20" t="n">
-        <v>71.2255389720694</v>
+        <v>76.40911280206747</v>
       </c>
       <c r="AM5" s="18" t="b">
         <v>1</v>
@@ -1934,7 +1832,7 @@
         <v>0</v>
       </c>
       <c r="BA5" s="5" t="n">
-        <v>14.69527587450415</v>
+        <v>12.72989542012261</v>
       </c>
       <c r="BB5" s="5" t="n">
         <v>9.087630724846736</v>
@@ -1977,14 +1875,14 @@
       </c>
       <c r="I6" s="15" t="inlineStr">
         <is>
-          <t>[0, 15, 24, 6, 0]</t>
+          <t>[0, 32, 28, 30, 27, 0]</t>
         </is>
       </c>
       <c r="J6" s="16" t="n">
-        <v>3680</v>
+        <v>4632</v>
       </c>
       <c r="K6" s="17" t="n">
-        <v>69.69004820678865</v>
+        <v>71.2255389720694</v>
       </c>
       <c r="L6" s="15" t="b">
         <v>1</v>
@@ -2040,7 +1938,7 @@
         <v>0</v>
       </c>
       <c r="AA6" s="5" t="n">
-        <v>28.16708959593988</v>
+        <v>9.584227991411282</v>
       </c>
       <c r="AB6" s="5" t="n">
         <v>1.737263322272106</v>
@@ -2072,14 +1970,14 @@
       </c>
       <c r="AJ6" s="18" t="inlineStr">
         <is>
-          <t>[0, 15, 24, 6, 28, 30, 0]</t>
+          <t>[0, 32, 23, 11, 28, 15, 30, 0]</t>
         </is>
       </c>
       <c r="AK6" s="19" t="n">
-        <v>4028</v>
+        <v>5063</v>
       </c>
       <c r="AL6" s="20" t="n">
-        <v>68.73277915287588</v>
+        <v>72.3529809644612</v>
       </c>
       <c r="AM6" s="18" t="b">
         <v>1</v>
@@ -2130,7 +2028,7 @@
         <v>0</v>
       </c>
       <c r="BA6" s="5" t="n">
-        <v>21.37419480772985</v>
+        <v>1.171188756587937</v>
       </c>
       <c r="BB6" s="5" t="n">
         <v>4.25531914893617</v>
@@ -2173,14 +2071,14 @@
       </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
-          <t>[1, 28, 24, 6, 11, 23, 1]</t>
+          <t>[1, 15, 32, 23, 1]</t>
         </is>
       </c>
       <c r="J7" s="16" t="n">
-        <v>5071</v>
+        <v>4341</v>
       </c>
       <c r="K7" s="17" t="n">
-        <v>74.74858517898794</v>
+        <v>67.5733073091066</v>
       </c>
       <c r="L7" s="15" t="b">
         <v>1</v>
@@ -2236,7 +2134,7 @@
         <v>0</v>
       </c>
       <c r="AA7" s="5" t="n">
-        <v>16.69130934779037</v>
+        <v>28.68408082799408</v>
       </c>
       <c r="AB7" s="5" t="n">
         <v>0</v>
@@ -2268,14 +2166,14 @@
       </c>
       <c r="AJ7" s="18" t="inlineStr">
         <is>
-          <t>[1, 28, 24, 6, 11, 23, 1]</t>
+          <t>[1, 23, 11, 28, 15, 0, 30, 32, 1]</t>
         </is>
       </c>
       <c r="AK7" s="19" t="n">
-        <v>5071</v>
+        <v>4996</v>
       </c>
       <c r="AL7" s="20" t="n">
-        <v>74.74858517898794</v>
+        <v>75.96593670627344</v>
       </c>
       <c r="AM7" s="18" t="b">
         <v>1</v>
@@ -2326,7 +2224,7 @@
         <v>0</v>
       </c>
       <c r="BA7" s="5" t="n">
-        <v>16.69130934779037</v>
+        <v>17.92344340397569</v>
       </c>
       <c r="BB7" s="5" t="n">
         <v>27.40266140956136</v>
@@ -2369,14 +2267,14 @@
       </c>
       <c r="I8" s="15" t="inlineStr">
         <is>
-          <t>[1, 32, 23, 28, 1]</t>
+          <t>[1, 32, 23, 13, 17, 12, 34, 1]</t>
         </is>
       </c>
       <c r="J8" s="16" t="n">
-        <v>4074</v>
+        <v>5723</v>
       </c>
       <c r="K8" s="17" t="n">
-        <v>71.44273641087563</v>
+        <v>76.75203292600122</v>
       </c>
       <c r="L8" s="15" t="b">
         <v>1</v>
@@ -2432,7 +2330,7 @@
         <v>0</v>
       </c>
       <c r="AA8" s="5" t="n">
-        <v>32.53849975161451</v>
+        <v>5.232654412982282</v>
       </c>
       <c r="AB8" s="5" t="n">
         <v>6.17651929127339</v>
@@ -2464,14 +2362,14 @@
       </c>
       <c r="AJ8" s="18" t="inlineStr">
         <is>
-          <t>[1, 32, 23, 28, 1]</t>
+          <t>[1, 32, 23, 13, 17, 12, 34, 1]</t>
         </is>
       </c>
       <c r="AK8" s="19" t="n">
-        <v>4074</v>
+        <v>5723</v>
       </c>
       <c r="AL8" s="20" t="n">
-        <v>71.44273641087563</v>
+        <v>76.75203292600122</v>
       </c>
       <c r="AM8" s="18" t="b">
         <v>1</v>
@@ -2522,7 +2420,7 @@
         <v>0</v>
       </c>
       <c r="BA8" s="5" t="n">
-        <v>32.53849975161451</v>
+        <v>5.232654412982282</v>
       </c>
       <c r="BB8" s="5" t="n">
         <v>13.92614671303196</v>
@@ -2565,14 +2463,14 @@
       </c>
       <c r="I9" s="15" t="inlineStr">
         <is>
-          <t>[1, 15, 6, 24, 11, 23, 1]</t>
+          <t>[1, 23, 32, 16, 34, 31, 12, 1]</t>
         </is>
       </c>
       <c r="J9" s="16" t="n">
-        <v>5007</v>
+        <v>6000</v>
       </c>
       <c r="K9" s="17" t="n">
-        <v>74.74621340588094</v>
+        <v>75.05137961520434</v>
       </c>
       <c r="L9" s="15" t="b">
         <v>1</v>
@@ -2628,7 +2526,7 @@
         <v>0</v>
       </c>
       <c r="AA9" s="5" t="n">
-        <v>16.55</v>
+        <v>0</v>
       </c>
       <c r="AB9" s="5" t="n">
         <v>2.833333333333333</v>
@@ -2660,14 +2558,14 @@
       </c>
       <c r="AJ9" s="18" t="inlineStr">
         <is>
-          <t>[1, 15, 6, 24, 11, 23, 1]</t>
+          <t>[1, 17, 34, 16, 31, 12, 32, 1]</t>
         </is>
       </c>
       <c r="AK9" s="19" t="n">
-        <v>5007</v>
+        <v>5519</v>
       </c>
       <c r="AL9" s="20" t="n">
-        <v>74.74621340588094</v>
+        <v>74.89144463759283</v>
       </c>
       <c r="AM9" s="18" t="b">
         <v>1</v>
@@ -2718,7 +2616,7 @@
         <v>0</v>
       </c>
       <c r="BA9" s="5" t="n">
-        <v>16.55</v>
+        <v>8.016666666666666</v>
       </c>
       <c r="BB9" s="5" t="n">
         <v>2.833333333333333</v>
@@ -2761,14 +2659,14 @@
       </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
-          <t>[2, 17, 23, 11, 8, 2]</t>
+          <t>[2, 17, 23, 13, 8, 18, 2]</t>
         </is>
       </c>
       <c r="J10" s="16" t="n">
-        <v>4724</v>
+        <v>4922</v>
       </c>
       <c r="K10" s="17" t="n">
-        <v>71.57785308163562</v>
+        <v>74.42240734974001</v>
       </c>
       <c r="L10" s="15" t="b">
         <v>1</v>
@@ -2824,7 +2722,7 @@
         <v>0</v>
       </c>
       <c r="AA10" s="5" t="n">
-        <v>9.623110770996748</v>
+        <v>5.835087048019897</v>
       </c>
       <c r="AB10" s="5" t="n">
         <v>5.835087048019897</v>
@@ -2856,14 +2754,14 @@
       </c>
       <c r="AJ10" s="18" t="inlineStr">
         <is>
-          <t>[2, 17, 23, 13, 8, 18, 2]</t>
+          <t>[2, 18, 17, 23, 11, 13, 2]</t>
         </is>
       </c>
       <c r="AK10" s="19" t="n">
-        <v>4922</v>
+        <v>5227</v>
       </c>
       <c r="AL10" s="20" t="n">
-        <v>74.42240734974001</v>
+        <v>75.43232651457264</v>
       </c>
       <c r="AM10" s="18" t="b">
         <v>1</v>
@@ -2914,7 +2812,7 @@
         <v>0</v>
       </c>
       <c r="BA10" s="5" t="n">
-        <v>5.835087048019897</v>
+        <v>0</v>
       </c>
       <c r="BB10" s="5" t="n">
         <v>10.94317964415535</v>
@@ -2957,14 +2855,14 @@
       </c>
       <c r="I11" s="15" t="inlineStr">
         <is>
-          <t>[2, 13, 23, 11, 8, 18, 2]</t>
+          <t>[2, 23, 11, 13, 8, 18, 2]</t>
         </is>
       </c>
       <c r="J11" s="16" t="n">
-        <v>5209</v>
+        <v>4965</v>
       </c>
       <c r="K11" s="17" t="n">
-        <v>76.11688487342525</v>
+        <v>74.84235419102524</v>
       </c>
       <c r="L11" s="15" t="b">
         <v>1</v>
@@ -3020,7 +2918,7 @@
         <v>0</v>
       </c>
       <c r="AA11" s="5" t="n">
-        <v>0</v>
+        <v>4.684200422345939</v>
       </c>
       <c r="AB11" s="5" t="n">
         <v>0</v>
@@ -3052,14 +2950,14 @@
       </c>
       <c r="AJ11" s="18" t="inlineStr">
         <is>
-          <t>[2, 29, 23, 13, 2]</t>
+          <t>[2, 13, 23, 11, 8, 18, 2]</t>
         </is>
       </c>
       <c r="AK11" s="19" t="n">
-        <v>3793</v>
+        <v>5209</v>
       </c>
       <c r="AL11" s="20" t="n">
-        <v>72.9990111521933</v>
+        <v>76.11688487342525</v>
       </c>
       <c r="AM11" s="18" t="b">
         <v>1</v>
@@ -3110,7 +3008,7 @@
         <v>0</v>
       </c>
       <c r="BA11" s="5" t="n">
-        <v>27.18372048377808</v>
+        <v>0</v>
       </c>
       <c r="BB11" s="5" t="n">
         <v>23.72816279516222</v>
@@ -3349,14 +3247,14 @@
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
-          <t>[3, 5, 14, 3]</t>
+          <t>[3, 33, 10, 4, 3]</t>
         </is>
       </c>
       <c r="J13" s="16" t="n">
-        <v>1721</v>
+        <v>2315</v>
       </c>
       <c r="K13" s="17" t="n">
-        <v>73.22606566043079</v>
+        <v>69.72629704336707</v>
       </c>
       <c r="L13" s="15" t="b">
         <v>1</v>
@@ -3412,7 +3310,7 @@
         <v>0</v>
       </c>
       <c r="AA13" s="5" t="n">
-        <v>25.65874730021599</v>
+        <v>0</v>
       </c>
       <c r="AB13" s="5" t="n">
         <v>0</v>
@@ -3444,14 +3342,14 @@
       </c>
       <c r="AJ13" s="18" t="inlineStr">
         <is>
-          <t>[3, 4, 14, 33, 3]</t>
+          <t>[3, 33, 10, 4, 3]</t>
         </is>
       </c>
       <c r="AK13" s="19" t="n">
-        <v>1937</v>
+        <v>2315</v>
       </c>
       <c r="AL13" s="20" t="n">
-        <v>76.12162017812862</v>
+        <v>69.72629704336707</v>
       </c>
       <c r="AM13" s="18" t="b">
         <v>1</v>
@@ -3502,7 +3400,7 @@
         <v>0</v>
       </c>
       <c r="BA13" s="5" t="n">
-        <v>16.32829373650108</v>
+        <v>0</v>
       </c>
       <c r="BB13" s="5" t="n">
         <v>0</v>
@@ -3741,14 +3639,14 @@
       </c>
       <c r="I15" s="15" t="inlineStr">
         <is>
-          <t>[3, 33, 14, 3]</t>
+          <t>[3, 33, 4, 10, 3]</t>
         </is>
       </c>
       <c r="J15" s="16" t="n">
-        <v>1791</v>
+        <v>1972</v>
       </c>
       <c r="K15" s="17" t="n">
-        <v>66.05977972411036</v>
+        <v>72.20133315988178</v>
       </c>
       <c r="L15" s="15" t="b">
         <v>1</v>
@@ -3804,7 +3702,7 @@
         <v>0</v>
       </c>
       <c r="AA15" s="5" t="n">
-        <v>21.3784021071115</v>
+        <v>13.43283582089552</v>
       </c>
       <c r="AB15" s="5" t="n">
         <v>0</v>
@@ -3836,14 +3734,14 @@
       </c>
       <c r="AJ15" s="18" t="inlineStr">
         <is>
-          <t>[3, 4, 14, 33, 3]</t>
+          <t>[3, 4, 10, 33, 3]</t>
         </is>
       </c>
       <c r="AK15" s="19" t="n">
-        <v>2105</v>
+        <v>2278</v>
       </c>
       <c r="AL15" s="20" t="n">
-        <v>76.12162017812862</v>
+        <v>69.57524485498676</v>
       </c>
       <c r="AM15" s="18" t="b">
         <v>1</v>
@@ -3894,7 +3792,7 @@
         <v>0</v>
       </c>
       <c r="BA15" s="5" t="n">
-        <v>7.594381035996488</v>
+        <v>0</v>
       </c>
       <c r="BB15" s="5" t="n">
         <v>0</v>
@@ -3937,14 +3835,14 @@
       </c>
       <c r="I16" s="15" t="inlineStr">
         <is>
-          <t>[4, 3, 14, 4]</t>
+          <t>[4, 14, 33, 3, 4]</t>
         </is>
       </c>
       <c r="J16" s="16" t="n">
-        <v>1719</v>
+        <v>2386</v>
       </c>
       <c r="K16" s="17" t="n">
-        <v>63.30871336570848</v>
+        <v>76.12162017812862</v>
       </c>
       <c r="L16" s="15" t="b">
         <v>1</v>
@@ -4000,7 +3898,7 @@
         <v>0</v>
       </c>
       <c r="AA16" s="5" t="n">
-        <v>27.9547359597653</v>
+        <v>0</v>
       </c>
       <c r="AB16" s="5" t="n">
         <v>0</v>
@@ -4032,14 +3930,14 @@
       </c>
       <c r="AJ16" s="18" t="inlineStr">
         <is>
-          <t>[4, 14, 5, 4]</t>
+          <t>[4, 33, 3, 14, 4]</t>
         </is>
       </c>
       <c r="AK16" s="19" t="n">
-        <v>1903</v>
+        <v>2013</v>
       </c>
       <c r="AL16" s="20" t="n">
-        <v>72.10731512057799</v>
+        <v>66.1231493674095</v>
       </c>
       <c r="AM16" s="18" t="b">
         <v>1</v>
@@ -4090,7 +3988,7 @@
         <v>0</v>
       </c>
       <c r="BA16" s="5" t="n">
-        <v>20.2430846605197</v>
+        <v>15.63285834031853</v>
       </c>
       <c r="BB16" s="5" t="n">
         <v>0</v>
@@ -4228,14 +4126,14 @@
       </c>
       <c r="AJ17" s="18" t="inlineStr">
         <is>
-          <t>[4, 33, 14, 4]</t>
+          <t>[4, 14, 33, 3, 4]</t>
         </is>
       </c>
       <c r="AK17" s="19" t="n">
-        <v>1770</v>
+        <v>2352</v>
       </c>
       <c r="AL17" s="20" t="n">
-        <v>52.73651937195241</v>
+        <v>76.12162017812862</v>
       </c>
       <c r="AM17" s="18" t="b">
         <v>1</v>
@@ -4286,7 +4184,7 @@
         <v>0</v>
       </c>
       <c r="BA17" s="5" t="n">
-        <v>24.74489795918367</v>
+        <v>0</v>
       </c>
       <c r="BB17" s="5" t="n">
         <v>0</v>
@@ -4329,14 +4227,14 @@
       </c>
       <c r="I18" s="15" t="inlineStr">
         <is>
-          <t>[4, 33, 14, 4]</t>
+          <t>[4, 3, 33, 10, 4]</t>
         </is>
       </c>
       <c r="J18" s="16" t="n">
-        <v>2378</v>
+        <v>2518</v>
       </c>
       <c r="K18" s="17" t="n">
-        <v>52.73651937195241</v>
+        <v>69.72629704336707</v>
       </c>
       <c r="L18" s="15" t="b">
         <v>1</v>
@@ -4392,7 +4290,7 @@
         <v>0</v>
       </c>
       <c r="AA18" s="5" t="n">
-        <v>5.559968228752978</v>
+        <v>0</v>
       </c>
       <c r="AB18" s="5" t="n">
         <v>0</v>
@@ -4424,14 +4322,14 @@
       </c>
       <c r="AJ18" s="18" t="inlineStr">
         <is>
-          <t>[4, 33, 14, 4]</t>
+          <t>[4, 14, 33, 3, 4]</t>
         </is>
       </c>
       <c r="AK18" s="19" t="n">
-        <v>2378</v>
+        <v>2408</v>
       </c>
       <c r="AL18" s="20" t="n">
-        <v>52.73651937195241</v>
+        <v>76.12162017812862</v>
       </c>
       <c r="AM18" s="18" t="b">
         <v>1</v>
@@ -4482,7 +4380,7 @@
         <v>0</v>
       </c>
       <c r="BA18" s="5" t="n">
-        <v>5.559968228752978</v>
+        <v>4.368546465448769</v>
       </c>
       <c r="BB18" s="5" t="n">
         <v>0</v>
@@ -4721,14 +4619,14 @@
       </c>
       <c r="I20" s="15" t="inlineStr">
         <is>
-          <t>[5, 14, 25, 5]</t>
+          <t>[5, 14, 4, 5]</t>
         </is>
       </c>
       <c r="J20" s="16" t="n">
-        <v>1670</v>
+        <v>2379</v>
       </c>
       <c r="K20" s="17" t="n">
-        <v>52.65000845783882</v>
+        <v>72.12551059405325</v>
       </c>
       <c r="L20" s="15" t="b">
         <v>1</v>
@@ -4784,7 +4682,7 @@
         <v>0</v>
       </c>
       <c r="AA20" s="5" t="n">
-        <v>29.80243799915931</v>
+        <v>0</v>
       </c>
       <c r="AB20" s="5" t="n">
         <v>0</v>
@@ -5404,14 +5302,14 @@
       </c>
       <c r="AJ23" s="18" t="inlineStr">
         <is>
-          <t>[6, 32, 23, 11, 24, 6]</t>
+          <t>[6, 11, 13, 23, 1, 15, 28, 6]</t>
         </is>
       </c>
       <c r="AK23" s="19" t="n">
-        <v>4331</v>
+        <v>5844</v>
       </c>
       <c r="AL23" s="20" t="n">
-        <v>68.63913955482947</v>
+        <v>76.9634944961675</v>
       </c>
       <c r="AM23" s="18" t="b">
         <v>1</v>
@@ -5462,7 +5360,7 @@
         <v>0</v>
       </c>
       <c r="BA23" s="5" t="n">
-        <v>25.88980150581793</v>
+        <v>0</v>
       </c>
       <c r="BB23" s="5" t="n">
         <v>23.57973990417522</v>
@@ -5505,14 +5403,14 @@
       </c>
       <c r="I24" s="15" t="inlineStr">
         <is>
-          <t>[6, 15, 27, 0, 30, 28, 6]</t>
+          <t>[6, 32, 23, 11, 28, 6]</t>
         </is>
       </c>
       <c r="J24" s="16" t="n">
-        <v>4099</v>
+        <v>4369</v>
       </c>
       <c r="K24" s="17" t="n">
-        <v>73.72894236809849</v>
+        <v>73.6113709824498</v>
       </c>
       <c r="L24" s="15" t="b">
         <v>1</v>
@@ -5568,7 +5466,7 @@
         <v>0</v>
       </c>
       <c r="AA24" s="5" t="n">
-        <v>20.14416520553283</v>
+        <v>14.88408338203779</v>
       </c>
       <c r="AB24" s="5" t="n">
         <v>2.824858757062147</v>
@@ -5600,14 +5498,14 @@
       </c>
       <c r="AJ24" s="18" t="inlineStr">
         <is>
-          <t>[6, 32, 23, 11, 28, 6]</t>
+          <t>[6, 28, 15, 32, 23, 24, 6]</t>
         </is>
       </c>
       <c r="AK24" s="19" t="n">
-        <v>4369</v>
+        <v>4700</v>
       </c>
       <c r="AL24" s="20" t="n">
-        <v>73.6113709824498</v>
+        <v>76.94478559885567</v>
       </c>
       <c r="AM24" s="18" t="b">
         <v>1</v>
@@ -5658,7 +5556,7 @@
         <v>0</v>
       </c>
       <c r="BA24" s="5" t="n">
-        <v>14.88408338203779</v>
+        <v>8.435612702123514</v>
       </c>
       <c r="BB24" s="5" t="n">
         <v>14.88408338203779</v>
@@ -5701,14 +5599,14 @@
       </c>
       <c r="I25" s="15" t="inlineStr">
         <is>
-          <t>[7, 28, 24, 6, 7]</t>
+          <t>[7, 28, 24, 11, 6, 7]</t>
         </is>
       </c>
       <c r="J25" s="16" t="n">
-        <v>3837</v>
+        <v>4305</v>
       </c>
       <c r="K25" s="17" t="n">
-        <v>62.07798586670543</v>
+        <v>73.95218729374309</v>
       </c>
       <c r="L25" s="15" t="b">
         <v>1</v>
@@ -5764,7 +5662,7 @@
         <v>0</v>
       </c>
       <c r="AA25" s="5" t="n">
-        <v>18.25734980826587</v>
+        <v>8.287175117170856</v>
       </c>
       <c r="AB25" s="5" t="n">
         <v>0</v>
@@ -5796,14 +5694,14 @@
       </c>
       <c r="AJ25" s="18" t="inlineStr">
         <is>
-          <t>[7, 28, 24, 11, 6, 7]</t>
+          <t>[7, 28, 23, 11, 24, 7]</t>
         </is>
       </c>
       <c r="AK25" s="19" t="n">
-        <v>4305</v>
+        <v>4621</v>
       </c>
       <c r="AL25" s="20" t="n">
-        <v>73.95218729374309</v>
+        <v>75.83608168317812</v>
       </c>
       <c r="AM25" s="18" t="b">
         <v>1</v>
@@ -5854,7 +5752,7 @@
         <v>0</v>
       </c>
       <c r="BA25" s="5" t="n">
-        <v>8.287175117170856</v>
+        <v>1.555176821474223</v>
       </c>
       <c r="BB25" s="5" t="n">
         <v>1.555176821474223</v>
@@ -5992,14 +5890,14 @@
       </c>
       <c r="AJ26" s="18" t="inlineStr">
         <is>
-          <t>[7, 28, 24, 11, 6, 7]</t>
+          <t>[7, 24, 11, 13, 23, 6, 7]</t>
         </is>
       </c>
       <c r="AK26" s="19" t="n">
-        <v>4005</v>
+        <v>4432</v>
       </c>
       <c r="AL26" s="20" t="n">
-        <v>73.95218729374309</v>
+        <v>76.6364129964185</v>
       </c>
       <c r="AM26" s="18" t="b">
         <v>1</v>
@@ -6050,7 +5948,7 @@
         <v>0</v>
       </c>
       <c r="BA26" s="5" t="n">
-        <v>9.634476534296029</v>
+        <v>0</v>
       </c>
       <c r="BB26" s="5" t="n">
         <v>2.594765342960289</v>
@@ -6188,14 +6086,14 @@
       </c>
       <c r="AJ27" s="18" t="inlineStr">
         <is>
-          <t>[7, 23, 11, 24, 6, 7]</t>
+          <t>[7, 24, 11, 13, 23, 7]</t>
         </is>
       </c>
       <c r="AK27" s="19" t="n">
-        <v>3287</v>
+        <v>3386</v>
       </c>
       <c r="AL27" s="20" t="n">
-        <v>72.87174262696787</v>
+        <v>75.70525438457454</v>
       </c>
       <c r="AM27" s="18" t="b">
         <v>1</v>
@@ -6246,7 +6144,7 @@
         <v>0</v>
       </c>
       <c r="BA27" s="5" t="n">
-        <v>8.107352530053118</v>
+        <v>5.339670114621191</v>
       </c>
       <c r="BB27" s="5" t="n">
         <v>10.34386357282639</v>
@@ -6289,14 +6187,14 @@
       </c>
       <c r="I28" s="15" t="inlineStr">
         <is>
-          <t>[8, 18, 11, 23, 13, 8]</t>
+          <t>[8, 18, 2, 11, 13, 8]</t>
         </is>
       </c>
       <c r="J28" s="16" t="n">
-        <v>4539</v>
+        <v>4067</v>
       </c>
       <c r="K28" s="17" t="n">
-        <v>75.35012256935434</v>
+        <v>71.86492405207225</v>
       </c>
       <c r="L28" s="15" t="b">
         <v>1</v>
@@ -6352,7 +6250,7 @@
         <v>0</v>
       </c>
       <c r="AA28" s="5" t="n">
-        <v>12.82888419435375</v>
+        <v>21.89360476281928</v>
       </c>
       <c r="AB28" s="5" t="n">
         <v>0</v>
@@ -6485,14 +6383,14 @@
       </c>
       <c r="I29" s="15" t="inlineStr">
         <is>
-          <t>[8, 2, 11, 13, 8]</t>
+          <t>[8, 2, 13, 23, 1, 8]</t>
         </is>
       </c>
       <c r="J29" s="16" t="n">
-        <v>3081</v>
+        <v>4007</v>
       </c>
       <c r="K29" s="17" t="n">
-        <v>61.58036835652361</v>
+        <v>76.68615652701594</v>
       </c>
       <c r="L29" s="15" t="b">
         <v>1</v>
@@ -6548,7 +6446,7 @@
         <v>0</v>
       </c>
       <c r="AA29" s="5" t="n">
-        <v>28.3987915407855</v>
+        <v>6.878921682547061</v>
       </c>
       <c r="AB29" s="5" t="n">
         <v>0</v>
@@ -6580,14 +6478,14 @@
       </c>
       <c r="AJ29" s="18" t="inlineStr">
         <is>
-          <t>[8, 2, 11, 13, 8]</t>
+          <t>[8, 11, 23, 1, 12, 17, 8]</t>
         </is>
       </c>
       <c r="AK29" s="19" t="n">
-        <v>3081</v>
+        <v>4303</v>
       </c>
       <c r="AL29" s="20" t="n">
-        <v>61.58036835652361</v>
+        <v>76.61506080163667</v>
       </c>
       <c r="AM29" s="18" t="b">
         <v>1</v>
@@ -6638,7 +6536,7 @@
         <v>0</v>
       </c>
       <c r="BA29" s="5" t="n">
-        <v>28.3987915407855</v>
+        <v>0</v>
       </c>
       <c r="BB29" s="5" t="n">
         <v>3.044387636532652</v>
@@ -6776,14 +6674,14 @@
       </c>
       <c r="AJ30" s="18" t="inlineStr">
         <is>
-          <t>[8, 18, 1, 23, 13, 8]</t>
+          <t>[8, 2, 18, 1, 23, 13, 8]</t>
         </is>
       </c>
       <c r="AK30" s="19" t="n">
-        <v>6300</v>
+        <v>6563</v>
       </c>
       <c r="AL30" s="20" t="n">
-        <v>76.51908217378218</v>
+        <v>76.90062624855432</v>
       </c>
       <c r="AM30" s="18" t="b">
         <v>1</v>
@@ -6834,7 +6732,7 @@
         <v>0</v>
       </c>
       <c r="BA30" s="5" t="n">
-        <v>4.00731372847783</v>
+        <v>0</v>
       </c>
       <c r="BB30" s="5" t="n">
         <v>4.00731372847783</v>
@@ -6877,14 +6775,14 @@
       </c>
       <c r="I31" s="15" t="inlineStr">
         <is>
-          <t>[9, 31, 17, 34, 9]</t>
+          <t>[9, 12, 34, 31, 9]</t>
         </is>
       </c>
       <c r="J31" s="16" t="n">
-        <v>905</v>
+        <v>941</v>
       </c>
       <c r="K31" s="17" t="n">
-        <v>76.85670991144411</v>
+        <v>67.42178758205692</v>
       </c>
       <c r="L31" s="15" t="b">
         <v>1</v>
@@ -6940,7 +6838,7 @@
         <v>0</v>
       </c>
       <c r="AA31" s="5" t="n">
-        <v>20.96069868995633</v>
+        <v>17.81659388646288</v>
       </c>
       <c r="AB31" s="5" t="n">
         <v>0</v>
@@ -7661,14 +7559,14 @@
       </c>
       <c r="I35" s="15" t="inlineStr">
         <is>
-          <t>[10, 4, 3, 33, 10]</t>
+          <t>[10, 4, 33, 3, 10]</t>
         </is>
       </c>
       <c r="J35" s="16" t="n">
-        <v>2630</v>
+        <v>2880</v>
       </c>
       <c r="K35" s="17" t="n">
-        <v>69.72629704336707</v>
+        <v>72.48342803985913</v>
       </c>
       <c r="L35" s="15" t="b">
         <v>1</v>
@@ -7724,7 +7622,7 @@
         <v>0</v>
       </c>
       <c r="AA35" s="5" t="n">
-        <v>8.680555555555555</v>
+        <v>0</v>
       </c>
       <c r="AB35" s="5" t="n">
         <v>0</v>
@@ -7756,14 +7654,14 @@
       </c>
       <c r="AJ35" s="18" t="inlineStr">
         <is>
-          <t>[10, 4, 3, 33, 10]</t>
+          <t>[10, 4, 33, 3, 10]</t>
         </is>
       </c>
       <c r="AK35" s="19" t="n">
-        <v>2630</v>
+        <v>2880</v>
       </c>
       <c r="AL35" s="20" t="n">
-        <v>69.72629704336707</v>
+        <v>72.48342803985913</v>
       </c>
       <c r="AM35" s="18" t="b">
         <v>1</v>
@@ -7814,7 +7712,7 @@
         <v>0</v>
       </c>
       <c r="BA35" s="5" t="n">
-        <v>8.680555555555555</v>
+        <v>0</v>
       </c>
       <c r="BB35" s="5" t="n">
         <v>0</v>
@@ -8053,14 +7951,14 @@
       </c>
       <c r="I37" s="15" t="inlineStr">
         <is>
-          <t>[11, 13, 28, 24, 6, 11]</t>
+          <t>[11, 13, 1, 15, 28, 6, 11]</t>
         </is>
       </c>
       <c r="J37" s="16" t="n">
-        <v>3913</v>
+        <v>4772</v>
       </c>
       <c r="K37" s="17" t="n">
-        <v>63.88382379545</v>
+        <v>76.229668609641</v>
       </c>
       <c r="L37" s="15" t="b">
         <v>1</v>
@@ -8116,7 +8014,7 @@
         <v>0</v>
       </c>
       <c r="AA37" s="5" t="n">
-        <v>30.41081273341632</v>
+        <v>15.13426996265339</v>
       </c>
       <c r="AB37" s="5" t="n">
         <v>1.422728081095501</v>
@@ -8148,14 +8046,14 @@
       </c>
       <c r="AJ37" s="18" t="inlineStr">
         <is>
-          <t>[11, 13, 32, 15, 28, 11]</t>
+          <t>[11, 13, 23, 1, 15, 28, 6, 11]</t>
         </is>
       </c>
       <c r="AK37" s="19" t="n">
-        <v>4462</v>
+        <v>5623</v>
       </c>
       <c r="AL37" s="20" t="n">
-        <v>73.90563991005703</v>
+        <v>76.9634944961675</v>
       </c>
       <c r="AM37" s="18" t="b">
         <v>1</v>
@@ -8206,7 +8104,7 @@
         <v>0</v>
       </c>
       <c r="BA37" s="5" t="n">
-        <v>20.64734127689846</v>
+        <v>0</v>
       </c>
       <c r="BB37" s="5" t="n">
         <v>0</v>
@@ -8344,14 +8242,14 @@
       </c>
       <c r="AJ38" s="18" t="inlineStr">
         <is>
-          <t>[11, 13, 7, 6, 24, 11]</t>
+          <t>[11, 13, 23, 1, 15, 28, 6, 11]</t>
         </is>
       </c>
       <c r="AK38" s="19" t="n">
-        <v>4417</v>
+        <v>5088</v>
       </c>
       <c r="AL38" s="20" t="n">
-        <v>74.20205519431896</v>
+        <v>76.9634944961675</v>
       </c>
       <c r="AM38" s="18" t="b">
         <v>1</v>
@@ -8402,7 +8300,7 @@
         <v>0</v>
       </c>
       <c r="BA38" s="5" t="n">
-        <v>28.7350758309132</v>
+        <v>17.90900290416263</v>
       </c>
       <c r="BB38" s="5" t="n">
         <v>23.71732817037754</v>
@@ -8445,14 +8343,14 @@
       </c>
       <c r="I39" s="15" t="inlineStr">
         <is>
-          <t>[11, 13, 15, 28, 6, 24, 11]</t>
+          <t>[11, 13, 1, 15, 28, 6, 11]</t>
         </is>
       </c>
       <c r="J39" s="16" t="n">
-        <v>4455</v>
+        <v>4772</v>
       </c>
       <c r="K39" s="17" t="n">
-        <v>71.8544588928042</v>
+        <v>76.229668609641</v>
       </c>
       <c r="L39" s="15" t="b">
         <v>1</v>
@@ -8508,7 +8406,7 @@
         <v>0</v>
       </c>
       <c r="AA39" s="5" t="n">
-        <v>23.7549204175937</v>
+        <v>18.32962519253808</v>
       </c>
       <c r="AB39" s="5" t="n">
         <v>6.161218552113641</v>
@@ -8540,14 +8438,14 @@
       </c>
       <c r="AJ39" s="18" t="inlineStr">
         <is>
-          <t>[11, 13, 32, 15, 28, 11]</t>
+          <t>[11, 13, 23, 1, 32, 15, 28, 11]</t>
         </is>
       </c>
       <c r="AK39" s="19" t="n">
-        <v>4382</v>
+        <v>5843</v>
       </c>
       <c r="AL39" s="20" t="n">
-        <v>73.90563991005703</v>
+        <v>76.89611101445851</v>
       </c>
       <c r="AM39" s="18" t="b">
         <v>1</v>
@@ -8598,7 +8496,7 @@
         <v>0</v>
       </c>
       <c r="BA39" s="5" t="n">
-        <v>25.00427862399452</v>
+        <v>0</v>
       </c>
       <c r="BB39" s="5" t="n">
         <v>4.877631353756632</v>
@@ -8736,14 +8634,14 @@
       </c>
       <c r="AJ40" s="18" t="inlineStr">
         <is>
-          <t>[12, 13, 17, 16, 34, 12]</t>
+          <t>[12, 34, 16, 32, 23, 17, 12]</t>
         </is>
       </c>
       <c r="AK40" s="19" t="n">
-        <v>5449</v>
+        <v>5453</v>
       </c>
       <c r="AL40" s="20" t="n">
-        <v>75.91279165923</v>
+        <v>75.11649267211246</v>
       </c>
       <c r="AM40" s="18" t="b">
         <v>1</v>
@@ -8794,7 +8692,7 @@
         <v>0</v>
       </c>
       <c r="BA40" s="5" t="n">
-        <v>12.53611556982344</v>
+        <v>12.47191011235955</v>
       </c>
       <c r="BB40" s="5" t="n">
         <v>9.390048154093098</v>
@@ -8837,14 +8735,14 @@
       </c>
       <c r="I41" s="15" t="inlineStr">
         <is>
-          <t>[12, 34, 28, 32, 1, 12]</t>
+          <t>[12, 34, 16, 31, 17, 23, 1, 12]</t>
         </is>
       </c>
       <c r="J41" s="16" t="n">
-        <v>4053</v>
+        <v>5321</v>
       </c>
       <c r="K41" s="17" t="n">
-        <v>76.39477658299226</v>
+        <v>76.7741215108931</v>
       </c>
       <c r="L41" s="15" t="b">
         <v>1</v>
@@ -8900,7 +8798,7 @@
         <v>0</v>
       </c>
       <c r="AA41" s="5" t="n">
-        <v>31.5140250084488</v>
+        <v>10.08786752281176</v>
       </c>
       <c r="AB41" s="5" t="n">
         <v>0</v>
@@ -8932,14 +8830,14 @@
       </c>
       <c r="AJ41" s="18" t="inlineStr">
         <is>
-          <t>[12, 13, 23, 32, 16, 12]</t>
+          <t>[12, 34, 31, 16, 32, 23, 1, 12]</t>
         </is>
       </c>
       <c r="AK41" s="19" t="n">
-        <v>4975</v>
+        <v>5402</v>
       </c>
       <c r="AL41" s="20" t="n">
-        <v>73.12516974640894</v>
+        <v>75.08232804674387</v>
       </c>
       <c r="AM41" s="18" t="b">
         <v>1</v>
@@ -8990,7 +8888,7 @@
         <v>0</v>
       </c>
       <c r="BA41" s="5" t="n">
-        <v>15.93443730990199</v>
+        <v>8.71916187901318</v>
       </c>
       <c r="BB41" s="5" t="n">
         <v>32.12233862791484</v>
@@ -9033,14 +8931,14 @@
       </c>
       <c r="I42" s="15" t="inlineStr">
         <is>
-          <t>[12, 32, 28, 1, 34, 12]</t>
+          <t>[12, 17, 16, 34, 31, 1, 12]</t>
         </is>
       </c>
       <c r="J42" s="16" t="n">
-        <v>4454</v>
+        <v>4998</v>
       </c>
       <c r="K42" s="17" t="n">
-        <v>73.3141335518188</v>
+        <v>71.55969324712517</v>
       </c>
       <c r="L42" s="15" t="b">
         <v>1</v>
@@ -9096,7 +8994,7 @@
         <v>0</v>
       </c>
       <c r="AA42" s="5" t="n">
-        <v>22.71386430678466</v>
+        <v>13.27433628318584</v>
       </c>
       <c r="AB42" s="5" t="n">
         <v>0</v>
@@ -9128,14 +9026,14 @@
       </c>
       <c r="AJ42" s="18" t="inlineStr">
         <is>
-          <t>[12, 32, 23, 11, 1, 34, 12]</t>
+          <t>[12, 31, 34, 16, 32, 23, 1, 12]</t>
         </is>
       </c>
       <c r="AK42" s="19" t="n">
-        <v>4836</v>
+        <v>5519</v>
       </c>
       <c r="AL42" s="20" t="n">
-        <v>74.32410773430335</v>
+        <v>75.11269845882315</v>
       </c>
       <c r="AM42" s="18" t="b">
         <v>1</v>
@@ -9186,7 +9084,7 @@
         <v>0</v>
       </c>
       <c r="BA42" s="5" t="n">
-        <v>16.08537220197814</v>
+        <v>4.233905951761235</v>
       </c>
       <c r="BB42" s="5" t="n">
         <v>27.53774076002082</v>
@@ -9229,14 +9127,14 @@
       </c>
       <c r="I43" s="15" t="inlineStr">
         <is>
-          <t>[13, 23, 28, 24, 6, 11, 13]</t>
+          <t>[13, 1, 28, 11, 23, 13]</t>
         </is>
       </c>
       <c r="J43" s="16" t="n">
-        <v>5255</v>
+        <v>4558</v>
       </c>
       <c r="K43" s="17" t="n">
-        <v>69.26091319489262</v>
+        <v>72.75626993085845</v>
       </c>
       <c r="L43" s="15" t="b">
         <v>1</v>
@@ -9292,7 +9190,7 @@
         <v>0</v>
       </c>
       <c r="AA43" s="5" t="n">
-        <v>9.800892550635085</v>
+        <v>21.76450394782012</v>
       </c>
       <c r="AB43" s="5" t="n">
         <v>0</v>
@@ -9425,14 +9323,14 @@
       </c>
       <c r="I44" s="15" t="inlineStr">
         <is>
-          <t>[13, 7, 6, 24, 11, 13]</t>
+          <t>[13, 1, 16, 34, 12, 23, 13]</t>
         </is>
       </c>
       <c r="J44" s="16" t="n">
-        <v>4454</v>
+        <v>5237</v>
       </c>
       <c r="K44" s="17" t="n">
-        <v>74.20205519431896</v>
+        <v>76.5606625994937</v>
       </c>
       <c r="L44" s="15" t="b">
         <v>1</v>
@@ -9488,7 +9386,7 @@
         <v>0</v>
       </c>
       <c r="AA44" s="5" t="n">
-        <v>22.18728162124388</v>
+        <v>8.508036338225017</v>
       </c>
       <c r="AB44" s="5" t="n">
         <v>0.628930817610063</v>
@@ -9520,14 +9418,14 @@
       </c>
       <c r="AJ44" s="18" t="inlineStr">
         <is>
-          <t>[13, 7, 6, 11, 23, 13]</t>
+          <t>[13, 1, 16, 34, 12, 23, 13]</t>
         </is>
       </c>
       <c r="AK44" s="19" t="n">
-        <v>4233</v>
+        <v>5237</v>
       </c>
       <c r="AL44" s="20" t="n">
-        <v>73.06439751541268</v>
+        <v>76.5606625994937</v>
       </c>
       <c r="AM44" s="18" t="b">
         <v>1</v>
@@ -9578,7 +9476,7 @@
         <v>0</v>
       </c>
       <c r="BA44" s="5" t="n">
-        <v>26.04821802935011</v>
+        <v>8.508036338225017</v>
       </c>
       <c r="BB44" s="5" t="n">
         <v>32.25017470300489</v>
@@ -9621,14 +9519,14 @@
       </c>
       <c r="I45" s="15" t="inlineStr">
         <is>
-          <t>[13, 1, 15, 28, 6, 11, 13]</t>
+          <t>[13, 1, 16, 31, 12, 34, 13]</t>
         </is>
       </c>
       <c r="J45" s="16" t="n">
-        <v>4663</v>
+        <v>5038</v>
       </c>
       <c r="K45" s="17" t="n">
-        <v>76.229668609641</v>
+        <v>73.88913350076947</v>
       </c>
       <c r="L45" s="15" t="b">
         <v>1</v>
@@ -9684,7 +9582,7 @@
         <v>0</v>
       </c>
       <c r="AA45" s="5" t="n">
-        <v>15.49474447263501</v>
+        <v>8.698803914461761</v>
       </c>
       <c r="AB45" s="5" t="n">
         <v>2.482783617252628</v>
@@ -9716,14 +9614,14 @@
       </c>
       <c r="AJ45" s="18" t="inlineStr">
         <is>
-          <t>[13, 1, 15, 28, 6, 11, 13]</t>
+          <t>[13, 23, 1, 34, 16, 12, 13]</t>
         </is>
       </c>
       <c r="AK45" s="19" t="n">
-        <v>4663</v>
+        <v>5378</v>
       </c>
       <c r="AL45" s="20" t="n">
-        <v>76.229668609641</v>
+        <v>73.81274093424776</v>
       </c>
       <c r="AM45" s="18" t="b">
         <v>1</v>
@@ -9774,7 +9672,7 @@
         <v>0</v>
       </c>
       <c r="BA45" s="5" t="n">
-        <v>15.49474447263501</v>
+        <v>2.537151141718014</v>
       </c>
       <c r="BB45" s="5" t="n">
         <v>5.799202609641174</v>
@@ -9817,14 +9715,14 @@
       </c>
       <c r="I46" s="15" t="inlineStr">
         <is>
-          <t>[14, 19, 5, 14]</t>
+          <t>[14, 3, 4, 14]</t>
         </is>
       </c>
       <c r="J46" s="16" t="n">
-        <v>3539</v>
+        <v>4132</v>
       </c>
       <c r="K46" s="17" t="n">
-        <v>75.84533600861732</v>
+        <v>63.4815652406223</v>
       </c>
       <c r="L46" s="15" t="b">
         <v>1</v>
@@ -9880,7 +9778,7 @@
         <v>0</v>
       </c>
       <c r="AA46" s="5" t="n">
-        <v>18.58753163100989</v>
+        <v>4.945939728548424</v>
       </c>
       <c r="AB46" s="5" t="n">
         <v>0</v>
@@ -9912,14 +9810,14 @@
       </c>
       <c r="AJ46" s="18" t="inlineStr">
         <is>
-          <t>[14, 19, 5, 14]</t>
+          <t>[14, 3, 4, 14]</t>
         </is>
       </c>
       <c r="AK46" s="19" t="n">
-        <v>3539</v>
+        <v>4132</v>
       </c>
       <c r="AL46" s="20" t="n">
-        <v>75.84533600861732</v>
+        <v>63.4815652406223</v>
       </c>
       <c r="AM46" s="18" t="b">
         <v>1</v>
@@ -9970,7 +9868,7 @@
         <v>0</v>
       </c>
       <c r="BA46" s="5" t="n">
-        <v>18.58753163100989</v>
+        <v>4.945939728548424</v>
       </c>
       <c r="BB46" s="5" t="n">
         <v>0</v>
@@ -10013,14 +9911,14 @@
       </c>
       <c r="I47" s="15" t="inlineStr">
         <is>
-          <t>[14, 19, 5, 14]</t>
+          <t>[14, 33, 10, 14]</t>
         </is>
       </c>
       <c r="J47" s="16" t="n">
-        <v>3140</v>
+        <v>3324</v>
       </c>
       <c r="K47" s="17" t="n">
-        <v>75.84533600861732</v>
+        <v>76.86345503101833</v>
       </c>
       <c r="L47" s="15" t="b">
         <v>1</v>
@@ -10076,7 +9974,7 @@
         <v>0</v>
       </c>
       <c r="AA47" s="5" t="n">
-        <v>5.535499398315283</v>
+        <v>0</v>
       </c>
       <c r="AB47" s="5" t="n">
         <v>0</v>
@@ -10108,14 +10006,14 @@
       </c>
       <c r="AJ47" s="18" t="inlineStr">
         <is>
-          <t>[14, 19, 5, 14]</t>
+          <t>[14, 33, 10, 14]</t>
         </is>
       </c>
       <c r="AK47" s="19" t="n">
-        <v>3140</v>
+        <v>3324</v>
       </c>
       <c r="AL47" s="20" t="n">
-        <v>75.84533600861732</v>
+        <v>76.86345503101833</v>
       </c>
       <c r="AM47" s="18" t="b">
         <v>1</v>
@@ -10166,7 +10064,7 @@
         <v>0</v>
       </c>
       <c r="BA47" s="5" t="n">
-        <v>5.535499398315283</v>
+        <v>0</v>
       </c>
       <c r="BB47" s="5" t="n">
         <v>0</v>
@@ -10405,14 +10303,14 @@
       </c>
       <c r="I49" s="15" t="inlineStr">
         <is>
-          <t>[15, 28, 27, 0, 30, 15]</t>
+          <t>[15, 30, 26, 27, 0, 32, 15]</t>
         </is>
       </c>
       <c r="J49" s="16" t="n">
-        <v>3829</v>
+        <v>5266</v>
       </c>
       <c r="K49" s="17" t="n">
-        <v>56.31056538297734</v>
+        <v>74.58649448949348</v>
       </c>
       <c r="L49" s="15" t="b">
         <v>1</v>
@@ -10468,7 +10366,7 @@
         <v>0</v>
       </c>
       <c r="AA49" s="5" t="n">
-        <v>27.28826433725788</v>
+        <v>0</v>
       </c>
       <c r="AB49" s="5" t="n">
         <v>0</v>
@@ -10500,14 +10398,14 @@
       </c>
       <c r="AJ49" s="18" t="inlineStr">
         <is>
-          <t>[15, 32, 23, 11, 6, 28, 15]</t>
+          <t>[15, 30, 26, 27, 0, 32, 15]</t>
         </is>
       </c>
       <c r="AK49" s="19" t="n">
-        <v>4567</v>
+        <v>5266</v>
       </c>
       <c r="AL49" s="20" t="n">
-        <v>68.80721202182097</v>
+        <v>74.58649448949348</v>
       </c>
       <c r="AM49" s="18" t="b">
         <v>1</v>
@@ -10558,7 +10456,7 @@
         <v>0</v>
       </c>
       <c r="BA49" s="5" t="n">
-        <v>13.27383213064945</v>
+        <v>0</v>
       </c>
       <c r="BB49" s="5" t="n">
         <v>9.077098366881883</v>
@@ -10601,14 +10499,14 @@
       </c>
       <c r="I50" s="15" t="inlineStr">
         <is>
-          <t>[15, 27, 0, 26, 30, 15]</t>
+          <t>[15, 32, 23, 11, 28, 15]</t>
         </is>
       </c>
       <c r="J50" s="16" t="n">
-        <v>3752</v>
+        <v>4327</v>
       </c>
       <c r="K50" s="17" t="n">
-        <v>72.11445761460965</v>
+        <v>63.51717547150033</v>
       </c>
       <c r="L50" s="15" t="b">
         <v>1</v>
@@ -10664,7 +10562,7 @@
         <v>0</v>
       </c>
       <c r="AA50" s="5" t="n">
-        <v>26.60406885758999</v>
+        <v>15.35602503912363</v>
       </c>
       <c r="AB50" s="5" t="n">
         <v>2.36697965571205</v>
@@ -10696,14 +10594,14 @@
       </c>
       <c r="AJ50" s="18" t="inlineStr">
         <is>
-          <t>[15, 32, 23, 11, 28, 15]</t>
+          <t>[15, 30, 27, 0, 32, 28, 15]</t>
         </is>
       </c>
       <c r="AK50" s="19" t="n">
-        <v>4327</v>
+        <v>4975</v>
       </c>
       <c r="AL50" s="20" t="n">
-        <v>63.51717547150033</v>
+        <v>71.99648707255528</v>
       </c>
       <c r="AM50" s="18" t="b">
         <v>1</v>
@@ -10754,7 +10652,7 @@
         <v>0</v>
       </c>
       <c r="BA50" s="5" t="n">
-        <v>15.35602503912363</v>
+        <v>2.679968701095462</v>
       </c>
       <c r="BB50" s="5" t="n">
         <v>11.15023474178404</v>
@@ -10797,14 +10695,14 @@
       </c>
       <c r="I51" s="15" t="inlineStr">
         <is>
-          <t>[15, 27, 0, 26, 30, 15]</t>
+          <t>[15, 28, 1, 16, 32, 15]</t>
         </is>
       </c>
       <c r="J51" s="16" t="n">
-        <v>4139</v>
+        <v>4442</v>
       </c>
       <c r="K51" s="17" t="n">
-        <v>72.11445761460965</v>
+        <v>76.5146070335218</v>
       </c>
       <c r="L51" s="15" t="b">
         <v>1</v>
@@ -10860,7 +10758,7 @@
         <v>0</v>
       </c>
       <c r="AA51" s="5" t="n">
-        <v>19.84895429899303</v>
+        <v>13.98140975987607</v>
       </c>
       <c r="AB51" s="5" t="n">
         <v>0</v>
@@ -10892,14 +10790,14 @@
       </c>
       <c r="AJ51" s="18" t="inlineStr">
         <is>
-          <t>[15, 27, 0, 26, 30, 15]</t>
+          <t>[15, 28, 30, 27, 0, 32, 15]</t>
         </is>
       </c>
       <c r="AK51" s="19" t="n">
-        <v>4139</v>
+        <v>5164</v>
       </c>
       <c r="AL51" s="20" t="n">
-        <v>72.11445761460965</v>
+        <v>76.11262178500536</v>
       </c>
       <c r="AM51" s="18" t="b">
         <v>1</v>
@@ -10950,7 +10848,7 @@
         <v>0</v>
       </c>
       <c r="BA51" s="5" t="n">
-        <v>19.84895429899303</v>
+        <v>0</v>
       </c>
       <c r="BB51" s="5" t="n">
         <v>9.9147947327653</v>
@@ -10993,14 +10891,14 @@
       </c>
       <c r="I52" s="15" t="inlineStr">
         <is>
-          <t>[16, 31, 32, 23, 1, 12, 16]</t>
+          <t>[16, 34, 23, 32, 1, 12, 16]</t>
         </is>
       </c>
       <c r="J52" s="16" t="n">
-        <v>4863</v>
+        <v>4652</v>
       </c>
       <c r="K52" s="17" t="n">
-        <v>75.34279720288458</v>
+        <v>76.2305482238408</v>
       </c>
       <c r="L52" s="15" t="b">
         <v>1</v>
@@ -11056,7 +10954,7 @@
         <v>0</v>
       </c>
       <c r="AA52" s="5" t="n">
-        <v>16.75795960287573</v>
+        <v>20.36973639164669</v>
       </c>
       <c r="AB52" s="5" t="n">
         <v>0</v>
@@ -11088,14 +10986,14 @@
       </c>
       <c r="AJ52" s="18" t="inlineStr">
         <is>
-          <t>[16, 32, 23, 11, 1, 16]</t>
+          <t>[16, 31, 12, 34, 23, 1, 32, 16]</t>
         </is>
       </c>
       <c r="AK52" s="19" t="n">
-        <v>4530</v>
+        <v>5447</v>
       </c>
       <c r="AL52" s="20" t="n">
-        <v>72.63749840307037</v>
+        <v>74.13570591081958</v>
       </c>
       <c r="AM52" s="18" t="b">
         <v>1</v>
@@ -11146,7 +11044,7 @@
         <v>0</v>
       </c>
       <c r="BA52" s="5" t="n">
-        <v>22.45806230742896</v>
+        <v>6.761383087983567</v>
       </c>
       <c r="BB52" s="5" t="n">
         <v>19.89044847654913</v>
@@ -11189,14 +11087,14 @@
       </c>
       <c r="I53" s="15" t="inlineStr">
         <is>
-          <t>[16, 0, 27, 30, 32, 16]</t>
+          <t>[16, 34, 31, 23, 32, 16]</t>
         </is>
       </c>
       <c r="J53" s="16" t="n">
-        <v>4684</v>
+        <v>4984</v>
       </c>
       <c r="K53" s="17" t="n">
-        <v>76.30266589653553</v>
+        <v>73.1911804597428</v>
       </c>
       <c r="L53" s="15" t="b">
         <v>1</v>
@@ -11252,7 +11150,7 @@
         <v>0</v>
       </c>
       <c r="AA53" s="5" t="n">
-        <v>16.17752326413743</v>
+        <v>10.80887616320687</v>
       </c>
       <c r="AB53" s="5" t="n">
         <v>0</v>
@@ -11284,14 +11182,14 @@
       </c>
       <c r="AJ53" s="18" t="inlineStr">
         <is>
-          <t>[16, 0, 27, 30, 32, 16]</t>
+          <t>[16, 34, 31, 12, 17, 1, 32, 16]</t>
         </is>
       </c>
       <c r="AK53" s="19" t="n">
-        <v>4684</v>
+        <v>5401</v>
       </c>
       <c r="AL53" s="20" t="n">
-        <v>76.30266589653553</v>
+        <v>72.5721514654558</v>
       </c>
       <c r="AM53" s="18" t="b">
         <v>1</v>
@@ -11342,7 +11240,7 @@
         <v>0</v>
       </c>
       <c r="BA53" s="5" t="n">
-        <v>16.17752326413743</v>
+        <v>3.346456692913386</v>
       </c>
       <c r="BB53" s="5" t="n">
         <v>5.368647100930565</v>
@@ -11385,14 +11283,14 @@
       </c>
       <c r="I54" s="15" t="inlineStr">
         <is>
-          <t>[16, 1, 15, 28, 32, 16]</t>
+          <t>[16, 32, 23, 1, 31, 12, 34, 16]</t>
         </is>
       </c>
       <c r="J54" s="16" t="n">
-        <v>4762</v>
+        <v>5895</v>
       </c>
       <c r="K54" s="17" t="n">
-        <v>76.76485671650801</v>
+        <v>75.53118521626951</v>
       </c>
       <c r="L54" s="15" t="b">
         <v>1</v>
@@ -11448,7 +11346,7 @@
         <v>0</v>
       </c>
       <c r="AA54" s="5" t="n">
-        <v>21.7933979306947</v>
+        <v>3.186073246838561</v>
       </c>
       <c r="AB54" s="5" t="n">
         <v>0</v>
@@ -11480,14 +11378,14 @@
       </c>
       <c r="AJ54" s="18" t="inlineStr">
         <is>
-          <t>[16, 32, 23, 17, 31, 16]</t>
+          <t>[16, 31, 34, 12, 17, 1, 32, 16]</t>
         </is>
       </c>
       <c r="AK54" s="19" t="n">
-        <v>5418</v>
+        <v>5273</v>
       </c>
       <c r="AL54" s="20" t="n">
-        <v>72.35135449120544</v>
+        <v>72.30535305191131</v>
       </c>
       <c r="AM54" s="18" t="b">
         <v>1</v>
@@ -11538,7 +11436,7 @@
         <v>0</v>
       </c>
       <c r="BA54" s="5" t="n">
-        <v>11.01987190014781</v>
+        <v>13.40121530629003</v>
       </c>
       <c r="BB54" s="5" t="n">
         <v>0</v>
@@ -11581,14 +11479,14 @@
       </c>
       <c r="I55" s="15" t="inlineStr">
         <is>
-          <t>[17, 16, 34, 13, 23, 17]</t>
+          <t>[17, 16, 31, 34, 12, 1, 23, 17]</t>
         </is>
       </c>
       <c r="J55" s="16" t="n">
-        <v>4830</v>
+        <v>5429</v>
       </c>
       <c r="K55" s="17" t="n">
-        <v>76.25890703910102</v>
+        <v>76.42768627131306</v>
       </c>
       <c r="L55" s="15" t="b">
         <v>1</v>
@@ -11644,7 +11542,7 @@
         <v>0</v>
       </c>
       <c r="AA55" s="5" t="n">
-        <v>14.84485190409027</v>
+        <v>4.284203102961919</v>
       </c>
       <c r="AB55" s="5" t="n">
         <v>0</v>
@@ -11676,14 +11574,14 @@
       </c>
       <c r="AJ55" s="18" t="inlineStr">
         <is>
-          <t>[17, 16, 32, 23, 13, 17]</t>
+          <t>[17, 16, 31, 34, 12, 1, 23, 17]</t>
         </is>
       </c>
       <c r="AK55" s="19" t="n">
-        <v>4986</v>
+        <v>5429</v>
       </c>
       <c r="AL55" s="20" t="n">
-        <v>75.7315799968933</v>
+        <v>76.42768627131306</v>
       </c>
       <c r="AM55" s="18" t="b">
         <v>1</v>
@@ -11734,7 +11632,7 @@
         <v>0</v>
       </c>
       <c r="BA55" s="5" t="n">
-        <v>12.09449929478138</v>
+        <v>4.284203102961919</v>
       </c>
       <c r="BB55" s="5" t="n">
         <v>12.09449929478138</v>
@@ -11777,14 +11675,14 @@
       </c>
       <c r="I56" s="15" t="inlineStr">
         <is>
-          <t>[17, 23, 11, 28, 1, 34, 17]</t>
+          <t>[17, 23, 1, 12, 31, 34, 16, 17]</t>
         </is>
       </c>
       <c r="J56" s="16" t="n">
-        <v>5351</v>
+        <v>6237</v>
       </c>
       <c r="K56" s="17" t="n">
-        <v>76.1899113397222</v>
+        <v>76.54036331337797</v>
       </c>
       <c r="L56" s="15" t="b">
         <v>1</v>
@@ -11840,7 +11738,7 @@
         <v>0</v>
       </c>
       <c r="AA56" s="5" t="n">
-        <v>17.26963512677798</v>
+        <v>3.571428571428571</v>
       </c>
       <c r="AB56" s="5" t="n">
         <v>0</v>
@@ -11872,14 +11770,14 @@
       </c>
       <c r="AJ56" s="18" t="inlineStr">
         <is>
-          <t>[17, 23, 11, 28, 1, 34, 17]</t>
+          <t>[17, 23, 1, 12, 34, 16, 31, 17]</t>
         </is>
       </c>
       <c r="AK56" s="19" t="n">
-        <v>5351</v>
+        <v>6468</v>
       </c>
       <c r="AL56" s="20" t="n">
-        <v>76.1899113397222</v>
+        <v>76.77412151089311</v>
       </c>
       <c r="AM56" s="18" t="b">
         <v>1</v>
@@ -11930,7 +11828,7 @@
         <v>0</v>
       </c>
       <c r="BA56" s="5" t="n">
-        <v>17.26963512677798</v>
+        <v>0</v>
       </c>
       <c r="BB56" s="5" t="n">
         <v>30.70500927643785</v>
@@ -11973,14 +11871,14 @@
       </c>
       <c r="I57" s="15" t="inlineStr">
         <is>
-          <t>[17, 34, 28, 11, 23, 17]</t>
+          <t>[17, 16, 34, 31, 12, 1, 23, 17]</t>
         </is>
       </c>
       <c r="J57" s="16" t="n">
-        <v>4464</v>
+        <v>5215</v>
       </c>
       <c r="K57" s="17" t="n">
-        <v>76.18133393187054</v>
+        <v>76.69448468485756</v>
       </c>
       <c r="L57" s="15" t="b">
         <v>1</v>
@@ -12036,7 +11934,7 @@
         <v>0</v>
       </c>
       <c r="AA57" s="5" t="n">
-        <v>19.01306240928882</v>
+        <v>5.388243831640057</v>
       </c>
       <c r="AB57" s="5" t="n">
         <v>0</v>
@@ -12068,14 +11966,14 @@
       </c>
       <c r="AJ57" s="18" t="inlineStr">
         <is>
-          <t>[17, 34, 28, 11, 23, 17]</t>
+          <t>[17, 34, 16, 31, 12, 1, 23, 17]</t>
         </is>
       </c>
       <c r="AK57" s="19" t="n">
-        <v>4464</v>
+        <v>5195</v>
       </c>
       <c r="AL57" s="20" t="n">
-        <v>76.18133393187054</v>
+        <v>70.20300405918695</v>
       </c>
       <c r="AM57" s="18" t="b">
         <v>1</v>
@@ -12126,7 +12024,7 @@
         <v>0</v>
       </c>
       <c r="BA57" s="5" t="n">
-        <v>19.01306240928882</v>
+        <v>5.751088534107402</v>
       </c>
       <c r="BB57" s="5" t="n">
         <v>28.37445573294629</v>
@@ -12264,14 +12162,14 @@
       </c>
       <c r="AJ58" s="18" t="inlineStr">
         <is>
-          <t>[18, 29, 13, 2, 18]</t>
+          <t>[18, 2, 13, 23, 11, 8, 18]</t>
         </is>
       </c>
       <c r="AK58" s="19" t="n">
-        <v>4162</v>
+        <v>5233</v>
       </c>
       <c r="AL58" s="20" t="n">
-        <v>69.37263132606104</v>
+        <v>76.11688487342524</v>
       </c>
       <c r="AM58" s="18" t="b">
         <v>1</v>
@@ -12322,7 +12220,7 @@
         <v>0</v>
       </c>
       <c r="BA58" s="5" t="n">
-        <v>20.46627173705332</v>
+        <v>0</v>
       </c>
       <c r="BB58" s="5" t="n">
         <v>20.46627173705332</v>
@@ -12365,14 +12263,14 @@
       </c>
       <c r="I59" s="15" t="inlineStr">
         <is>
-          <t>[18, 1, 23, 13, 2, 18]</t>
+          <t>[18, 2, 13, 8, 29, 18]</t>
         </is>
       </c>
       <c r="J59" s="16" t="n">
-        <v>3888</v>
+        <v>3968</v>
       </c>
       <c r="K59" s="17" t="n">
-        <v>72.29713270193817</v>
+        <v>69.18855473644203</v>
       </c>
       <c r="L59" s="15" t="b">
         <v>1</v>
@@ -12428,7 +12326,7 @@
         <v>0</v>
       </c>
       <c r="AA59" s="5" t="n">
-        <v>21.54963680387409</v>
+        <v>19.93543179983858</v>
       </c>
       <c r="AB59" s="5" t="n">
         <v>10.49233252623083</v>
@@ -12460,14 +12358,14 @@
       </c>
       <c r="AJ59" s="18" t="inlineStr">
         <is>
-          <t>[18, 1, 23, 13, 2, 18]</t>
+          <t>[18, 2, 13, 23, 11, 8, 18]</t>
         </is>
       </c>
       <c r="AK59" s="19" t="n">
-        <v>3888</v>
+        <v>4956</v>
       </c>
       <c r="AL59" s="20" t="n">
-        <v>72.29713270193817</v>
+        <v>76.11688487342524</v>
       </c>
       <c r="AM59" s="18" t="b">
         <v>1</v>
@@ -12518,7 +12416,7 @@
         <v>0</v>
       </c>
       <c r="BA59" s="5" t="n">
-        <v>21.54963680387409</v>
+        <v>0</v>
       </c>
       <c r="BB59" s="5" t="n">
         <v>5.104923325262308</v>
@@ -14521,14 +14419,14 @@
       </c>
       <c r="I70" s="15" t="inlineStr">
         <is>
-          <t>[22, 17, 19, 22]</t>
+          <t>[22, 17, 34, 12, 22]</t>
         </is>
       </c>
       <c r="J70" s="16" t="n">
-        <v>3093</v>
+        <v>3132</v>
       </c>
       <c r="K70" s="17" t="n">
-        <v>61.46521819304558</v>
+        <v>63.5149522683278</v>
       </c>
       <c r="L70" s="15" t="b">
         <v>1</v>
@@ -14584,7 +14482,7 @@
         <v>0</v>
       </c>
       <c r="AA70" s="5" t="n">
-        <v>1.245210727969349</v>
+        <v>0</v>
       </c>
       <c r="AB70" s="5" t="n">
         <v>0</v>
@@ -15109,14 +15007,14 @@
       </c>
       <c r="I73" s="15" t="inlineStr">
         <is>
-          <t>[23, 1, 28, 24, 6, 11, 23]</t>
+          <t>[23, 13, 32, 28, 11, 23]</t>
         </is>
       </c>
       <c r="J73" s="16" t="n">
-        <v>4915</v>
+        <v>4473</v>
       </c>
       <c r="K73" s="17" t="n">
-        <v>74.74858517898794</v>
+        <v>76.18882301483481</v>
       </c>
       <c r="L73" s="15" t="b">
         <v>1</v>
@@ -15172,7 +15070,7 @@
         <v>0</v>
       </c>
       <c r="AA73" s="5" t="n">
-        <v>15.17086641353124</v>
+        <v>22.79944770452192</v>
       </c>
       <c r="AB73" s="5" t="n">
         <v>0</v>
@@ -15204,14 +15102,14 @@
       </c>
       <c r="AJ73" s="18" t="inlineStr">
         <is>
-          <t>[23, 1, 28, 24, 6, 11, 23]</t>
+          <t>[23, 11, 13, 1, 34, 12, 31, 23]</t>
         </is>
       </c>
       <c r="AK73" s="19" t="n">
-        <v>4915</v>
+        <v>5127</v>
       </c>
       <c r="AL73" s="20" t="n">
-        <v>74.74858517898794</v>
+        <v>76.87628149444748</v>
       </c>
       <c r="AM73" s="18" t="b">
         <v>1</v>
@@ -15262,7 +15160,7 @@
         <v>0</v>
       </c>
       <c r="BA73" s="5" t="n">
-        <v>15.17086641353124</v>
+        <v>11.51190887124612</v>
       </c>
       <c r="BB73" s="5" t="n">
         <v>11.51190887124612</v>
@@ -15305,14 +15203,14 @@
       </c>
       <c r="I74" s="15" t="inlineStr">
         <is>
-          <t>[23, 1, 15, 28, 6, 24, 11, 23]</t>
+          <t>[23, 1, 15, 28, 24, 11, 23]</t>
         </is>
       </c>
       <c r="J74" s="16" t="n">
-        <v>5723</v>
+        <v>5416</v>
       </c>
       <c r="K74" s="17" t="n">
-        <v>74.8418810837676</v>
+        <v>75.65980089436411</v>
       </c>
       <c r="L74" s="15" t="b">
         <v>1</v>
@@ -15368,7 +15266,7 @@
         <v>0</v>
       </c>
       <c r="AA74" s="5" t="n">
-        <v>8.999840992208618</v>
+        <v>13.88138018762919</v>
       </c>
       <c r="AB74" s="5" t="n">
         <v>0</v>
@@ -15400,14 +15298,14 @@
       </c>
       <c r="AJ74" s="18" t="inlineStr">
         <is>
-          <t>[23, 1, 15, 28, 6, 24, 11, 23]</t>
+          <t>[23, 1, 12, 31, 34, 16, 32, 23]</t>
         </is>
       </c>
       <c r="AK74" s="19" t="n">
-        <v>5723</v>
+        <v>6289</v>
       </c>
       <c r="AL74" s="20" t="n">
-        <v>74.8418810837676</v>
+        <v>75.11269845882313</v>
       </c>
       <c r="AM74" s="18" t="b">
         <v>1</v>
@@ -15458,7 +15356,7 @@
         <v>0</v>
       </c>
       <c r="BA74" s="5" t="n">
-        <v>8.999840992208618</v>
+        <v>0</v>
       </c>
       <c r="BB74" s="5" t="n">
         <v>7.362060740976307</v>
@@ -15501,14 +15399,14 @@
       </c>
       <c r="I75" s="15" t="inlineStr">
         <is>
-          <t>[23, 13, 7, 6, 11, 23]</t>
+          <t>[23, 32, 28, 11, 13, 23]</t>
         </is>
       </c>
       <c r="J75" s="16" t="n">
-        <v>4200</v>
+        <v>4533</v>
       </c>
       <c r="K75" s="17" t="n">
-        <v>73.06439751541267</v>
+        <v>69.07047928218503</v>
       </c>
       <c r="L75" s="15" t="b">
         <v>1</v>
@@ -15564,7 +15462,7 @@
         <v>0</v>
       </c>
       <c r="AA75" s="5" t="n">
-        <v>27.23492723492724</v>
+        <v>21.46569646569646</v>
       </c>
       <c r="AB75" s="5" t="n">
         <v>2.165627165627166</v>
@@ -15596,14 +15494,14 @@
       </c>
       <c r="AJ75" s="18" t="inlineStr">
         <is>
-          <t>[23, 32, 28, 15, 11, 23]</t>
+          <t>[23, 13, 17, 34, 12, 31, 32, 23]</t>
         </is>
       </c>
       <c r="AK75" s="19" t="n">
-        <v>4445</v>
+        <v>5687</v>
       </c>
       <c r="AL75" s="20" t="n">
-        <v>71.48623866776363</v>
+        <v>76.58381500748465</v>
       </c>
       <c r="AM75" s="18" t="b">
         <v>1</v>
@@ -15654,7 +15552,7 @@
         <v>0</v>
       </c>
       <c r="BA75" s="5" t="n">
-        <v>22.99029799029799</v>
+        <v>1.472626472626473</v>
       </c>
       <c r="BB75" s="5" t="n">
         <v>13.79071379071379</v>
@@ -15893,14 +15791,14 @@
       </c>
       <c r="I77" s="15" t="inlineStr">
         <is>
-          <t>[24, 7, 28, 15, 11, 24]</t>
+          <t>[24, 6, 7, 11, 28, 24]</t>
         </is>
       </c>
       <c r="J77" s="16" t="n">
-        <v>4144</v>
+        <v>4178</v>
       </c>
       <c r="K77" s="17" t="n">
-        <v>72.98261099156952</v>
+        <v>74.11489988317319</v>
       </c>
       <c r="L77" s="15" t="b">
         <v>1</v>
@@ -15956,7 +15854,7 @@
         <v>0</v>
       </c>
       <c r="AA77" s="5" t="n">
-        <v>20.35364212954065</v>
+        <v>19.70017297712858</v>
       </c>
       <c r="AB77" s="5" t="n">
         <v>0</v>
@@ -15988,14 +15886,14 @@
       </c>
       <c r="AJ77" s="18" t="inlineStr">
         <is>
-          <t>[24, 7, 28, 23, 11, 24]</t>
+          <t>[24, 6, 11, 23, 13, 28, 24]</t>
         </is>
       </c>
       <c r="AK77" s="19" t="n">
-        <v>4621</v>
+        <v>5043</v>
       </c>
       <c r="AL77" s="20" t="n">
-        <v>75.83608168317812</v>
+        <v>71.05408971316373</v>
       </c>
       <c r="AM77" s="18" t="b">
         <v>1</v>
@@ -16046,7 +15944,7 @@
         <v>0</v>
       </c>
       <c r="BA77" s="5" t="n">
-        <v>11.18585431481837</v>
+        <v>3.075148952527388</v>
       </c>
       <c r="BB77" s="5" t="n">
         <v>10.78224101479915</v>
@@ -16873,14 +16771,14 @@
       </c>
       <c r="I82" s="15" t="inlineStr">
         <is>
-          <t>[26, 27, 15, 28, 30, 26]</t>
+          <t>[26, 32, 27, 0, 30, 26]</t>
         </is>
       </c>
       <c r="J82" s="16" t="n">
-        <v>4131</v>
+        <v>4002</v>
       </c>
       <c r="K82" s="17" t="n">
-        <v>67.64939649894049</v>
+        <v>76.92218514933194</v>
       </c>
       <c r="L82" s="15" t="b">
         <v>1</v>
@@ -16936,7 +16834,7 @@
         <v>0</v>
       </c>
       <c r="AA82" s="5" t="n">
-        <v>13.77582968065122</v>
+        <v>16.46837820914214</v>
       </c>
       <c r="AB82" s="5" t="n">
         <v>0</v>
@@ -17069,14 +16967,14 @@
       </c>
       <c r="I83" s="15" t="inlineStr">
         <is>
-          <t>[26, 30, 27, 0, 26]</t>
+          <t>[26, 32, 27, 30, 0, 26]</t>
         </is>
       </c>
       <c r="J83" s="16" t="n">
-        <v>3533</v>
+        <v>3594</v>
       </c>
       <c r="K83" s="17" t="n">
-        <v>55.68327082178065</v>
+        <v>76.91993454870524</v>
       </c>
       <c r="L83" s="15" t="b">
         <v>1</v>
@@ -17132,7 +17030,7 @@
         <v>0</v>
       </c>
       <c r="AA83" s="5" t="n">
-        <v>28.35124721151896</v>
+        <v>27.11417562360576</v>
       </c>
       <c r="AB83" s="5" t="n">
         <v>0</v>
@@ -17164,14 +17062,14 @@
       </c>
       <c r="AJ83" s="18" t="inlineStr">
         <is>
-          <t>[26, 0, 27, 15, 30, 26]</t>
+          <t>[26, 0, 15, 32, 30, 27, 26]</t>
         </is>
       </c>
       <c r="AK83" s="19" t="n">
-        <v>4094</v>
+        <v>4931</v>
       </c>
       <c r="AL83" s="20" t="n">
-        <v>71.99200992760311</v>
+        <v>75.54466765939436</v>
       </c>
       <c r="AM83" s="18" t="b">
         <v>1</v>
@@ -17222,7 +17120,7 @@
         <v>0</v>
       </c>
       <c r="BA83" s="5" t="n">
-        <v>16.97424457513689</v>
+        <v>0</v>
       </c>
       <c r="BB83" s="5" t="n">
         <v>0</v>
@@ -17265,14 +17163,14 @@
       </c>
       <c r="I84" s="15" t="inlineStr">
         <is>
-          <t>[26, 32, 15, 0, 27, 26]</t>
+          <t>[26, 15, 27, 0, 26]</t>
         </is>
       </c>
       <c r="J84" s="16" t="n">
-        <v>3665</v>
+        <v>3584</v>
       </c>
       <c r="K84" s="17" t="n">
-        <v>68.63828577887914</v>
+        <v>71.8104412073879</v>
       </c>
       <c r="L84" s="15" t="b">
         <v>1</v>
@@ -17328,7 +17226,7 @@
         <v>0</v>
       </c>
       <c r="AA84" s="5" t="n">
-        <v>20.9277238403452</v>
+        <v>22.67529665587918</v>
       </c>
       <c r="AB84" s="5" t="n">
         <v>0</v>
@@ -17360,14 +17258,14 @@
       </c>
       <c r="AJ84" s="18" t="inlineStr">
         <is>
-          <t>[26, 32, 15, 0, 30, 27, 26]</t>
+          <t>[26, 27, 0, 15, 32, 30, 26]</t>
         </is>
       </c>
       <c r="AK84" s="19" t="n">
-        <v>4272</v>
+        <v>4616</v>
       </c>
       <c r="AL84" s="20" t="n">
-        <v>74.49544940808406</v>
+        <v>75.5383145684329</v>
       </c>
       <c r="AM84" s="18" t="b">
         <v>1</v>
@@ -17418,7 +17316,7 @@
         <v>0</v>
       </c>
       <c r="BA84" s="5" t="n">
-        <v>7.831715210355987</v>
+        <v>0.4099244875943905</v>
       </c>
       <c r="BB84" s="5" t="n">
         <v>4.681769147788565</v>
@@ -17461,14 +17359,14 @@
       </c>
       <c r="I85" s="15" t="inlineStr">
         <is>
-          <t>[27, 0, 26, 30, 15, 27]</t>
+          <t>[27, 0, 32, 16, 30, 27]</t>
         </is>
       </c>
       <c r="J85" s="16" t="n">
-        <v>4092</v>
+        <v>4750</v>
       </c>
       <c r="K85" s="17" t="n">
-        <v>72.11445761460965</v>
+        <v>76.77474853392994</v>
       </c>
       <c r="L85" s="15" t="b">
         <v>1</v>
@@ -17524,7 +17422,7 @@
         <v>0</v>
       </c>
       <c r="AA85" s="5" t="n">
-        <v>19.85898942420681</v>
+        <v>6.972189580885233</v>
       </c>
       <c r="AB85" s="5" t="n">
         <v>-3.388170779475128</v>
@@ -17657,14 +17555,14 @@
       </c>
       <c r="I86" s="15" t="inlineStr">
         <is>
-          <t>[27, 0, 26, 15, 30, 27]</t>
+          <t>[27, 0, 26, 32, 30, 27]</t>
         </is>
       </c>
       <c r="J86" s="16" t="n">
-        <v>3735</v>
+        <v>3841</v>
       </c>
       <c r="K86" s="17" t="n">
-        <v>71.99201126406429</v>
+        <v>74.68578731833021</v>
       </c>
       <c r="L86" s="15" t="b">
         <v>1</v>
@@ -17720,7 +17618,7 @@
         <v>0</v>
       </c>
       <c r="AA86" s="5" t="n">
-        <v>23.02143446001649</v>
+        <v>20.83676834295136</v>
       </c>
       <c r="AB86" s="5" t="n">
         <v>0</v>
@@ -17752,14 +17650,14 @@
       </c>
       <c r="AJ86" s="18" t="inlineStr">
         <is>
-          <t>[27, 15, 26, 0, 27]</t>
+          <t>[27, 0, 32, 28, 15, 30, 27]</t>
         </is>
       </c>
       <c r="AK86" s="19" t="n">
-        <v>3245</v>
+        <v>4761</v>
       </c>
       <c r="AL86" s="20" t="n">
-        <v>71.81044143013141</v>
+        <v>71.99648707255528</v>
       </c>
       <c r="AM86" s="18" t="b">
         <v>1</v>
@@ -17810,7 +17708,7 @@
         <v>0</v>
       </c>
       <c r="BA86" s="5" t="n">
-        <v>33.12036273701566</v>
+        <v>1.875515251442704</v>
       </c>
       <c r="BB86" s="5" t="n">
         <v>0</v>
@@ -17853,14 +17751,14 @@
       </c>
       <c r="I87" s="15" t="inlineStr">
         <is>
-          <t>[27, 0, 26, 30, 15, 27]</t>
+          <t>[27, 30, 32, 16, 0, 27]</t>
         </is>
       </c>
       <c r="J87" s="16" t="n">
-        <v>4151</v>
+        <v>4898</v>
       </c>
       <c r="K87" s="17" t="n">
-        <v>72.11445761460965</v>
+        <v>76.30266589653553</v>
       </c>
       <c r="L87" s="15" t="b">
         <v>1</v>
@@ -17916,7 +17814,7 @@
         <v>0</v>
       </c>
       <c r="AA87" s="5" t="n">
-        <v>16.76358532183678</v>
+        <v>1.784640064166834</v>
       </c>
       <c r="AB87" s="5" t="n">
         <v>-0.08020854220974534</v>
@@ -17948,14 +17846,14 @@
       </c>
       <c r="AJ87" s="18" t="inlineStr">
         <is>
-          <t>[27, 0, 26, 32, 30, 27]</t>
+          <t>[27, 0, 32, 28, 15, 30, 27]</t>
         </is>
       </c>
       <c r="AK87" s="19" t="n">
-        <v>4318</v>
+        <v>4937</v>
       </c>
       <c r="AL87" s="20" t="n">
-        <v>74.68578731833021</v>
+        <v>71.99648707255528</v>
       </c>
       <c r="AM87" s="18" t="b">
         <v>1</v>
@@ -18006,7 +17904,7 @@
         <v>0</v>
       </c>
       <c r="BA87" s="5" t="n">
-        <v>13.41487868457991</v>
+        <v>1.002606777621817</v>
       </c>
       <c r="BB87" s="5" t="n">
         <v>0</v>
@@ -18049,14 +17947,14 @@
       </c>
       <c r="I88" s="15" t="inlineStr">
         <is>
-          <t>[28, 6, 27, 0, 30, 15, 28]</t>
+          <t>[28, 27, 0, 15, 6, 28]</t>
         </is>
       </c>
       <c r="J88" s="16" t="n">
-        <v>4946</v>
+        <v>4707</v>
       </c>
       <c r="K88" s="17" t="n">
-        <v>74.8499243526344</v>
+        <v>74.48323704856701</v>
       </c>
       <c r="L88" s="15" t="b">
         <v>1</v>
@@ -18112,7 +18010,7 @@
         <v>0</v>
       </c>
       <c r="AA88" s="5" t="n">
-        <v>7.169669669669669</v>
+        <v>11.65540540540541</v>
       </c>
       <c r="AB88" s="5" t="n">
         <v>3.190690690690691</v>
@@ -18245,14 +18143,14 @@
       </c>
       <c r="I89" s="15" t="inlineStr">
         <is>
-          <t>[28, 6, 27, 0, 30, 15, 28]</t>
+          <t>[28, 15, 32, 23, 11, 6, 28]</t>
         </is>
       </c>
       <c r="J89" s="16" t="n">
-        <v>4527</v>
+        <v>4726</v>
       </c>
       <c r="K89" s="17" t="n">
-        <v>74.8499243526344</v>
+        <v>68.80721202182097</v>
       </c>
       <c r="L89" s="15" t="b">
         <v>1</v>
@@ -18308,7 +18206,7 @@
         <v>0</v>
       </c>
       <c r="AA89" s="5" t="n">
-        <v>14.13125948406677</v>
+        <v>10.35660091047041</v>
       </c>
       <c r="AB89" s="5" t="n">
         <v>1.194992412746586</v>
@@ -18340,14 +18238,14 @@
       </c>
       <c r="AJ89" s="18" t="inlineStr">
         <is>
-          <t>[28, 1, 11, 6, 15, 28]</t>
+          <t>[28, 15, 30, 32, 23, 11, 6, 28]</t>
         </is>
       </c>
       <c r="AK89" s="19" t="n">
-        <v>4110</v>
+        <v>5126</v>
       </c>
       <c r="AL89" s="20" t="n">
-        <v>76.03247599000387</v>
+        <v>72.46790103387278</v>
       </c>
       <c r="AM89" s="18" t="b">
         <v>1</v>
@@ -18398,7 +18296,7 @@
         <v>0</v>
       </c>
       <c r="BA89" s="5" t="n">
-        <v>22.04097116843703</v>
+        <v>2.769347496206374</v>
       </c>
       <c r="BB89" s="5" t="n">
         <v>8.38391502276176</v>
@@ -18441,14 +18339,14 @@
       </c>
       <c r="I90" s="15" t="inlineStr">
         <is>
-          <t>[28, 6, 27, 0, 15, 28]</t>
+          <t>[28, 24, 13, 23, 11, 15, 28]</t>
         </is>
       </c>
       <c r="J90" s="16" t="n">
-        <v>4276</v>
+        <v>4620</v>
       </c>
       <c r="K90" s="17" t="n">
-        <v>74.54590794541265</v>
+        <v>76.64972214507708</v>
       </c>
       <c r="L90" s="15" t="b">
         <v>1</v>
@@ -18504,7 +18402,7 @@
         <v>0</v>
       </c>
       <c r="AA90" s="5" t="n">
-        <v>16.09105180533752</v>
+        <v>9.340659340659341</v>
       </c>
       <c r="AB90" s="5" t="n">
         <v>0</v>
@@ -18536,14 +18434,14 @@
       </c>
       <c r="AJ90" s="18" t="inlineStr">
         <is>
-          <t>[28, 30, 27, 0, 15, 11, 28]</t>
+          <t>[28, 30, 27, 0, 32, 15, 28]</t>
         </is>
       </c>
       <c r="AK90" s="19" t="n">
-        <v>4754</v>
+        <v>4948</v>
       </c>
       <c r="AL90" s="20" t="n">
-        <v>76.91777059531169</v>
+        <v>76.11262178500536</v>
       </c>
       <c r="AM90" s="18" t="b">
         <v>1</v>
@@ -18594,7 +18492,7 @@
         <v>0</v>
       </c>
       <c r="BA90" s="5" t="n">
-        <v>6.711145996860282</v>
+        <v>2.904238618524333</v>
       </c>
       <c r="BB90" s="5" t="n">
         <v>12.32339089481947</v>
@@ -18637,14 +18535,14 @@
       </c>
       <c r="I91" s="15" t="inlineStr">
         <is>
-          <t>[29, 13, 11, 8, 29]</t>
+          <t>[29, 2, 13, 18, 29]</t>
         </is>
       </c>
       <c r="J91" s="16" t="n">
-        <v>2755</v>
+        <v>2796</v>
       </c>
       <c r="K91" s="17" t="n">
-        <v>74.68409669493784</v>
+        <v>68.79768171714818</v>
       </c>
       <c r="L91" s="15" t="b">
         <v>1</v>
@@ -18700,7 +18598,7 @@
         <v>0</v>
       </c>
       <c r="AA91" s="5" t="n">
-        <v>7.982631930527723</v>
+        <v>6.613226452905812</v>
       </c>
       <c r="AB91" s="5" t="n">
         <v>0</v>
@@ -18833,14 +18731,14 @@
       </c>
       <c r="I92" s="15" t="inlineStr">
         <is>
-          <t>[29, 23, 13, 8, 29]</t>
+          <t>[29, 11, 13, 8, 29]</t>
         </is>
       </c>
       <c r="J92" s="16" t="n">
-        <v>3731</v>
+        <v>3946</v>
       </c>
       <c r="K92" s="17" t="n">
-        <v>69.87924455644378</v>
+        <v>74.53326791831809</v>
       </c>
       <c r="L92" s="15" t="b">
         <v>1</v>
@@ -18896,7 +18794,7 @@
         <v>0</v>
       </c>
       <c r="AA92" s="5" t="n">
-        <v>5.568210579600101</v>
+        <v>0.1265502404454568</v>
       </c>
       <c r="AB92" s="5" t="n">
         <v>0</v>
@@ -18928,14 +18826,14 @@
       </c>
       <c r="AJ92" s="18" t="inlineStr">
         <is>
-          <t>[29, 11, 13, 8, 29]</t>
+          <t>[29, 18, 2, 13, 8, 29]</t>
         </is>
       </c>
       <c r="AK92" s="19" t="n">
-        <v>3946</v>
+        <v>3951</v>
       </c>
       <c r="AL92" s="20" t="n">
-        <v>74.53326791831809</v>
+        <v>69.18855473644203</v>
       </c>
       <c r="AM92" s="18" t="b">
         <v>1</v>
@@ -18986,7 +18884,7 @@
         <v>0</v>
       </c>
       <c r="BA92" s="5" t="n">
-        <v>0.1265502404454568</v>
+        <v>0</v>
       </c>
       <c r="BB92" s="5" t="n">
         <v>0.1265502404454568</v>
@@ -19029,14 +18927,14 @@
       </c>
       <c r="I93" s="15" t="inlineStr">
         <is>
-          <t>[29, 13, 11, 8, 29]</t>
+          <t>[29, 18, 2, 13, 8, 29]</t>
         </is>
       </c>
       <c r="J93" s="16" t="n">
-        <v>3382</v>
+        <v>3377</v>
       </c>
       <c r="K93" s="17" t="n">
-        <v>74.68409669493784</v>
+        <v>69.18855473644203</v>
       </c>
       <c r="L93" s="15" t="b">
         <v>1</v>
@@ -19092,7 +18990,7 @@
         <v>0</v>
       </c>
       <c r="AA93" s="5" t="n">
-        <v>18.23017408123791</v>
+        <v>18.35106382978723</v>
       </c>
       <c r="AB93" s="5" t="n">
         <v>0</v>
@@ -19124,14 +19022,14 @@
       </c>
       <c r="AJ93" s="18" t="inlineStr">
         <is>
-          <t>[29, 13, 11, 8, 29]</t>
+          <t>[29, 2, 13, 23, 29]</t>
         </is>
       </c>
       <c r="AK93" s="19" t="n">
-        <v>3382</v>
+        <v>3664</v>
       </c>
       <c r="AL93" s="20" t="n">
-        <v>74.68409669493784</v>
+        <v>73.05730580690584</v>
       </c>
       <c r="AM93" s="18" t="b">
         <v>1</v>
@@ -19182,7 +19080,7 @@
         <v>0</v>
       </c>
       <c r="BA93" s="5" t="n">
-        <v>18.23017408123791</v>
+        <v>11.41199226305609</v>
       </c>
       <c r="BB93" s="5" t="n">
         <v>0</v>
@@ -19225,14 +19123,14 @@
       </c>
       <c r="I94" s="15" t="inlineStr">
         <is>
-          <t>[30, 27, 15, 28, 32, 30]</t>
+          <t>[30, 32, 23, 11, 28, 15, 0, 30]</t>
         </is>
       </c>
       <c r="J94" s="16" t="n">
-        <v>4114</v>
+        <v>5012</v>
       </c>
       <c r="K94" s="17" t="n">
-        <v>72.68549295147056</v>
+        <v>73.08182586017075</v>
       </c>
       <c r="L94" s="15" t="b">
         <v>1</v>
@@ -19288,7 +19186,7 @@
         <v>0</v>
       </c>
       <c r="AA94" s="5" t="n">
-        <v>18.35681682873586</v>
+        <v>0.5358205993252629</v>
       </c>
       <c r="AB94" s="5" t="n">
         <v>0</v>
@@ -19320,14 +19218,14 @@
       </c>
       <c r="AJ94" s="18" t="inlineStr">
         <is>
-          <t>[30, 32, 28, 15, 27, 0, 30]</t>
+          <t>[30, 27, 0, 15, 28, 32, 30]</t>
         </is>
       </c>
       <c r="AK94" s="19" t="n">
-        <v>4769</v>
+        <v>4809</v>
       </c>
       <c r="AL94" s="20" t="n">
-        <v>72.72533241375191</v>
+        <v>72.91611180167446</v>
       </c>
       <c r="AM94" s="18" t="b">
         <v>1</v>
@@ -19378,7 +19276,7 @@
         <v>0</v>
       </c>
       <c r="BA94" s="5" t="n">
-        <v>5.358205993252629</v>
+        <v>4.564397697955943</v>
       </c>
       <c r="BB94" s="5" t="n">
         <v>1.647152212740623</v>
@@ -19421,14 +19319,14 @@
       </c>
       <c r="I95" s="15" t="inlineStr">
         <is>
-          <t>[30, 27, 0, 15, 11, 28, 30]</t>
+          <t>[30, 32, 23, 11, 6, 28, 15, 30]</t>
         </is>
       </c>
       <c r="J95" s="16" t="n">
-        <v>4847</v>
+        <v>5257</v>
       </c>
       <c r="K95" s="17" t="n">
-        <v>76.91777059531171</v>
+        <v>72.46790103387276</v>
       </c>
       <c r="L95" s="15" t="b">
         <v>1</v>
@@ -19484,7 +19382,7 @@
         <v>0</v>
       </c>
       <c r="AA95" s="5" t="n">
-        <v>7.799124976222179</v>
+        <v>0</v>
       </c>
       <c r="AB95" s="5" t="n">
         <v>5.250142666920297</v>
@@ -19516,14 +19414,14 @@
       </c>
       <c r="AJ95" s="18" t="inlineStr">
         <is>
-          <t>[30, 27, 0, 15, 6, 28, 30]</t>
+          <t>[30, 27, 0, 15, 28, 11, 30]</t>
         </is>
       </c>
       <c r="AK95" s="19" t="n">
-        <v>4799</v>
+        <v>4937</v>
       </c>
       <c r="AL95" s="20" t="n">
-        <v>73.51814501913856</v>
+        <v>76.80221904799268</v>
       </c>
       <c r="AM95" s="18" t="b">
         <v>1</v>
@@ -19574,7 +19472,7 @@
         <v>0</v>
       </c>
       <c r="BA95" s="5" t="n">
-        <v>8.712193266121362</v>
+        <v>6.087121932661214</v>
       </c>
       <c r="BB95" s="5" t="n">
         <v>0</v>
@@ -19617,14 +19515,14 @@
       </c>
       <c r="I96" s="15" t="inlineStr">
         <is>
-          <t>[30, 27, 0, 15, 11, 28, 30]</t>
+          <t>[30, 32, 23, 28, 15, 0, 30]</t>
         </is>
       </c>
       <c r="J96" s="16" t="n">
-        <v>4971</v>
+        <v>4680</v>
       </c>
       <c r="K96" s="17" t="n">
-        <v>76.91777059531171</v>
+        <v>71.0738771346476</v>
       </c>
       <c r="L96" s="15" t="b">
         <v>1</v>
@@ -19680,7 +19578,7 @@
         <v>0</v>
       </c>
       <c r="AA96" s="5" t="n">
-        <v>5.745164960182024</v>
+        <v>11.26279863481229</v>
       </c>
       <c r="AB96" s="5" t="n">
         <v>5.745164960182024</v>
@@ -19712,14 +19610,14 @@
       </c>
       <c r="AJ96" s="18" t="inlineStr">
         <is>
-          <t>[30, 27, 0, 26, 15, 30]</t>
+          <t>[30, 32, 23, 11, 28, 15, 0, 30]</t>
         </is>
       </c>
       <c r="AK96" s="19" t="n">
-        <v>4380</v>
+        <v>5274</v>
       </c>
       <c r="AL96" s="20" t="n">
-        <v>71.99201126406429</v>
+        <v>73.08182586017075</v>
       </c>
       <c r="AM96" s="18" t="b">
         <v>1</v>
@@ -19770,7 +19668,7 @@
         <v>0</v>
       </c>
       <c r="BA96" s="5" t="n">
-        <v>16.95108077360637</v>
+        <v>0</v>
       </c>
       <c r="BB96" s="5" t="n">
         <v>9.878649981039061</v>
@@ -19813,14 +19711,14 @@
       </c>
       <c r="I97" s="15" t="inlineStr">
         <is>
-          <t>[31, 32, 23, 13, 1, 12, 31]</t>
+          <t>[31, 16, 32, 23, 1, 12, 34, 31]</t>
         </is>
       </c>
       <c r="J97" s="16" t="n">
-        <v>4957</v>
+        <v>6177</v>
       </c>
       <c r="K97" s="17" t="n">
-        <v>74.09062907991833</v>
+        <v>75.08232804674387</v>
       </c>
       <c r="L97" s="15" t="b">
         <v>1</v>
@@ -19876,7 +19774,7 @@
         <v>0</v>
       </c>
       <c r="AA97" s="5" t="n">
-        <v>25.50345656747821</v>
+        <v>7.168620378719567</v>
       </c>
       <c r="AB97" s="5" t="n">
         <v>0</v>
@@ -19908,14 +19806,14 @@
       </c>
       <c r="AJ97" s="18" t="inlineStr">
         <is>
-          <t>[31, 32, 23, 13, 1, 12, 31]</t>
+          <t>[31, 1, 23, 17, 34, 16, 12, 31]</t>
         </is>
       </c>
       <c r="AK97" s="19" t="n">
-        <v>4957</v>
+        <v>6055</v>
       </c>
       <c r="AL97" s="20" t="n">
-        <v>74.09062907991833</v>
+        <v>70.30796949750116</v>
       </c>
       <c r="AM97" s="18" t="b">
         <v>1</v>
@@ -19966,7 +19864,7 @@
         <v>0</v>
       </c>
       <c r="BA97" s="5" t="n">
-        <v>25.50345656747821</v>
+        <v>9.002103997595432</v>
       </c>
       <c r="BB97" s="5" t="n">
         <v>18.04929365795011</v>
@@ -20009,14 +19907,14 @@
       </c>
       <c r="I98" s="15" t="inlineStr">
         <is>
-          <t>[31, 32, 23, 11, 1, 12, 31]</t>
+          <t>[31, 23, 32, 16, 12, 34, 31]</t>
         </is>
       </c>
       <c r="J98" s="16" t="n">
-        <v>4618</v>
+        <v>5179</v>
       </c>
       <c r="K98" s="17" t="n">
-        <v>74.80886715147479</v>
+        <v>75.10551564821257</v>
       </c>
       <c r="L98" s="15" t="b">
         <v>1</v>
@@ -20072,7 +19970,7 @@
         <v>0</v>
       </c>
       <c r="AA98" s="5" t="n">
-        <v>22.58172673931266</v>
+        <v>13.17686504610226</v>
       </c>
       <c r="AB98" s="5" t="n">
         <v>0.03352891869237217</v>
@@ -20104,14 +20002,14 @@
       </c>
       <c r="AJ98" s="18" t="inlineStr">
         <is>
-          <t>[31, 32, 23, 1, 17, 34, 12, 31]</t>
+          <t>[31, 34, 16, 12, 1, 23, 17, 31]</t>
         </is>
       </c>
       <c r="AK98" s="19" t="n">
-        <v>5341</v>
+        <v>5965</v>
       </c>
       <c r="AL98" s="20" t="n">
-        <v>74.27718948263991</v>
+        <v>76.58623801160354</v>
       </c>
       <c r="AM98" s="18" t="b">
         <v>1</v>
@@ -20162,7 +20060,7 @@
         <v>0</v>
       </c>
       <c r="BA98" s="5" t="n">
-        <v>10.46102263202012</v>
+        <v>0</v>
       </c>
       <c r="BB98" s="5" t="n">
         <v>13.17686504610226</v>
@@ -20205,14 +20103,14 @@
       </c>
       <c r="I99" s="15" t="inlineStr">
         <is>
-          <t>[31, 32, 23, 1, 12, 16, 31]</t>
+          <t>[31, 23, 1, 12, 34, 16, 31]</t>
         </is>
       </c>
       <c r="J99" s="16" t="n">
-        <v>5758</v>
+        <v>5712</v>
       </c>
       <c r="K99" s="17" t="n">
-        <v>75.34279720288458</v>
+        <v>69.64229689432317</v>
       </c>
       <c r="L99" s="15" t="b">
         <v>1</v>
@@ -20268,7 +20166,7 @@
         <v>0</v>
       </c>
       <c r="AA99" s="5" t="n">
-        <v>4.999175053621514</v>
+        <v>5.758125721828081</v>
       </c>
       <c r="AB99" s="5" t="n">
         <v>0</v>
@@ -20300,14 +20198,14 @@
       </c>
       <c r="AJ99" s="18" t="inlineStr">
         <is>
-          <t>[31, 32, 23, 1, 12, 16, 31]</t>
+          <t>[31, 23, 1, 12, 34, 16, 31]</t>
         </is>
       </c>
       <c r="AK99" s="19" t="n">
-        <v>5758</v>
+        <v>5712</v>
       </c>
       <c r="AL99" s="20" t="n">
-        <v>75.34279720288458</v>
+        <v>69.64229689432317</v>
       </c>
       <c r="AM99" s="18" t="b">
         <v>1</v>
@@ -20358,7 +20256,7 @@
         <v>0</v>
       </c>
       <c r="BA99" s="5" t="n">
-        <v>4.999175053621514</v>
+        <v>5.758125721828081</v>
       </c>
       <c r="BB99" s="5" t="n">
         <v>23.13149645273057</v>
@@ -20401,14 +20299,14 @@
       </c>
       <c r="I100" s="15" t="inlineStr">
         <is>
-          <t>[32, 23, 6, 24, 28, 32]</t>
+          <t>[32, 16, 34, 31, 12, 17, 1, 32]</t>
         </is>
       </c>
       <c r="J100" s="16" t="n">
-        <v>4596</v>
+        <v>5403</v>
       </c>
       <c r="K100" s="17" t="n">
-        <v>76.84161636436706</v>
+        <v>72.5721514654558</v>
       </c>
       <c r="L100" s="15" t="b">
         <v>1</v>
@@ -20464,7 +20362,7 @@
         <v>0</v>
       </c>
       <c r="AA100" s="5" t="n">
-        <v>23.47652347652348</v>
+        <v>10.03996003996004</v>
       </c>
       <c r="AB100" s="5" t="n">
         <v>5.328005328005328</v>
@@ -20496,14 +20394,14 @@
       </c>
       <c r="AJ100" s="18" t="inlineStr">
         <is>
-          <t>[32, 23, 6, 24, 28, 32]</t>
+          <t>[32, 16, 12, 34, 31, 1, 23, 32]</t>
         </is>
       </c>
       <c r="AK100" s="19" t="n">
-        <v>4596</v>
+        <v>5853</v>
       </c>
       <c r="AL100" s="20" t="n">
-        <v>76.84161636436706</v>
+        <v>75.01421864387075</v>
       </c>
       <c r="AM100" s="18" t="b">
         <v>1</v>
@@ -20554,7 +20452,7 @@
         <v>0</v>
       </c>
       <c r="BA100" s="5" t="n">
-        <v>23.47652347652348</v>
+        <v>2.547452547452548</v>
       </c>
       <c r="BB100" s="5" t="n">
         <v>19.3972693972694</v>
@@ -20597,14 +20495,14 @@
       </c>
       <c r="I101" s="15" t="inlineStr">
         <is>
-          <t>[32, 23, 11, 0, 30, 32]</t>
+          <t>[32, 23, 16, 34, 12, 32]</t>
         </is>
       </c>
       <c r="J101" s="16" t="n">
-        <v>4304</v>
+        <v>4998</v>
       </c>
       <c r="K101" s="17" t="n">
-        <v>69.90498947637992</v>
+        <v>73.86462458468102</v>
       </c>
       <c r="L101" s="15" t="b">
         <v>1</v>
@@ -20660,7 +20558,7 @@
         <v>0</v>
       </c>
       <c r="AA101" s="5" t="n">
-        <v>22.79820627802691</v>
+        <v>10.34977578475336</v>
       </c>
       <c r="AB101" s="5" t="n">
         <v>1.991031390134529</v>
@@ -20692,14 +20590,14 @@
       </c>
       <c r="AJ101" s="18" t="inlineStr">
         <is>
-          <t>[32, 23, 11, 30, 15, 32]</t>
+          <t>[32, 16, 31, 34, 12, 1, 23, 32]</t>
         </is>
       </c>
       <c r="AK101" s="19" t="n">
-        <v>4347</v>
+        <v>5534</v>
       </c>
       <c r="AL101" s="20" t="n">
-        <v>76.95309526898431</v>
+        <v>74.78458120165985</v>
       </c>
       <c r="AM101" s="18" t="b">
         <v>1</v>
@@ -20750,7 +20648,7 @@
         <v>0</v>
       </c>
       <c r="BA101" s="5" t="n">
-        <v>22.02690582959641</v>
+        <v>0.7354260089686099</v>
       </c>
       <c r="BB101" s="5" t="n">
         <v>4.089686098654709</v>
@@ -20793,14 +20691,14 @@
       </c>
       <c r="I102" s="15" t="inlineStr">
         <is>
-          <t>[32, 28, 27, 0, 30, 32]</t>
+          <t>[32, 23, 13, 1, 12, 34, 32]</t>
         </is>
       </c>
       <c r="J102" s="16" t="n">
-        <v>4717</v>
+        <v>5069</v>
       </c>
       <c r="K102" s="17" t="n">
-        <v>73.10104639937089</v>
+        <v>75.76383326003132</v>
       </c>
       <c r="L102" s="15" t="b">
         <v>1</v>
@@ -20856,7 +20754,7 @@
         <v>0</v>
       </c>
       <c r="AA102" s="5" t="n">
-        <v>22.50698209298505</v>
+        <v>16.72416625595531</v>
       </c>
       <c r="AB102" s="5" t="n">
         <v>3.400689995071464</v>
@@ -20888,14 +20786,14 @@
       </c>
       <c r="AJ102" s="18" t="inlineStr">
         <is>
-          <t>[32, 28, 27, 0, 30, 32]</t>
+          <t>[32, 16, 12, 34, 31, 1, 23, 32]</t>
         </is>
       </c>
       <c r="AK102" s="19" t="n">
-        <v>4717</v>
+        <v>6087</v>
       </c>
       <c r="AL102" s="20" t="n">
-        <v>73.10104639937089</v>
+        <v>75.01421864387075</v>
       </c>
       <c r="AM102" s="18" t="b">
         <v>1</v>
@@ -20946,7 +20844,7 @@
         <v>0</v>
       </c>
       <c r="BA102" s="5" t="n">
-        <v>22.50698209298505</v>
+        <v>0</v>
       </c>
       <c r="BB102" s="5" t="n">
         <v>2.365697387875801</v>
@@ -21577,14 +21475,14 @@
       </c>
       <c r="I106" s="15" t="inlineStr">
         <is>
-          <t>[34, 32, 15, 28, 1, 34]</t>
+          <t>[34, 32, 23, 1, 16, 12, 34]</t>
         </is>
       </c>
       <c r="J106" s="16" t="n">
-        <v>4188</v>
+        <v>5192</v>
       </c>
       <c r="K106" s="17" t="n">
-        <v>76.31065503872455</v>
+        <v>74.0692681981388</v>
       </c>
       <c r="L106" s="15" t="b">
         <v>1</v>
@@ -21640,7 +21538,7 @@
         <v>0</v>
       </c>
       <c r="AA106" s="5" t="n">
-        <v>32.15616393973757</v>
+        <v>15.89178681354285</v>
       </c>
       <c r="AB106" s="5" t="n">
         <v>1.052972622711809</v>
@@ -21672,14 +21570,14 @@
       </c>
       <c r="AJ106" s="18" t="inlineStr">
         <is>
-          <t>[34, 32, 23, 1, 16, 12, 34]</t>
+          <t>[34, 17, 23, 1, 32, 16, 31, 34]</t>
         </is>
       </c>
       <c r="AK106" s="19" t="n">
-        <v>5192</v>
+        <v>6173</v>
       </c>
       <c r="AL106" s="20" t="n">
-        <v>74.0692681981388</v>
+        <v>76.40202087081711</v>
       </c>
       <c r="AM106" s="18" t="b">
         <v>1</v>
@@ -21730,7 +21628,7 @@
         <v>0</v>
       </c>
       <c r="BA106" s="5" t="n">
-        <v>15.89178681354285</v>
+        <v>0</v>
       </c>
       <c r="BB106" s="5" t="n">
         <v>30.37421027053296</v>
@@ -21773,14 +21671,14 @@
       </c>
       <c r="I107" s="15" t="inlineStr">
         <is>
-          <t>[34, 16, 11, 23, 17, 34]</t>
+          <t>[34, 23, 11, 13, 1, 12, 31, 34]</t>
         </is>
       </c>
       <c r="J107" s="16" t="n">
-        <v>4647</v>
+        <v>5505</v>
       </c>
       <c r="K107" s="17" t="n">
-        <v>75.80977144016293</v>
+        <v>74.42838266767468</v>
       </c>
       <c r="L107" s="15" t="b">
         <v>1</v>
@@ -21836,7 +21734,7 @@
         <v>0</v>
       </c>
       <c r="AA107" s="5" t="n">
-        <v>18.11453744493392</v>
+        <v>2.995594713656387</v>
       </c>
       <c r="AB107" s="5" t="n">
         <v>0.2819383259911895</v>
@@ -21868,14 +21766,14 @@
       </c>
       <c r="AJ107" s="18" t="inlineStr">
         <is>
-          <t>[34, 32, 23, 11, 13, 34]</t>
+          <t>[34, 23, 11, 13, 1, 12, 31, 34]</t>
         </is>
       </c>
       <c r="AK107" s="19" t="n">
-        <v>4860</v>
+        <v>5505</v>
       </c>
       <c r="AL107" s="20" t="n">
-        <v>75.73655029602078</v>
+        <v>74.42838266767468</v>
       </c>
       <c r="AM107" s="18" t="b">
         <v>1</v>
@@ -21926,7 +21824,7 @@
         <v>0</v>
       </c>
       <c r="BA107" s="5" t="n">
-        <v>14.36123348017621</v>
+        <v>2.995594713656387</v>
       </c>
       <c r="BB107" s="5" t="n">
         <v>11.9647577092511</v>
@@ -21969,14 +21867,14 @@
       </c>
       <c r="I108" s="15" t="inlineStr">
         <is>
-          <t>[34, 23, 32, 16, 31, 12, 34]</t>
+          <t>[34, 16, 11, 23, 17, 34]</t>
         </is>
       </c>
       <c r="J108" s="16" t="n">
-        <v>5489</v>
+        <v>5028</v>
       </c>
       <c r="K108" s="17" t="n">
-        <v>71.19715699148207</v>
+        <v>75.80977144016293</v>
       </c>
       <c r="L108" s="15" t="b">
         <v>1</v>
@@ -22032,7 +21930,7 @@
         <v>0</v>
       </c>
       <c r="AA108" s="5" t="n">
-        <v>9.942575881870386</v>
+        <v>17.50615258408532</v>
       </c>
       <c r="AB108" s="5" t="n">
         <v>0</v>
@@ -22064,14 +21962,14 @@
       </c>
       <c r="AJ108" s="18" t="inlineStr">
         <is>
-          <t>[34, 16, 11, 23, 17, 34]</t>
+          <t>[34, 31, 16, 12, 32, 1, 17, 34]</t>
         </is>
       </c>
       <c r="AK108" s="19" t="n">
-        <v>5028</v>
+        <v>5445</v>
       </c>
       <c r="AL108" s="20" t="n">
-        <v>75.80977144016293</v>
+        <v>74.5329364759455</v>
       </c>
       <c r="AM108" s="18" t="b">
         <v>1</v>
@@ -22122,7 +22020,7 @@
         <v>0</v>
       </c>
       <c r="BA108" s="5" t="n">
-        <v>17.50615258408532</v>
+        <v>10.66447908121411</v>
       </c>
       <c r="BB108" s="5" t="n">
         <v>9.942575881870386</v>
@@ -22229,25 +22127,25 @@
         <v>105</v>
       </c>
       <c r="D2" t="n">
-        <v>4001.780952380952</v>
+        <v>4408.571428571428</v>
       </c>
       <c r="E2" t="n">
-        <v>1269.581449662056</v>
+        <v>1439.446560695777</v>
       </c>
       <c r="F2" t="n">
-        <v>3146</v>
+        <v>3287</v>
       </c>
       <c r="G2" t="n">
-        <v>4331</v>
+        <v>4946</v>
       </c>
       <c r="H2" t="n">
-        <v>4915</v>
+        <v>5406</v>
       </c>
       <c r="I2" t="n">
         <v>555</v>
       </c>
       <c r="J2" t="n">
-        <v>6402</v>
+        <v>6563</v>
       </c>
     </row>
     <row r="3">
@@ -22418,19 +22316,19 @@
         <v>105</v>
       </c>
       <c r="C2" t="n">
-        <v>1248.685714285714</v>
+        <v>1655.47619047619</v>
       </c>
       <c r="D2" t="n">
-        <v>1113</v>
+        <v>1540</v>
       </c>
       <c r="E2" t="n">
-        <v>1125.963419223099</v>
+        <v>1055.819970224001</v>
       </c>
       <c r="F2" t="n">
-        <v>91.5</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>2.001847981512037e-16</v>
+        <v>8.330397473485909e-18</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -22446,19 +22344,19 @@
         <v>105</v>
       </c>
       <c r="C3" t="n">
-        <v>-120.9333333333333</v>
+        <v>285.8571428571428</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>559.5057789394732</v>
+        <v>519.0248517203166</v>
       </c>
       <c r="F3" t="n">
-        <v>883.5</v>
+        <v>347</v>
       </c>
       <c r="G3" t="n">
-        <v>0.01024736895989458</v>
+        <v>2.676543543477171e-07</v>
       </c>
       <c r="H3" t="b">
         <v>1</v>
@@ -22474,19 +22372,19 @@
         <v>105</v>
       </c>
       <c r="C4" t="n">
-        <v>-83.93333333333334</v>
+        <v>322.8571428571428</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>677.9303099347344</v>
+        <v>614.2533840201613</v>
       </c>
       <c r="F4" t="n">
-        <v>866</v>
+        <v>349</v>
       </c>
       <c r="G4" t="n">
-        <v>0.003158797213910822</v>
+        <v>1.020354055672476e-07</v>
       </c>
       <c r="H4" t="b">
         <v>1</v>
@@ -22495,416 +22393,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Q14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="24" customWidth="1" min="17" max="17"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="24" t="inlineStr">
-        <is>
-          <t>CHEQUEO DE CONVERGENCIA PPO  ·  35 nodos</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="24" t="inlineStr">
-        <is>
-          <t>CRITERIOS DE CONVERGENCIA  (evaluados sobre las últimas W = 50 PPO updates)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="25" t="inlineStr">
-        <is>
-          <t>Condición</t>
-        </is>
-      </c>
-      <c r="B4" s="25" t="inlineStr">
-        <is>
-          <t>Métrica observada</t>
-        </is>
-      </c>
-      <c r="C4" s="25" t="inlineStr">
-        <is>
-          <t>Cómo se mide</t>
-        </is>
-      </c>
-      <c r="D4" s="25" t="inlineStr">
-        <is>
-          <t>Umbral de aprobación</t>
-        </is>
-      </c>
-      <c r="E4" s="25" t="inlineStr">
-        <is>
-          <t>Nota de diseño</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>C1 — Reward aplanado</t>
-        </is>
-      </c>
-      <c r="B5" s="27" t="inlineStr">
-        <is>
-          <t>Pendiente relativa del reward de entrenamiento</t>
-        </is>
-      </c>
-      <c r="C5" s="27" t="inlineStr">
-        <is>
-          <t>Regresión lineal sobre la ventana → slope / |media reward|</t>
-        </is>
-      </c>
-      <c r="D5" s="27" t="inlineStr">
-        <is>
-          <t>&lt; 0.001  (adimensional)</t>
-        </is>
-      </c>
-      <c r="E5" s="27" t="inlineStr">
-        <is>
-          <t>Valor relativo para que sea comparable entre escalas de reward distintas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="26" t="inlineStr">
-        <is>
-          <t>C2 — Explained Variance estable</t>
-        </is>
-      </c>
-      <c r="B6" s="27" t="inlineStr">
-        <is>
-          <t>Media y pendiente relativa de explained_var del crítico</t>
-        </is>
-      </c>
-      <c r="C6" s="27" t="inlineStr">
-        <is>
-          <t>Media aritmética + regresión lineal sobre la ventana</t>
-        </is>
-      </c>
-      <c r="D6" s="27" t="inlineStr">
-        <is>
-          <t>Media ≥ 0.5  Y  |pendiente rel.| &lt; 0.001</t>
-        </is>
-      </c>
-      <c r="E6" s="27" t="inlineStr">
-        <is>
-          <t>Umbral 0.5 coincide con la línea de referencia en PPO_Diagnostics_AM.png.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="26" t="inlineStr">
-        <is>
-          <t>C3 — KL divergence controlada</t>
-        </is>
-      </c>
-      <c r="B7" s="27" t="inlineStr">
-        <is>
-          <t>Fracción de updates en ventana con KL &gt; umbral KL</t>
-        </is>
-      </c>
-      <c r="C7" s="27" t="inlineStr">
-        <is>
-          <t>Proporción de filas donde kl_divergence &gt; kl_threshold</t>
-        </is>
-      </c>
-      <c r="D7" s="27" t="inlineStr">
-        <is>
-          <t>Fracción de violaciones ≤ 5%  (umbral KL = 0.02)</t>
-        </is>
-      </c>
-      <c r="E7" s="27" t="inlineStr">
-        <is>
-          <t>Umbral KL 0.02 coincide con la línea de referencia en PPO_Diagnostics_AM.png.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="26" t="inlineStr">
-        <is>
-          <t>C4 — Entropía estabilizada</t>
-        </is>
-      </c>
-      <c r="B8" s="27" t="inlineStr">
-        <is>
-          <t>Pendiente ABSOLUTA de la entropía de la política</t>
-        </is>
-      </c>
-      <c r="C8" s="27" t="inlineStr">
-        <is>
-          <t>Regresión lineal sobre la ventana → |slope| en nats/update</t>
-        </is>
-      </c>
-      <c r="D8" s="27" t="inlineStr">
-        <is>
-          <t>&lt; 0.0005  nats/update</t>
-        </is>
-      </c>
-      <c r="E8" s="27" t="inlineStr">
-        <is>
-          <t>Se usa pendiente absoluta (no relativa) porque la entropía puede pasar por 0.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="40" customHeight="1"/>
-    <row r="10" ht="40" customHeight="1"/>
-    <row r="11">
-      <c r="A11" s="24" t="inlineStr">
-        <is>
-          <t>RESULTADOS DEL CHEQUEO</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="28" t="inlineStr">
-        <is>
-          <t>Identificación</t>
-        </is>
-      </c>
-      <c r="B12" s="29" t="n"/>
-      <c r="C12" s="29" t="n"/>
-      <c r="D12" s="1" t="inlineStr">
-        <is>
-          <t>C1 — Reward Aplanado</t>
-        </is>
-      </c>
-      <c r="E12" s="30" t="n"/>
-      <c r="F12" s="30" t="n"/>
-      <c r="G12" s="7" t="inlineStr">
-        <is>
-          <t>C2 — Explained Variance</t>
-        </is>
-      </c>
-      <c r="H12" s="31" t="n"/>
-      <c r="I12" s="31" t="n"/>
-      <c r="J12" s="31" t="n"/>
-      <c r="K12" s="9" t="inlineStr">
-        <is>
-          <t>C3 — KL Divergence</t>
-        </is>
-      </c>
-      <c r="L12" s="32" t="n"/>
-      <c r="M12" s="32" t="n"/>
-      <c r="N12" s="33" t="inlineStr">
-        <is>
-          <t>C4 — Entropía</t>
-        </is>
-      </c>
-      <c r="O12" s="34" t="n"/>
-      <c r="P12" s="34" t="n"/>
-      <c r="Q12" s="35" t="inlineStr">
-        <is>
-          <t>Veredicto Final</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="28" t="inlineStr">
-        <is>
-          <t>Nodos</t>
-        </is>
-      </c>
-      <c r="B13" s="28" t="inlineStr">
-        <is>
-          <t>Total
-Updates</t>
-        </is>
-      </c>
-      <c r="C13" s="28" t="inlineStr">
-        <is>
-          <t>Ventana
-(W usado)</t>
-        </is>
-      </c>
-      <c r="D13" s="1" t="inlineStr">
-        <is>
-          <t>Pendiente
-Reward Rel.
-(medido)</t>
-        </is>
-      </c>
-      <c r="E13" s="1" t="inlineStr">
-        <is>
-          <t>Umbral
-(&lt; 0.001)</t>
-        </is>
-      </c>
-      <c r="F13" s="1" t="inlineStr">
-        <is>
-          <t>C1
-Resultado</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>EV Media
-(medido)</t>
-        </is>
-      </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>EV Pendiente
-Rel. (medido)</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="inlineStr">
-        <is>
-          <t>Umbral
-Media ≥ 0.5</t>
-        </is>
-      </c>
-      <c r="J13" s="7" t="inlineStr">
-        <is>
-          <t>C2
-Resultado</t>
-        </is>
-      </c>
-      <c r="K13" s="9" t="inlineStr">
-        <is>
-          <t>Fracc.
-Violaciones
-KL (medido)</t>
-        </is>
-      </c>
-      <c r="L13" s="9" t="inlineStr">
-        <is>
-          <t>Umbral
-(≤ 5%)</t>
-        </is>
-      </c>
-      <c r="M13" s="9" t="inlineStr">
-        <is>
-          <t>C3
-Resultado</t>
-        </is>
-      </c>
-      <c r="N13" s="33" t="inlineStr">
-        <is>
-          <t>Pendiente
-Entropía Abs.
-(medido)</t>
-        </is>
-      </c>
-      <c r="O13" s="33" t="inlineStr">
-        <is>
-          <t>Umbral
-(&lt; 0.0005)</t>
-        </is>
-      </c>
-      <c r="P13" s="33" t="inlineStr">
-        <is>
-          <t>C4
-Resultado</t>
-        </is>
-      </c>
-      <c r="Q13" s="35" t="inlineStr">
-        <is>
-          <t>CONVERGIDO</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="36" t="n">
-        <v>35</v>
-      </c>
-      <c r="B14" s="37" t="n">
-        <v>500</v>
-      </c>
-      <c r="C14" s="37" t="n">
-        <v>50</v>
-      </c>
-      <c r="D14" s="38" t="n">
-        <v>8.1e-05</v>
-      </c>
-      <c r="E14" s="39" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="F14" s="40" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G14" s="41" t="n">
-        <v>0.8205</v>
-      </c>
-      <c r="H14" s="38" t="n">
-        <v>0.000125</v>
-      </c>
-      <c r="I14" s="42" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J14" s="40" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K14" s="41" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="42" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="M14" s="40" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="N14" s="38" t="n">
-        <v>0.000212</v>
-      </c>
-      <c r="O14" s="39" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="P14" s="40" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="Q14" s="43" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="K12:M12"/>
-    <mergeCell ref="G12:J12"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A11:Q11"/>
-    <mergeCell ref="N12:P12"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Resultados con 35 nodos, gap est 2.9 y det 7.4
</commit_message>
<xml_diff>
--- a/results_35nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_35nodes/DRL_Routing_Summary_AM.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Per Node Results" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Stochastic Descriptive Stats" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Wilcoxon Significance" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="PPO Convergence" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,10 +20,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.00&quot;%&quot;"/>
+    <numFmt numFmtId="165" formatCode="0.000000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,8 +46,32 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00548235"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -89,6 +116,41 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C55A11"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00595959"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00404040"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00833C00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE0E0"/>
       </patternFill>
     </fill>
   </fills>
@@ -138,7 +200,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -202,6 +264,59 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -622,7 +737,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>32.4363594963437</v>
+        <v>35.26441483270555</v>
       </c>
     </row>
     <row r="4">
@@ -632,13 +747,13 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>4183.628571428571</v>
+        <v>4202.838095238095</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>7.699473677278425</v>
+        <v>7.366119880473141</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>559.4056061335972</v>
+        <v>566.8754305158342</v>
       </c>
     </row>
     <row r="5">
@@ -654,7 +769,7 @@
         <v>0.7830855557137725</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>12493.53005999611</v>
+        <v>13714.20839400519</v>
       </c>
     </row>
     <row r="6">
@@ -670,7 +785,7 @@
         <v>13.09578163496531</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>4.917651131039573</v>
+        <v>5.311296099708194</v>
       </c>
     </row>
     <row r="7">
@@ -686,7 +801,7 @@
         <v>52.95029311789443</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.4690283820742653</v>
+        <v>0.5005405062720889</v>
       </c>
     </row>
     <row r="9">
@@ -734,7 +849,7 @@
         <v>0</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>93.94339606875465</v>
+        <v>98.01252910069057</v>
       </c>
     </row>
     <row r="12">
@@ -744,13 +859,13 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>4408.571428571428</v>
+        <v>4417.114285714286</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>3.146613048719591</v>
+        <v>2.906151551462991</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>559.4056061335972</v>
+        <v>566.8754305158342</v>
       </c>
     </row>
     <row r="13">
@@ -766,7 +881,7 @@
         <v>11.87591998359568</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>13.07282447814941</v>
+        <v>13.8415881565639</v>
       </c>
     </row>
     <row r="14">
@@ -796,7 +911,7 @@
         <v>14.13950847586963</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>10.56132089524042</v>
+        <v>11.01879392351423</v>
       </c>
     </row>
     <row r="17">
@@ -826,7 +941,7 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>0</v>
+        <v>893.2330803871155</v>
       </c>
     </row>
     <row r="20">
@@ -836,7 +951,7 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>559.4056061335972</v>
+        <v>566.8754305158342</v>
       </c>
     </row>
     <row r="21">
@@ -846,7 +961,7 @@
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>12493.53005999611</v>
+        <v>13714.20839400519</v>
       </c>
     </row>
     <row r="22">
@@ -856,7 +971,7 @@
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>32.4363594963437</v>
+        <v>35.26441483270555</v>
       </c>
     </row>
     <row r="23">
@@ -866,7 +981,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>0.4690283820742653</v>
+        <v>0.5005405062720889</v>
       </c>
     </row>
     <row r="24">
@@ -876,7 +991,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>4.917651131039573</v>
+        <v>5.311296099708194</v>
       </c>
     </row>
     <row r="25">
@@ -886,7 +1001,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>13.07282447814941</v>
+        <v>13.8415881565639</v>
       </c>
     </row>
     <row r="26">
@@ -896,7 +1011,7 @@
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>10.56132089524042</v>
+        <v>11.01879392351423</v>
       </c>
     </row>
     <row r="27">
@@ -906,7 +1021,7 @@
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>93.94339606875465</v>
+        <v>98.01252910069057</v>
       </c>
     </row>
   </sheetData>
@@ -1483,14 +1598,14 @@
       </c>
       <c r="I4" s="15" t="inlineStr">
         <is>
-          <t>[0, 32, 23, 13, 30, 0]</t>
+          <t>[0, 27, 30, 15, 28, 6, 0]</t>
         </is>
       </c>
       <c r="J4" s="16" t="n">
-        <v>4586</v>
+        <v>4378</v>
       </c>
       <c r="K4" s="17" t="n">
-        <v>76.99346174245754</v>
+        <v>74.87284755753305</v>
       </c>
       <c r="L4" s="15" t="b">
         <v>1</v>
@@ -1546,7 +1661,7 @@
         <v>0</v>
       </c>
       <c r="AA4" s="5" t="n">
-        <v>8.845160007950707</v>
+        <v>12.97952693301531</v>
       </c>
       <c r="AB4" s="5" t="n">
         <v>0</v>
@@ -1679,14 +1794,14 @@
       </c>
       <c r="I5" s="15" t="inlineStr">
         <is>
-          <t>[0, 32, 23, 11, 28, 15, 30, 0]</t>
+          <t>[0, 32, 28, 30, 27, 0]</t>
         </is>
       </c>
       <c r="J5" s="16" t="n">
-        <v>4915</v>
+        <v>4731</v>
       </c>
       <c r="K5" s="17" t="n">
-        <v>72.3529809644612</v>
+        <v>71.2255389720694</v>
       </c>
       <c r="L5" s="15" t="b">
         <v>1</v>
@@ -1742,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="AA5" s="5" t="n">
-        <v>11.37756941940137</v>
+        <v>14.69527587450415</v>
       </c>
       <c r="AB5" s="5" t="n">
         <v>0</v>
@@ -1774,14 +1889,14 @@
       </c>
       <c r="AJ5" s="18" t="inlineStr">
         <is>
-          <t>[0, 32, 23, 1, 15, 30, 0]</t>
+          <t>[0, 26, 27, 15, 32, 30, 0]</t>
         </is>
       </c>
       <c r="AK5" s="19" t="n">
-        <v>4840</v>
+        <v>4807</v>
       </c>
       <c r="AL5" s="20" t="n">
-        <v>76.40911280206747</v>
+        <v>75.53606396780619</v>
       </c>
       <c r="AM5" s="18" t="b">
         <v>1</v>
@@ -1832,7 +1947,7 @@
         <v>0</v>
       </c>
       <c r="BA5" s="5" t="n">
-        <v>12.72989542012261</v>
+        <v>13.32491886043996</v>
       </c>
       <c r="BB5" s="5" t="n">
         <v>9.087630724846736</v>
@@ -2166,14 +2281,14 @@
       </c>
       <c r="AJ7" s="18" t="inlineStr">
         <is>
-          <t>[1, 23, 11, 28, 15, 0, 30, 32, 1]</t>
+          <t>[1, 17, 23, 11, 28, 15, 1]</t>
         </is>
       </c>
       <c r="AK7" s="19" t="n">
-        <v>4996</v>
+        <v>5074</v>
       </c>
       <c r="AL7" s="20" t="n">
-        <v>75.96593670627344</v>
+        <v>74.01125865514462</v>
       </c>
       <c r="AM7" s="18" t="b">
         <v>1</v>
@@ -2224,7 +2339,7 @@
         <v>0</v>
       </c>
       <c r="BA7" s="5" t="n">
-        <v>17.92344340397569</v>
+        <v>16.64202398554296</v>
       </c>
       <c r="BB7" s="5" t="n">
         <v>27.40266140956136</v>
@@ -2855,14 +2970,14 @@
       </c>
       <c r="I11" s="15" t="inlineStr">
         <is>
-          <t>[2, 23, 11, 13, 8, 18, 2]</t>
+          <t>[2, 13, 23, 11, 8, 18, 2]</t>
         </is>
       </c>
       <c r="J11" s="16" t="n">
-        <v>4965</v>
+        <v>5209</v>
       </c>
       <c r="K11" s="17" t="n">
-        <v>74.84235419102524</v>
+        <v>76.11688487342525</v>
       </c>
       <c r="L11" s="15" t="b">
         <v>1</v>
@@ -2918,7 +3033,7 @@
         <v>0</v>
       </c>
       <c r="AA11" s="5" t="n">
-        <v>4.684200422345939</v>
+        <v>0</v>
       </c>
       <c r="AB11" s="5" t="n">
         <v>0</v>
@@ -3639,14 +3754,14 @@
       </c>
       <c r="I15" s="15" t="inlineStr">
         <is>
-          <t>[3, 33, 4, 10, 3]</t>
+          <t>[3, 4, 14, 33, 3]</t>
         </is>
       </c>
       <c r="J15" s="16" t="n">
-        <v>1972</v>
+        <v>2105</v>
       </c>
       <c r="K15" s="17" t="n">
-        <v>72.20133315988178</v>
+        <v>76.12162017812862</v>
       </c>
       <c r="L15" s="15" t="b">
         <v>1</v>
@@ -3702,7 +3817,7 @@
         <v>0</v>
       </c>
       <c r="AA15" s="5" t="n">
-        <v>13.43283582089552</v>
+        <v>7.594381035996488</v>
       </c>
       <c r="AB15" s="5" t="n">
         <v>0</v>
@@ -3930,14 +4045,14 @@
       </c>
       <c r="AJ16" s="18" t="inlineStr">
         <is>
-          <t>[4, 33, 3, 14, 4]</t>
+          <t>[4, 14, 33, 3, 4]</t>
         </is>
       </c>
       <c r="AK16" s="19" t="n">
-        <v>2013</v>
+        <v>2386</v>
       </c>
       <c r="AL16" s="20" t="n">
-        <v>66.1231493674095</v>
+        <v>76.12162017812862</v>
       </c>
       <c r="AM16" s="18" t="b">
         <v>1</v>
@@ -3988,7 +4103,7 @@
         <v>0</v>
       </c>
       <c r="BA16" s="5" t="n">
-        <v>15.63285834031853</v>
+        <v>0</v>
       </c>
       <c r="BB16" s="5" t="n">
         <v>0</v>
@@ -4227,14 +4342,14 @@
       </c>
       <c r="I18" s="15" t="inlineStr">
         <is>
-          <t>[4, 3, 33, 10, 4]</t>
+          <t>[4, 14, 33, 3, 4]</t>
         </is>
       </c>
       <c r="J18" s="16" t="n">
-        <v>2518</v>
+        <v>2408</v>
       </c>
       <c r="K18" s="17" t="n">
-        <v>69.72629704336707</v>
+        <v>76.12162017812862</v>
       </c>
       <c r="L18" s="15" t="b">
         <v>1</v>
@@ -4290,7 +4405,7 @@
         <v>0</v>
       </c>
       <c r="AA18" s="5" t="n">
-        <v>0</v>
+        <v>4.368546465448769</v>
       </c>
       <c r="AB18" s="5" t="n">
         <v>0</v>
@@ -5106,14 +5221,14 @@
       </c>
       <c r="AJ22" s="18" t="inlineStr">
         <is>
-          <t>[6, 32, 23, 11, 24, 6]</t>
+          <t>[6, 28, 32, 23, 11, 24, 6]</t>
         </is>
       </c>
       <c r="AK22" s="19" t="n">
-        <v>5248</v>
+        <v>5126</v>
       </c>
       <c r="AL22" s="20" t="n">
-        <v>68.63913955482947</v>
+        <v>72.19802163182189</v>
       </c>
       <c r="AM22" s="18" t="b">
         <v>1</v>
@@ -5164,7 +5279,7 @@
         <v>0</v>
       </c>
       <c r="BA22" s="5" t="n">
-        <v>4.023408924652524</v>
+        <v>6.254572055596196</v>
       </c>
       <c r="BB22" s="5" t="n">
         <v>4.023408924652524</v>
@@ -5207,14 +5322,14 @@
       </c>
       <c r="I23" s="15" t="inlineStr">
         <is>
-          <t>[6, 15, 32, 28, 24, 6]</t>
+          <t>[6, 32, 15, 28, 24, 6]</t>
         </is>
       </c>
       <c r="J23" s="16" t="n">
-        <v>4321</v>
+        <v>4466</v>
       </c>
       <c r="K23" s="17" t="n">
-        <v>76.91467601944998</v>
+        <v>73.35659403721718</v>
       </c>
       <c r="L23" s="15" t="b">
         <v>1</v>
@@ -5270,7 +5385,7 @@
         <v>0</v>
       </c>
       <c r="AA23" s="5" t="n">
-        <v>26.06091718001369</v>
+        <v>23.57973990417522</v>
       </c>
       <c r="AB23" s="5" t="n">
         <v>0</v>
@@ -5302,14 +5417,14 @@
       </c>
       <c r="AJ23" s="18" t="inlineStr">
         <is>
-          <t>[6, 11, 13, 23, 1, 15, 28, 6]</t>
+          <t>[6, 11, 23, 1, 32, 30, 15, 28, 6]</t>
         </is>
       </c>
       <c r="AK23" s="19" t="n">
-        <v>5844</v>
+        <v>5393</v>
       </c>
       <c r="AL23" s="20" t="n">
-        <v>76.9634944961675</v>
+        <v>75.83384333344556</v>
       </c>
       <c r="AM23" s="18" t="b">
         <v>1</v>
@@ -5360,7 +5475,7 @@
         <v>0</v>
       </c>
       <c r="BA23" s="5" t="n">
-        <v>0</v>
+        <v>7.717316906228611</v>
       </c>
       <c r="BB23" s="5" t="n">
         <v>23.57973990417522</v>
@@ -5498,14 +5613,14 @@
       </c>
       <c r="AJ24" s="18" t="inlineStr">
         <is>
-          <t>[6, 28, 15, 32, 23, 24, 6]</t>
+          <t>[6, 15, 32, 23, 24, 6]</t>
         </is>
       </c>
       <c r="AK24" s="19" t="n">
-        <v>4700</v>
+        <v>4521</v>
       </c>
       <c r="AL24" s="20" t="n">
-        <v>76.94478559885567</v>
+        <v>76.91179015427582</v>
       </c>
       <c r="AM24" s="18" t="b">
         <v>1</v>
@@ -5556,7 +5671,7 @@
         <v>0</v>
       </c>
       <c r="BA24" s="5" t="n">
-        <v>8.435612702123514</v>
+        <v>11.92285213325541</v>
       </c>
       <c r="BB24" s="5" t="n">
         <v>14.88408338203779</v>
@@ -6086,14 +6201,14 @@
       </c>
       <c r="AJ27" s="18" t="inlineStr">
         <is>
-          <t>[7, 24, 11, 13, 23, 7]</t>
+          <t>[7, 24, 6, 11, 13, 7]</t>
         </is>
       </c>
       <c r="AK27" s="19" t="n">
-        <v>3386</v>
+        <v>3367</v>
       </c>
       <c r="AL27" s="20" t="n">
-        <v>75.70525438457454</v>
+        <v>70.93372623736701</v>
       </c>
       <c r="AM27" s="18" t="b">
         <v>1</v>
@@ -6144,7 +6259,7 @@
         <v>0</v>
       </c>
       <c r="BA27" s="5" t="n">
-        <v>5.339670114621191</v>
+        <v>5.870841487279844</v>
       </c>
       <c r="BB27" s="5" t="n">
         <v>10.34386357282639</v>
@@ -6187,14 +6302,14 @@
       </c>
       <c r="I28" s="15" t="inlineStr">
         <is>
-          <t>[8, 18, 2, 11, 13, 8]</t>
+          <t>[8, 18, 11, 23, 13, 8]</t>
         </is>
       </c>
       <c r="J28" s="16" t="n">
-        <v>4067</v>
+        <v>4539</v>
       </c>
       <c r="K28" s="17" t="n">
-        <v>71.86492405207225</v>
+        <v>75.35012256935434</v>
       </c>
       <c r="L28" s="15" t="b">
         <v>1</v>
@@ -6250,7 +6365,7 @@
         <v>0</v>
       </c>
       <c r="AA28" s="5" t="n">
-        <v>21.89360476281928</v>
+        <v>12.82888419435375</v>
       </c>
       <c r="AB28" s="5" t="n">
         <v>0</v>
@@ -6282,14 +6397,14 @@
       </c>
       <c r="AJ28" s="18" t="inlineStr">
         <is>
-          <t>[8, 18, 11, 23, 13, 8]</t>
+          <t>[8, 18, 2, 13, 23, 11, 8]</t>
         </is>
       </c>
       <c r="AK28" s="19" t="n">
-        <v>4539</v>
+        <v>5207</v>
       </c>
       <c r="AL28" s="20" t="n">
-        <v>75.35012256935434</v>
+        <v>76.11688487342524</v>
       </c>
       <c r="AM28" s="18" t="b">
         <v>1</v>
@@ -6340,7 +6455,7 @@
         <v>0</v>
       </c>
       <c r="BA28" s="5" t="n">
-        <v>12.82888419435375</v>
+        <v>0</v>
       </c>
       <c r="BB28" s="5" t="n">
         <v>12.82888419435375</v>
@@ -6478,14 +6593,14 @@
       </c>
       <c r="AJ29" s="18" t="inlineStr">
         <is>
-          <t>[8, 11, 23, 1, 12, 17, 8]</t>
+          <t>[8, 2, 13, 23, 1, 8]</t>
         </is>
       </c>
       <c r="AK29" s="19" t="n">
-        <v>4303</v>
+        <v>4007</v>
       </c>
       <c r="AL29" s="20" t="n">
-        <v>76.61506080163667</v>
+        <v>76.68615652701594</v>
       </c>
       <c r="AM29" s="18" t="b">
         <v>1</v>
@@ -6536,7 +6651,7 @@
         <v>0</v>
       </c>
       <c r="BA29" s="5" t="n">
-        <v>0</v>
+        <v>6.878921682547061</v>
       </c>
       <c r="BB29" s="5" t="n">
         <v>3.044387636532652</v>
@@ -8343,14 +8458,14 @@
       </c>
       <c r="I39" s="15" t="inlineStr">
         <is>
-          <t>[11, 13, 1, 15, 28, 6, 11]</t>
+          <t>[11, 23, 1, 15, 28, 6, 24, 11]</t>
         </is>
       </c>
       <c r="J39" s="16" t="n">
-        <v>4772</v>
+        <v>5393</v>
       </c>
       <c r="K39" s="17" t="n">
-        <v>76.229668609641</v>
+        <v>74.8418810837676</v>
       </c>
       <c r="L39" s="15" t="b">
         <v>1</v>
@@ -8406,7 +8521,7 @@
         <v>0</v>
       </c>
       <c r="AA39" s="5" t="n">
-        <v>18.32962519253808</v>
+        <v>7.70152319014205</v>
       </c>
       <c r="AB39" s="5" t="n">
         <v>6.161218552113641</v>
@@ -8539,14 +8654,14 @@
       </c>
       <c r="I40" s="15" t="inlineStr">
         <is>
-          <t>[12, 13, 17, 16, 34, 12]</t>
+          <t>[12, 17, 23, 32, 16, 34, 12]</t>
         </is>
       </c>
       <c r="J40" s="16" t="n">
-        <v>5449</v>
+        <v>5891</v>
       </c>
       <c r="K40" s="17" t="n">
-        <v>75.91279165923</v>
+        <v>75.5234513381658</v>
       </c>
       <c r="L40" s="15" t="b">
         <v>1</v>
@@ -8602,7 +8717,7 @@
         <v>0</v>
       </c>
       <c r="AA40" s="5" t="n">
-        <v>12.53611556982344</v>
+        <v>5.441412520064206</v>
       </c>
       <c r="AB40" s="5" t="n">
         <v>0.7383627608346709</v>
@@ -8634,14 +8749,14 @@
       </c>
       <c r="AJ40" s="18" t="inlineStr">
         <is>
-          <t>[12, 34, 16, 32, 23, 17, 12]</t>
+          <t>[12, 17, 23, 11, 13, 1, 34, 12]</t>
         </is>
       </c>
       <c r="AK40" s="19" t="n">
-        <v>5453</v>
+        <v>6184</v>
       </c>
       <c r="AL40" s="20" t="n">
-        <v>75.11649267211246</v>
+        <v>76.94862502908157</v>
       </c>
       <c r="AM40" s="18" t="b">
         <v>1</v>
@@ -8692,7 +8807,7 @@
         <v>0</v>
       </c>
       <c r="BA40" s="5" t="n">
-        <v>12.47191011235955</v>
+        <v>0.7383627608346709</v>
       </c>
       <c r="BB40" s="5" t="n">
         <v>9.390048154093098</v>
@@ -8735,14 +8850,14 @@
       </c>
       <c r="I41" s="15" t="inlineStr">
         <is>
-          <t>[12, 34, 16, 31, 17, 23, 1, 12]</t>
+          <t>[12, 34, 16, 31, 1, 23, 17, 12]</t>
         </is>
       </c>
       <c r="J41" s="16" t="n">
-        <v>5321</v>
+        <v>5502</v>
       </c>
       <c r="K41" s="17" t="n">
-        <v>76.7741215108931</v>
+        <v>76.09879587135731</v>
       </c>
       <c r="L41" s="15" t="b">
         <v>1</v>
@@ -8798,7 +8913,7 @@
         <v>0</v>
       </c>
       <c r="AA41" s="5" t="n">
-        <v>10.08786752281176</v>
+        <v>7.029401824940859</v>
       </c>
       <c r="AB41" s="5" t="n">
         <v>0</v>
@@ -8830,14 +8945,14 @@
       </c>
       <c r="AJ41" s="18" t="inlineStr">
         <is>
-          <t>[12, 34, 31, 16, 32, 23, 1, 12]</t>
+          <t>[12, 34, 16, 31, 17, 23, 1, 12]</t>
         </is>
       </c>
       <c r="AK41" s="19" t="n">
-        <v>5402</v>
+        <v>5321</v>
       </c>
       <c r="AL41" s="20" t="n">
-        <v>75.08232804674387</v>
+        <v>76.7741215108931</v>
       </c>
       <c r="AM41" s="18" t="b">
         <v>1</v>
@@ -8888,7 +9003,7 @@
         <v>0</v>
       </c>
       <c r="BA41" s="5" t="n">
-        <v>8.71916187901318</v>
+        <v>10.08786752281176</v>
       </c>
       <c r="BB41" s="5" t="n">
         <v>32.12233862791484</v>
@@ -8931,14 +9046,14 @@
       </c>
       <c r="I42" s="15" t="inlineStr">
         <is>
-          <t>[12, 17, 16, 34, 31, 1, 12]</t>
+          <t>[12, 34, 16, 31, 1, 23, 17, 12]</t>
         </is>
       </c>
       <c r="J42" s="16" t="n">
-        <v>4998</v>
+        <v>5371</v>
       </c>
       <c r="K42" s="17" t="n">
-        <v>71.55969324712517</v>
+        <v>76.09879587135731</v>
       </c>
       <c r="L42" s="15" t="b">
         <v>1</v>
@@ -8994,7 +9109,7 @@
         <v>0</v>
       </c>
       <c r="AA42" s="5" t="n">
-        <v>13.27433628318584</v>
+        <v>6.802012840534443</v>
       </c>
       <c r="AB42" s="5" t="n">
         <v>0</v>
@@ -9026,14 +9141,14 @@
       </c>
       <c r="AJ42" s="18" t="inlineStr">
         <is>
-          <t>[12, 31, 34, 16, 32, 23, 1, 12]</t>
+          <t>[12, 34, 16, 31, 1, 23, 17, 12]</t>
         </is>
       </c>
       <c r="AK42" s="19" t="n">
-        <v>5519</v>
+        <v>5371</v>
       </c>
       <c r="AL42" s="20" t="n">
-        <v>75.11269845882315</v>
+        <v>76.09879587135731</v>
       </c>
       <c r="AM42" s="18" t="b">
         <v>1</v>
@@ -9084,7 +9199,7 @@
         <v>0</v>
       </c>
       <c r="BA42" s="5" t="n">
-        <v>4.233905951761235</v>
+        <v>6.802012840534443</v>
       </c>
       <c r="BB42" s="5" t="n">
         <v>27.53774076002082</v>
@@ -9127,14 +9242,14 @@
       </c>
       <c r="I43" s="15" t="inlineStr">
         <is>
-          <t>[13, 1, 28, 11, 23, 13]</t>
+          <t>[13, 23, 32, 16, 12, 34, 13]</t>
         </is>
       </c>
       <c r="J43" s="16" t="n">
-        <v>4558</v>
+        <v>5378</v>
       </c>
       <c r="K43" s="17" t="n">
-        <v>72.75626993085845</v>
+        <v>76.53013715791758</v>
       </c>
       <c r="L43" s="15" t="b">
         <v>1</v>
@@ -9190,7 +9305,7 @@
         <v>0</v>
       </c>
       <c r="AA43" s="5" t="n">
-        <v>21.76450394782012</v>
+        <v>7.689667009955373</v>
       </c>
       <c r="AB43" s="5" t="n">
         <v>0</v>
@@ -9222,14 +9337,14 @@
       </c>
       <c r="AJ43" s="18" t="inlineStr">
         <is>
-          <t>[13, 23, 32, 16, 12, 34, 13]</t>
+          <t>[13, 1, 34, 31, 12, 23, 11, 13]</t>
         </is>
       </c>
       <c r="AK43" s="19" t="n">
-        <v>5378</v>
+        <v>5826</v>
       </c>
       <c r="AL43" s="20" t="n">
-        <v>76.53013715791758</v>
+        <v>76.56785031046195</v>
       </c>
       <c r="AM43" s="18" t="b">
         <v>1</v>
@@ -9280,7 +9395,7 @@
         <v>0</v>
       </c>
       <c r="BA43" s="5" t="n">
-        <v>7.689667009955373</v>
+        <v>0</v>
       </c>
       <c r="BB43" s="5" t="n">
         <v>24.01304497082046</v>
@@ -9323,14 +9438,14 @@
       </c>
       <c r="I44" s="15" t="inlineStr">
         <is>
-          <t>[13, 1, 16, 34, 12, 23, 13]</t>
+          <t>[13, 6, 24, 7, 13]</t>
         </is>
       </c>
       <c r="J44" s="16" t="n">
-        <v>5237</v>
+        <v>4227</v>
       </c>
       <c r="K44" s="17" t="n">
-        <v>76.5606625994937</v>
+        <v>70.66009204763162</v>
       </c>
       <c r="L44" s="15" t="b">
         <v>1</v>
@@ -9386,7 +9501,7 @@
         <v>0</v>
       </c>
       <c r="AA44" s="5" t="n">
-        <v>8.508036338225017</v>
+        <v>26.15303983228511</v>
       </c>
       <c r="AB44" s="5" t="n">
         <v>0.628930817610063</v>
@@ -9418,14 +9533,14 @@
       </c>
       <c r="AJ44" s="18" t="inlineStr">
         <is>
-          <t>[13, 1, 16, 34, 12, 23, 13]</t>
+          <t>[13, 17, 34, 31, 12, 1, 23, 11, 13]</t>
         </is>
       </c>
       <c r="AK44" s="19" t="n">
-        <v>5237</v>
+        <v>5688</v>
       </c>
       <c r="AL44" s="20" t="n">
-        <v>76.5606625994937</v>
+        <v>72.6154835462869</v>
       </c>
       <c r="AM44" s="18" t="b">
         <v>1</v>
@@ -9476,7 +9591,7 @@
         <v>0</v>
       </c>
       <c r="BA44" s="5" t="n">
-        <v>8.508036338225017</v>
+        <v>0.628930817610063</v>
       </c>
       <c r="BB44" s="5" t="n">
         <v>32.25017470300489</v>
@@ -9519,14 +9634,14 @@
       </c>
       <c r="I45" s="15" t="inlineStr">
         <is>
-          <t>[13, 1, 16, 31, 12, 34, 13]</t>
+          <t>[13, 6, 15, 28, 11, 23, 13]</t>
         </is>
       </c>
       <c r="J45" s="16" t="n">
-        <v>5038</v>
+        <v>4718</v>
       </c>
       <c r="K45" s="17" t="n">
-        <v>73.88913350076947</v>
+        <v>72.63224967453041</v>
       </c>
       <c r="L45" s="15" t="b">
         <v>1</v>
@@ -9582,7 +9697,7 @@
         <v>0</v>
       </c>
       <c r="AA45" s="5" t="n">
-        <v>8.698803914461761</v>
+        <v>14.49800652410294</v>
       </c>
       <c r="AB45" s="5" t="n">
         <v>2.482783617252628</v>
@@ -10695,14 +10810,14 @@
       </c>
       <c r="I51" s="15" t="inlineStr">
         <is>
-          <t>[15, 28, 1, 16, 32, 15]</t>
+          <t>[15, 26, 27, 0, 32, 15]</t>
         </is>
       </c>
       <c r="J51" s="16" t="n">
-        <v>4442</v>
+        <v>4332</v>
       </c>
       <c r="K51" s="17" t="n">
-        <v>76.5146070335218</v>
+        <v>74.40492599202177</v>
       </c>
       <c r="L51" s="15" t="b">
         <v>1</v>
@@ -10758,7 +10873,7 @@
         <v>0</v>
       </c>
       <c r="AA51" s="5" t="n">
-        <v>13.98140975987607</v>
+        <v>16.11154144074361</v>
       </c>
       <c r="AB51" s="5" t="n">
         <v>0</v>
@@ -10891,14 +11006,14 @@
       </c>
       <c r="I52" s="15" t="inlineStr">
         <is>
-          <t>[16, 34, 23, 32, 1, 12, 16]</t>
+          <t>[16, 31, 32, 23, 1, 12, 16]</t>
         </is>
       </c>
       <c r="J52" s="16" t="n">
-        <v>4652</v>
+        <v>4863</v>
       </c>
       <c r="K52" s="17" t="n">
-        <v>76.2305482238408</v>
+        <v>75.34279720288458</v>
       </c>
       <c r="L52" s="15" t="b">
         <v>1</v>
@@ -10954,7 +11069,7 @@
         <v>0</v>
       </c>
       <c r="AA52" s="5" t="n">
-        <v>20.36973639164669</v>
+        <v>16.75795960287573</v>
       </c>
       <c r="AB52" s="5" t="n">
         <v>0</v>
@@ -10986,14 +11101,14 @@
       </c>
       <c r="AJ52" s="18" t="inlineStr">
         <is>
-          <t>[16, 31, 12, 34, 23, 1, 32, 16]</t>
+          <t>[16, 31, 34, 12, 23, 32, 16]</t>
         </is>
       </c>
       <c r="AK52" s="19" t="n">
-        <v>5447</v>
+        <v>5501</v>
       </c>
       <c r="AL52" s="20" t="n">
-        <v>74.13570591081958</v>
+        <v>74.87587820600167</v>
       </c>
       <c r="AM52" s="18" t="b">
         <v>1</v>
@@ -11044,7 +11159,7 @@
         <v>0</v>
       </c>
       <c r="BA52" s="5" t="n">
-        <v>6.761383087983567</v>
+        <v>5.837042108866827</v>
       </c>
       <c r="BB52" s="5" t="n">
         <v>19.89044847654913</v>
@@ -11087,14 +11202,14 @@
       </c>
       <c r="I53" s="15" t="inlineStr">
         <is>
-          <t>[16, 34, 31, 23, 32, 16]</t>
+          <t>[16, 34, 31, 23, 1, 32, 16]</t>
         </is>
       </c>
       <c r="J53" s="16" t="n">
-        <v>4984</v>
+        <v>5054</v>
       </c>
       <c r="K53" s="17" t="n">
-        <v>73.1911804597428</v>
+        <v>76.12972937908032</v>
       </c>
       <c r="L53" s="15" t="b">
         <v>1</v>
@@ -11150,7 +11265,7 @@
         <v>0</v>
       </c>
       <c r="AA53" s="5" t="n">
-        <v>10.80887616320687</v>
+        <v>9.556191839656407</v>
       </c>
       <c r="AB53" s="5" t="n">
         <v>0</v>
@@ -11182,14 +11297,14 @@
       </c>
       <c r="AJ53" s="18" t="inlineStr">
         <is>
-          <t>[16, 34, 31, 12, 17, 1, 32, 16]</t>
+          <t>[16, 12, 34, 31, 23, 32, 16]</t>
         </is>
       </c>
       <c r="AK53" s="19" t="n">
-        <v>5401</v>
+        <v>5311</v>
       </c>
       <c r="AL53" s="20" t="n">
-        <v>72.5721514654558</v>
+        <v>75.10551564821257</v>
       </c>
       <c r="AM53" s="18" t="b">
         <v>1</v>
@@ -11240,7 +11355,7 @@
         <v>0</v>
       </c>
       <c r="BA53" s="5" t="n">
-        <v>3.346456692913386</v>
+        <v>4.957050823192556</v>
       </c>
       <c r="BB53" s="5" t="n">
         <v>5.368647100930565</v>
@@ -11378,14 +11493,14 @@
       </c>
       <c r="AJ54" s="18" t="inlineStr">
         <is>
-          <t>[16, 31, 34, 12, 17, 1, 32, 16]</t>
+          <t>[16, 32, 23, 1, 12, 34, 31, 16]</t>
         </is>
       </c>
       <c r="AK54" s="19" t="n">
-        <v>5273</v>
+        <v>6089</v>
       </c>
       <c r="AL54" s="20" t="n">
-        <v>72.30535305191131</v>
+        <v>75.08232804674387</v>
       </c>
       <c r="AM54" s="18" t="b">
         <v>1</v>
@@ -11436,7 +11551,7 @@
         <v>0</v>
       </c>
       <c r="BA54" s="5" t="n">
-        <v>13.40121530629003</v>
+        <v>0</v>
       </c>
       <c r="BB54" s="5" t="n">
         <v>0</v>
@@ -11479,14 +11594,14 @@
       </c>
       <c r="I55" s="15" t="inlineStr">
         <is>
-          <t>[17, 16, 31, 34, 12, 1, 23, 17]</t>
+          <t>[17, 16, 31, 1, 23, 13, 17]</t>
         </is>
       </c>
       <c r="J55" s="16" t="n">
-        <v>5429</v>
+        <v>5179</v>
       </c>
       <c r="K55" s="17" t="n">
-        <v>76.42768627131306</v>
+        <v>76.71388319613814</v>
       </c>
       <c r="L55" s="15" t="b">
         <v>1</v>
@@ -11542,7 +11657,7 @@
         <v>0</v>
       </c>
       <c r="AA55" s="5" t="n">
-        <v>4.284203102961919</v>
+        <v>8.69181946403385</v>
       </c>
       <c r="AB55" s="5" t="n">
         <v>0</v>
@@ -11574,14 +11689,14 @@
       </c>
       <c r="AJ55" s="18" t="inlineStr">
         <is>
-          <t>[17, 16, 31, 34, 12, 1, 23, 17]</t>
+          <t>[17, 16, 12, 34, 31, 1, 23, 17]</t>
         </is>
       </c>
       <c r="AK55" s="19" t="n">
-        <v>5429</v>
+        <v>5472</v>
       </c>
       <c r="AL55" s="20" t="n">
-        <v>76.42768627131306</v>
+        <v>76.65732371352398</v>
       </c>
       <c r="AM55" s="18" t="b">
         <v>1</v>
@@ -11632,7 +11747,7 @@
         <v>0</v>
       </c>
       <c r="BA55" s="5" t="n">
-        <v>4.284203102961919</v>
+        <v>3.526093088857546</v>
       </c>
       <c r="BB55" s="5" t="n">
         <v>12.09449929478138</v>
@@ -11675,14 +11790,14 @@
       </c>
       <c r="I56" s="15" t="inlineStr">
         <is>
-          <t>[17, 23, 1, 12, 31, 34, 16, 17]</t>
+          <t>[17, 23, 1, 16, 31, 34, 12, 17]</t>
         </is>
       </c>
       <c r="J56" s="16" t="n">
-        <v>6237</v>
+        <v>6048</v>
       </c>
       <c r="K56" s="17" t="n">
-        <v>76.54036331337797</v>
+        <v>73.14600940832835</v>
       </c>
       <c r="L56" s="15" t="b">
         <v>1</v>
@@ -11738,7 +11853,7 @@
         <v>0</v>
       </c>
       <c r="AA56" s="5" t="n">
-        <v>3.571428571428571</v>
+        <v>6.493506493506493</v>
       </c>
       <c r="AB56" s="5" t="n">
         <v>0</v>
@@ -12263,14 +12378,14 @@
       </c>
       <c r="I59" s="15" t="inlineStr">
         <is>
-          <t>[18, 2, 13, 8, 29, 18]</t>
+          <t>[18, 1, 23, 13, 2, 18]</t>
         </is>
       </c>
       <c r="J59" s="16" t="n">
-        <v>3968</v>
+        <v>3888</v>
       </c>
       <c r="K59" s="17" t="n">
-        <v>69.18855473644203</v>
+        <v>72.29713270193817</v>
       </c>
       <c r="L59" s="15" t="b">
         <v>1</v>
@@ -12326,7 +12441,7 @@
         <v>0</v>
       </c>
       <c r="AA59" s="5" t="n">
-        <v>19.93543179983858</v>
+        <v>21.54963680387409</v>
       </c>
       <c r="AB59" s="5" t="n">
         <v>10.49233252623083</v>
@@ -14514,14 +14629,14 @@
       </c>
       <c r="AJ70" s="18" t="inlineStr">
         <is>
-          <t>[22, 17, 19, 22]</t>
+          <t>[22, 17, 34, 12, 22]</t>
         </is>
       </c>
       <c r="AK70" s="19" t="n">
-        <v>3093</v>
+        <v>3132</v>
       </c>
       <c r="AL70" s="20" t="n">
-        <v>61.46521819304558</v>
+        <v>63.5149522683278</v>
       </c>
       <c r="AM70" s="18" t="b">
         <v>1</v>
@@ -14572,7 +14687,7 @@
         <v>0</v>
       </c>
       <c r="BA70" s="5" t="n">
-        <v>1.245210727969349</v>
+        <v>0</v>
       </c>
       <c r="BB70" s="5" t="n">
         <v>1.245210727969349</v>
@@ -15007,14 +15122,14 @@
       </c>
       <c r="I73" s="15" t="inlineStr">
         <is>
-          <t>[23, 13, 32, 28, 11, 23]</t>
+          <t>[23, 1, 28, 24, 6, 11, 23]</t>
         </is>
       </c>
       <c r="J73" s="16" t="n">
-        <v>4473</v>
+        <v>4915</v>
       </c>
       <c r="K73" s="17" t="n">
-        <v>76.18882301483481</v>
+        <v>74.74858517898794</v>
       </c>
       <c r="L73" s="15" t="b">
         <v>1</v>
@@ -15070,7 +15185,7 @@
         <v>0</v>
       </c>
       <c r="AA73" s="5" t="n">
-        <v>22.79944770452192</v>
+        <v>15.17086641353124</v>
       </c>
       <c r="AB73" s="5" t="n">
         <v>0</v>
@@ -15399,14 +15514,14 @@
       </c>
       <c r="I75" s="15" t="inlineStr">
         <is>
-          <t>[23, 32, 28, 11, 13, 23]</t>
+          <t>[23, 32, 15, 11, 13, 23]</t>
         </is>
       </c>
       <c r="J75" s="16" t="n">
-        <v>4533</v>
+        <v>4540</v>
       </c>
       <c r="K75" s="17" t="n">
-        <v>69.07047928218503</v>
+        <v>71.66722469090448</v>
       </c>
       <c r="L75" s="15" t="b">
         <v>1</v>
@@ -15462,7 +15577,7 @@
         <v>0</v>
       </c>
       <c r="AA75" s="5" t="n">
-        <v>21.46569646569646</v>
+        <v>21.34442134442135</v>
       </c>
       <c r="AB75" s="5" t="n">
         <v>2.165627165627166</v>
@@ -15494,14 +15609,14 @@
       </c>
       <c r="AJ75" s="18" t="inlineStr">
         <is>
-          <t>[23, 13, 17, 34, 12, 31, 32, 23]</t>
+          <t>[23, 17, 34, 31, 12, 1, 32, 23]</t>
         </is>
       </c>
       <c r="AK75" s="19" t="n">
-        <v>5687</v>
+        <v>5318</v>
       </c>
       <c r="AL75" s="20" t="n">
-        <v>76.58381500748465</v>
+        <v>69.36592006350338</v>
       </c>
       <c r="AM75" s="18" t="b">
         <v>1</v>
@@ -15552,7 +15667,7 @@
         <v>0</v>
       </c>
       <c r="BA75" s="5" t="n">
-        <v>1.472626472626473</v>
+        <v>7.865557865557865</v>
       </c>
       <c r="BB75" s="5" t="n">
         <v>13.79071379071379</v>
@@ -15791,14 +15906,14 @@
       </c>
       <c r="I77" s="15" t="inlineStr">
         <is>
-          <t>[24, 6, 7, 11, 28, 24]</t>
+          <t>[24, 6, 7, 28, 11, 24]</t>
         </is>
       </c>
       <c r="J77" s="16" t="n">
-        <v>4178</v>
+        <v>4177</v>
       </c>
       <c r="K77" s="17" t="n">
-        <v>74.11489988317319</v>
+        <v>67.77527243161661</v>
       </c>
       <c r="L77" s="15" t="b">
         <v>1</v>
@@ -15854,7 +15969,7 @@
         <v>0</v>
       </c>
       <c r="AA77" s="5" t="n">
-        <v>19.70017297712858</v>
+        <v>19.71939265808188</v>
       </c>
       <c r="AB77" s="5" t="n">
         <v>0</v>
@@ -15886,14 +16001,14 @@
       </c>
       <c r="AJ77" s="18" t="inlineStr">
         <is>
-          <t>[24, 6, 11, 23, 13, 28, 24]</t>
+          <t>[24, 11, 23, 13, 28, 24]</t>
         </is>
       </c>
       <c r="AK77" s="19" t="n">
-        <v>5043</v>
+        <v>4327</v>
       </c>
       <c r="AL77" s="20" t="n">
-        <v>71.05408971316373</v>
+        <v>66.6828000597107</v>
       </c>
       <c r="AM77" s="18" t="b">
         <v>1</v>
@@ -15944,7 +16059,7 @@
         <v>0</v>
       </c>
       <c r="BA77" s="5" t="n">
-        <v>3.075148952527388</v>
+        <v>16.83644051508745</v>
       </c>
       <c r="BB77" s="5" t="n">
         <v>10.78224101479915</v>
@@ -16082,14 +16197,14 @@
       </c>
       <c r="AJ78" s="18" t="inlineStr">
         <is>
-          <t>[24, 6, 32, 23, 13, 24]</t>
+          <t>[24, 6, 13, 1, 23, 11, 24]</t>
         </is>
       </c>
       <c r="AK78" s="19" t="n">
-        <v>5406</v>
+        <v>4920</v>
       </c>
       <c r="AL78" s="20" t="n">
-        <v>76.09168411593276</v>
+        <v>72.39237672163087</v>
       </c>
       <c r="AM78" s="18" t="b">
         <v>1</v>
@@ -16140,7 +16255,7 @@
         <v>0</v>
       </c>
       <c r="BA78" s="5" t="n">
-        <v>0</v>
+        <v>8.990011098779133</v>
       </c>
       <c r="BB78" s="5" t="n">
         <v>0</v>
@@ -16866,14 +16981,14 @@
       </c>
       <c r="AJ82" s="18" t="inlineStr">
         <is>
-          <t>[26, 27, 15, 28, 0, 30, 26]</t>
+          <t>[26, 27, 0, 15, 32, 30, 26]</t>
         </is>
       </c>
       <c r="AK82" s="19" t="n">
-        <v>4567</v>
+        <v>4791</v>
       </c>
       <c r="AL82" s="20" t="n">
-        <v>74.7251928762152</v>
+        <v>75.5383145684329</v>
       </c>
       <c r="AM82" s="18" t="b">
         <v>1</v>
@@ -16924,7 +17039,7 @@
         <v>0</v>
       </c>
       <c r="BA82" s="5" t="n">
-        <v>4.675433103736172</v>
+        <v>0</v>
       </c>
       <c r="BB82" s="5" t="n">
         <v>8.286370277603842</v>
@@ -16967,14 +17082,14 @@
       </c>
       <c r="I83" s="15" t="inlineStr">
         <is>
-          <t>[26, 32, 27, 30, 0, 26]</t>
+          <t>[26, 32, 30, 27, 0, 26]</t>
         </is>
       </c>
       <c r="J83" s="16" t="n">
-        <v>3594</v>
+        <v>4225</v>
       </c>
       <c r="K83" s="17" t="n">
-        <v>76.91993454870524</v>
+        <v>74.68578731833023</v>
       </c>
       <c r="L83" s="15" t="b">
         <v>1</v>
@@ -17030,7 +17145,7 @@
         <v>0</v>
       </c>
       <c r="AA83" s="5" t="n">
-        <v>27.11417562360576</v>
+        <v>14.31758264043805</v>
       </c>
       <c r="AB83" s="5" t="n">
         <v>0</v>
@@ -17163,14 +17278,14 @@
       </c>
       <c r="I84" s="15" t="inlineStr">
         <is>
-          <t>[26, 15, 27, 0, 26]</t>
+          <t>[26, 32, 27, 0, 30, 26]</t>
         </is>
       </c>
       <c r="J84" s="16" t="n">
-        <v>3584</v>
+        <v>4029</v>
       </c>
       <c r="K84" s="17" t="n">
-        <v>71.8104412073879</v>
+        <v>76.92218514933194</v>
       </c>
       <c r="L84" s="15" t="b">
         <v>1</v>
@@ -17226,7 +17341,7 @@
         <v>0</v>
       </c>
       <c r="AA84" s="5" t="n">
-        <v>22.67529665587918</v>
+        <v>13.07443365695793</v>
       </c>
       <c r="AB84" s="5" t="n">
         <v>0</v>
@@ -17359,14 +17474,14 @@
       </c>
       <c r="I85" s="15" t="inlineStr">
         <is>
-          <t>[27, 0, 32, 16, 30, 27]</t>
+          <t>[27, 0, 32, 28, 15, 30, 27]</t>
         </is>
       </c>
       <c r="J85" s="16" t="n">
-        <v>4750</v>
+        <v>4902</v>
       </c>
       <c r="K85" s="17" t="n">
-        <v>76.77474853392994</v>
+        <v>71.99648707255528</v>
       </c>
       <c r="L85" s="15" t="b">
         <v>1</v>
@@ -17422,7 +17537,7 @@
         <v>0</v>
       </c>
       <c r="AA85" s="5" t="n">
-        <v>6.972189580885233</v>
+        <v>3.99529964747356</v>
       </c>
       <c r="AB85" s="5" t="n">
         <v>-3.388170779475128</v>
@@ -17454,14 +17569,14 @@
       </c>
       <c r="AJ85" s="18" t="inlineStr">
         <is>
-          <t>[27, 0, 15, 32, 30, 26, 27]</t>
+          <t>[27, 0, 15, 28, 32, 30, 27]</t>
         </is>
       </c>
       <c r="AK85" s="19" t="n">
-        <v>4885</v>
+        <v>5106</v>
       </c>
       <c r="AL85" s="20" t="n">
-        <v>75.5383145684329</v>
+        <v>72.91611180167446</v>
       </c>
       <c r="AM85" s="18" t="b">
         <v>1</v>
@@ -17512,7 +17627,7 @@
         <v>0</v>
       </c>
       <c r="BA85" s="5" t="n">
-        <v>4.328241284763024</v>
+        <v>0</v>
       </c>
       <c r="BB85" s="5" t="n">
         <v>3.99529964747356</v>
@@ -17555,14 +17670,14 @@
       </c>
       <c r="I86" s="15" t="inlineStr">
         <is>
-          <t>[27, 0, 26, 32, 30, 27]</t>
+          <t>[27, 15, 26, 0, 27]</t>
         </is>
       </c>
       <c r="J86" s="16" t="n">
-        <v>3841</v>
+        <v>3245</v>
       </c>
       <c r="K86" s="17" t="n">
-        <v>74.68578731833021</v>
+        <v>71.81044143013141</v>
       </c>
       <c r="L86" s="15" t="b">
         <v>1</v>
@@ -17618,7 +17733,7 @@
         <v>0</v>
       </c>
       <c r="AA86" s="5" t="n">
-        <v>20.83676834295136</v>
+        <v>33.12036273701566</v>
       </c>
       <c r="AB86" s="5" t="n">
         <v>0</v>
@@ -17650,14 +17765,14 @@
       </c>
       <c r="AJ86" s="18" t="inlineStr">
         <is>
-          <t>[27, 0, 32, 28, 15, 30, 27]</t>
+          <t>[27, 0, 32, 1, 15, 30, 27]</t>
         </is>
       </c>
       <c r="AK86" s="19" t="n">
-        <v>4761</v>
+        <v>4852</v>
       </c>
       <c r="AL86" s="20" t="n">
-        <v>71.99648707255528</v>
+        <v>76.98869770383878</v>
       </c>
       <c r="AM86" s="18" t="b">
         <v>1</v>
@@ -17708,7 +17823,7 @@
         <v>0</v>
       </c>
       <c r="BA86" s="5" t="n">
-        <v>1.875515251442704</v>
+        <v>0</v>
       </c>
       <c r="BB86" s="5" t="n">
         <v>0</v>
@@ -17751,14 +17866,14 @@
       </c>
       <c r="I87" s="15" t="inlineStr">
         <is>
-          <t>[27, 30, 32, 16, 0, 27]</t>
+          <t>[27, 30, 32, 28, 15, 0, 27]</t>
         </is>
       </c>
       <c r="J87" s="16" t="n">
-        <v>4898</v>
+        <v>4987</v>
       </c>
       <c r="K87" s="17" t="n">
-        <v>76.30266589653553</v>
+        <v>72.72308136763816</v>
       </c>
       <c r="L87" s="15" t="b">
         <v>1</v>
@@ -17814,7 +17929,7 @@
         <v>0</v>
       </c>
       <c r="AA87" s="5" t="n">
-        <v>1.784640064166834</v>
+        <v>0</v>
       </c>
       <c r="AB87" s="5" t="n">
         <v>-0.08020854220974534</v>
@@ -17846,14 +17961,14 @@
       </c>
       <c r="AJ87" s="18" t="inlineStr">
         <is>
-          <t>[27, 0, 32, 28, 15, 30, 27]</t>
+          <t>[27, 30, 32, 28, 15, 0, 27]</t>
         </is>
       </c>
       <c r="AK87" s="19" t="n">
-        <v>4937</v>
+        <v>4987</v>
       </c>
       <c r="AL87" s="20" t="n">
-        <v>71.99648707255528</v>
+        <v>72.72308136763816</v>
       </c>
       <c r="AM87" s="18" t="b">
         <v>1</v>
@@ -17904,7 +18019,7 @@
         <v>0</v>
       </c>
       <c r="BA87" s="5" t="n">
-        <v>1.002606777621817</v>
+        <v>0</v>
       </c>
       <c r="BB87" s="5" t="n">
         <v>0</v>
@@ -17947,14 +18062,14 @@
       </c>
       <c r="I88" s="15" t="inlineStr">
         <is>
-          <t>[28, 27, 0, 15, 6, 28]</t>
+          <t>[28, 6, 27, 0, 30, 15, 28]</t>
         </is>
       </c>
       <c r="J88" s="16" t="n">
-        <v>4707</v>
+        <v>4946</v>
       </c>
       <c r="K88" s="17" t="n">
-        <v>74.48323704856701</v>
+        <v>74.8499243526344</v>
       </c>
       <c r="L88" s="15" t="b">
         <v>1</v>
@@ -18010,7 +18125,7 @@
         <v>0</v>
       </c>
       <c r="AA88" s="5" t="n">
-        <v>11.65540540540541</v>
+        <v>7.169669669669669</v>
       </c>
       <c r="AB88" s="5" t="n">
         <v>3.190690690690691</v>
@@ -18042,14 +18157,14 @@
       </c>
       <c r="AJ88" s="18" t="inlineStr">
         <is>
-          <t>[28, 6, 27, 0, 30, 15, 28]</t>
+          <t>[28, 15, 32, 23, 11, 6, 28]</t>
         </is>
       </c>
       <c r="AK88" s="19" t="n">
-        <v>4946</v>
+        <v>5028</v>
       </c>
       <c r="AL88" s="20" t="n">
-        <v>74.8499243526344</v>
+        <v>68.80721202182097</v>
       </c>
       <c r="AM88" s="18" t="b">
         <v>1</v>
@@ -18100,7 +18215,7 @@
         <v>0</v>
       </c>
       <c r="BA88" s="5" t="n">
-        <v>7.169669669669669</v>
+        <v>5.63063063063063</v>
       </c>
       <c r="BB88" s="5" t="n">
         <v>7.169669669669669</v>
@@ -18143,14 +18258,14 @@
       </c>
       <c r="I89" s="15" t="inlineStr">
         <is>
-          <t>[28, 15, 32, 23, 11, 6, 28]</t>
+          <t>[28, 32, 23, 11, 24, 6, 28]</t>
         </is>
       </c>
       <c r="J89" s="16" t="n">
-        <v>4726</v>
+        <v>4733</v>
       </c>
       <c r="K89" s="17" t="n">
-        <v>68.80721202182097</v>
+        <v>72.19802163182189</v>
       </c>
       <c r="L89" s="15" t="b">
         <v>1</v>
@@ -18206,7 +18321,7 @@
         <v>0</v>
       </c>
       <c r="AA89" s="5" t="n">
-        <v>10.35660091047041</v>
+        <v>10.22382397572079</v>
       </c>
       <c r="AB89" s="5" t="n">
         <v>1.194992412746586</v>
@@ -18238,14 +18353,14 @@
       </c>
       <c r="AJ89" s="18" t="inlineStr">
         <is>
-          <t>[28, 15, 30, 32, 23, 11, 6, 28]</t>
+          <t>[28, 15, 0, 30, 32, 23, 11, 28]</t>
         </is>
       </c>
       <c r="AK89" s="19" t="n">
-        <v>5126</v>
+        <v>5209</v>
       </c>
       <c r="AL89" s="20" t="n">
-        <v>72.46790103387278</v>
+        <v>73.08182586017077</v>
       </c>
       <c r="AM89" s="18" t="b">
         <v>1</v>
@@ -18296,7 +18411,7 @@
         <v>0</v>
       </c>
       <c r="BA89" s="5" t="n">
-        <v>2.769347496206374</v>
+        <v>1.194992412746586</v>
       </c>
       <c r="BB89" s="5" t="n">
         <v>8.38391502276176</v>
@@ -18339,14 +18454,14 @@
       </c>
       <c r="I90" s="15" t="inlineStr">
         <is>
-          <t>[28, 24, 13, 23, 11, 15, 28]</t>
+          <t>[28, 32, 23, 11, 24, 6, 28]</t>
         </is>
       </c>
       <c r="J90" s="16" t="n">
-        <v>4620</v>
+        <v>4468</v>
       </c>
       <c r="K90" s="17" t="n">
-        <v>76.64972214507708</v>
+        <v>72.19802163182189</v>
       </c>
       <c r="L90" s="15" t="b">
         <v>1</v>
@@ -18402,7 +18517,7 @@
         <v>0</v>
       </c>
       <c r="AA90" s="5" t="n">
-        <v>9.340659340659341</v>
+        <v>12.32339089481947</v>
       </c>
       <c r="AB90" s="5" t="n">
         <v>0</v>
@@ -18630,14 +18745,14 @@
       </c>
       <c r="AJ91" s="18" t="inlineStr">
         <is>
-          <t>[29, 2, 13, 18, 29]</t>
+          <t>[29, 2, 8, 18, 29]</t>
         </is>
       </c>
       <c r="AK91" s="19" t="n">
-        <v>2796</v>
+        <v>2994</v>
       </c>
       <c r="AL91" s="20" t="n">
-        <v>68.79768171714818</v>
+        <v>60.6221310364861</v>
       </c>
       <c r="AM91" s="18" t="b">
         <v>1</v>
@@ -18688,7 +18803,7 @@
         <v>0</v>
       </c>
       <c r="BA91" s="5" t="n">
-        <v>6.613226452905812</v>
+        <v>0</v>
       </c>
       <c r="BB91" s="5" t="n">
         <v>0</v>
@@ -18826,14 +18941,14 @@
       </c>
       <c r="AJ92" s="18" t="inlineStr">
         <is>
-          <t>[29, 18, 2, 13, 8, 29]</t>
+          <t>[29, 11, 13, 8, 29]</t>
         </is>
       </c>
       <c r="AK92" s="19" t="n">
-        <v>3951</v>
+        <v>3946</v>
       </c>
       <c r="AL92" s="20" t="n">
-        <v>69.18855473644203</v>
+        <v>74.53326791831809</v>
       </c>
       <c r="AM92" s="18" t="b">
         <v>1</v>
@@ -18884,7 +18999,7 @@
         <v>0</v>
       </c>
       <c r="BA92" s="5" t="n">
-        <v>0</v>
+        <v>0.1265502404454568</v>
       </c>
       <c r="BB92" s="5" t="n">
         <v>0.1265502404454568</v>
@@ -19123,14 +19238,14 @@
       </c>
       <c r="I94" s="15" t="inlineStr">
         <is>
-          <t>[30, 32, 23, 11, 28, 15, 0, 30]</t>
+          <t>[30, 32, 28, 0, 27, 30]</t>
         </is>
       </c>
       <c r="J94" s="16" t="n">
-        <v>5012</v>
+        <v>4308</v>
       </c>
       <c r="K94" s="17" t="n">
-        <v>73.08182586017075</v>
+        <v>73.12396826780835</v>
       </c>
       <c r="L94" s="15" t="b">
         <v>1</v>
@@ -19186,7 +19301,7 @@
         <v>0</v>
       </c>
       <c r="AA94" s="5" t="n">
-        <v>0.5358205993252629</v>
+        <v>14.50684659654694</v>
       </c>
       <c r="AB94" s="5" t="n">
         <v>0</v>
@@ -19218,14 +19333,14 @@
       </c>
       <c r="AJ94" s="18" t="inlineStr">
         <is>
-          <t>[30, 27, 0, 15, 28, 32, 30]</t>
+          <t>[30, 32, 16, 31, 34, 1, 30]</t>
         </is>
       </c>
       <c r="AK94" s="19" t="n">
-        <v>4809</v>
+        <v>4736</v>
       </c>
       <c r="AL94" s="20" t="n">
-        <v>72.91611180167446</v>
+        <v>76.36835853210859</v>
       </c>
       <c r="AM94" s="18" t="b">
         <v>1</v>
@@ -19276,7 +19391,7 @@
         <v>0</v>
       </c>
       <c r="BA94" s="5" t="n">
-        <v>4.564397697955943</v>
+        <v>6.013097836872396</v>
       </c>
       <c r="BB94" s="5" t="n">
         <v>1.647152212740623</v>
@@ -19414,14 +19529,14 @@
       </c>
       <c r="AJ95" s="18" t="inlineStr">
         <is>
-          <t>[30, 27, 0, 15, 28, 11, 30]</t>
+          <t>[30, 27, 0, 32, 1, 15, 30]</t>
         </is>
       </c>
       <c r="AK95" s="19" t="n">
-        <v>4937</v>
+        <v>4981</v>
       </c>
       <c r="AL95" s="20" t="n">
-        <v>76.80221904799268</v>
+        <v>76.98869770383878</v>
       </c>
       <c r="AM95" s="18" t="b">
         <v>1</v>
@@ -19472,7 +19587,7 @@
         <v>0</v>
       </c>
       <c r="BA95" s="5" t="n">
-        <v>6.087121932661214</v>
+        <v>5.250142666920297</v>
       </c>
       <c r="BB95" s="5" t="n">
         <v>0</v>
@@ -19515,14 +19630,14 @@
       </c>
       <c r="I96" s="15" t="inlineStr">
         <is>
-          <t>[30, 32, 23, 28, 15, 0, 30]</t>
+          <t>[30, 27, 0, 15, 11, 28, 30]</t>
         </is>
       </c>
       <c r="J96" s="16" t="n">
-        <v>4680</v>
+        <v>4971</v>
       </c>
       <c r="K96" s="17" t="n">
-        <v>71.0738771346476</v>
+        <v>76.91777059531171</v>
       </c>
       <c r="L96" s="15" t="b">
         <v>1</v>
@@ -19578,7 +19693,7 @@
         <v>0</v>
       </c>
       <c r="AA96" s="5" t="n">
-        <v>11.26279863481229</v>
+        <v>5.745164960182024</v>
       </c>
       <c r="AB96" s="5" t="n">
         <v>5.745164960182024</v>
@@ -19610,14 +19725,14 @@
       </c>
       <c r="AJ96" s="18" t="inlineStr">
         <is>
-          <t>[30, 32, 23, 11, 28, 15, 0, 30]</t>
+          <t>[30, 27, 0, 15, 11, 28, 30]</t>
         </is>
       </c>
       <c r="AK96" s="19" t="n">
-        <v>5274</v>
+        <v>4971</v>
       </c>
       <c r="AL96" s="20" t="n">
-        <v>73.08182586017075</v>
+        <v>76.91777059531171</v>
       </c>
       <c r="AM96" s="18" t="b">
         <v>1</v>
@@ -19668,7 +19783,7 @@
         <v>0</v>
       </c>
       <c r="BA96" s="5" t="n">
-        <v>0</v>
+        <v>5.745164960182024</v>
       </c>
       <c r="BB96" s="5" t="n">
         <v>9.878649981039061</v>
@@ -19711,14 +19826,14 @@
       </c>
       <c r="I97" s="15" t="inlineStr">
         <is>
-          <t>[31, 16, 32, 23, 1, 12, 34, 31]</t>
+          <t>[31, 1, 23, 32, 16, 12, 34, 31]</t>
         </is>
       </c>
       <c r="J97" s="16" t="n">
-        <v>6177</v>
+        <v>6654</v>
       </c>
       <c r="K97" s="17" t="n">
-        <v>75.08232804674387</v>
+        <v>75.01421864387075</v>
       </c>
       <c r="L97" s="15" t="b">
         <v>1</v>
@@ -19774,7 +19889,7 @@
         <v>0</v>
       </c>
       <c r="AA97" s="5" t="n">
-        <v>7.168620378719567</v>
+        <v>0</v>
       </c>
       <c r="AB97" s="5" t="n">
         <v>0</v>
@@ -19806,14 +19921,14 @@
       </c>
       <c r="AJ97" s="18" t="inlineStr">
         <is>
-          <t>[31, 1, 23, 17, 34, 16, 12, 31]</t>
+          <t>[31, 1, 23, 11, 13, 17, 34, 12, 31]</t>
         </is>
       </c>
       <c r="AK97" s="19" t="n">
-        <v>6055</v>
+        <v>6142</v>
       </c>
       <c r="AL97" s="20" t="n">
-        <v>70.30796949750116</v>
+        <v>72.92391473027244</v>
       </c>
       <c r="AM97" s="18" t="b">
         <v>1</v>
@@ -19864,7 +19979,7 @@
         <v>0</v>
       </c>
       <c r="BA97" s="5" t="n">
-        <v>9.002103997595432</v>
+        <v>7.694619777577397</v>
       </c>
       <c r="BB97" s="5" t="n">
         <v>18.04929365795011</v>
@@ -20103,14 +20218,14 @@
       </c>
       <c r="I99" s="15" t="inlineStr">
         <is>
-          <t>[31, 23, 1, 12, 34, 16, 31]</t>
+          <t>[31, 23, 1, 32, 16, 34, 31]</t>
         </is>
       </c>
       <c r="J99" s="16" t="n">
-        <v>5712</v>
+        <v>5381</v>
       </c>
       <c r="K99" s="17" t="n">
-        <v>69.64229689432317</v>
+        <v>76.1297293790803</v>
       </c>
       <c r="L99" s="15" t="b">
         <v>1</v>
@@ -20166,7 +20281,7 @@
         <v>0</v>
       </c>
       <c r="AA99" s="5" t="n">
-        <v>5.758125721828081</v>
+        <v>11.21927074740142</v>
       </c>
       <c r="AB99" s="5" t="n">
         <v>0</v>
@@ -20198,14 +20313,14 @@
       </c>
       <c r="AJ99" s="18" t="inlineStr">
         <is>
-          <t>[31, 23, 1, 12, 34, 16, 31]</t>
+          <t>[31, 32, 23, 1, 12, 16, 31]</t>
         </is>
       </c>
       <c r="AK99" s="19" t="n">
-        <v>5712</v>
+        <v>5758</v>
       </c>
       <c r="AL99" s="20" t="n">
-        <v>69.64229689432317</v>
+        <v>75.34279720288458</v>
       </c>
       <c r="AM99" s="18" t="b">
         <v>1</v>
@@ -20256,7 +20371,7 @@
         <v>0</v>
       </c>
       <c r="BA99" s="5" t="n">
-        <v>5.758125721828081</v>
+        <v>4.999175053621514</v>
       </c>
       <c r="BB99" s="5" t="n">
         <v>23.13149645273057</v>
@@ -20299,14 +20414,14 @@
       </c>
       <c r="I100" s="15" t="inlineStr">
         <is>
-          <t>[32, 16, 34, 31, 12, 17, 1, 32]</t>
+          <t>[32, 16, 0, 27, 30, 32]</t>
         </is>
       </c>
       <c r="J100" s="16" t="n">
-        <v>5403</v>
+        <v>4475</v>
       </c>
       <c r="K100" s="17" t="n">
-        <v>72.5721514654558</v>
+        <v>76.30266589653552</v>
       </c>
       <c r="L100" s="15" t="b">
         <v>1</v>
@@ -20362,7 +20477,7 @@
         <v>0</v>
       </c>
       <c r="AA100" s="5" t="n">
-        <v>10.03996003996004</v>
+        <v>25.49117549117549</v>
       </c>
       <c r="AB100" s="5" t="n">
         <v>5.328005328005328</v>
@@ -20495,14 +20610,14 @@
       </c>
       <c r="I101" s="15" t="inlineStr">
         <is>
-          <t>[32, 23, 16, 34, 12, 32]</t>
+          <t>[32, 23, 11, 6, 28, 15, 30, 32]</t>
         </is>
       </c>
       <c r="J101" s="16" t="n">
-        <v>4998</v>
+        <v>5249</v>
       </c>
       <c r="K101" s="17" t="n">
-        <v>73.86462458468102</v>
+        <v>72.46790103387276</v>
       </c>
       <c r="L101" s="15" t="b">
         <v>1</v>
@@ -20558,7 +20673,7 @@
         <v>0</v>
       </c>
       <c r="AA101" s="5" t="n">
-        <v>10.34977578475336</v>
+        <v>5.847533632286996</v>
       </c>
       <c r="AB101" s="5" t="n">
         <v>1.991031390134529</v>
@@ -20590,14 +20705,14 @@
       </c>
       <c r="AJ101" s="18" t="inlineStr">
         <is>
-          <t>[32, 16, 31, 34, 12, 1, 23, 32]</t>
+          <t>[32, 16, 34, 31, 12, 1, 23, 32]</t>
         </is>
       </c>
       <c r="AK101" s="19" t="n">
-        <v>5534</v>
+        <v>5531</v>
       </c>
       <c r="AL101" s="20" t="n">
-        <v>74.78458120165985</v>
+        <v>75.05137961520435</v>
       </c>
       <c r="AM101" s="18" t="b">
         <v>1</v>
@@ -20648,7 +20763,7 @@
         <v>0</v>
       </c>
       <c r="BA101" s="5" t="n">
-        <v>0.7354260089686099</v>
+        <v>0.7892376681614349</v>
       </c>
       <c r="BB101" s="5" t="n">
         <v>4.089686098654709</v>
@@ -20691,14 +20806,14 @@
       </c>
       <c r="I102" s="15" t="inlineStr">
         <is>
-          <t>[32, 23, 13, 1, 12, 34, 32]</t>
+          <t>[32, 28, 27, 0, 30, 32]</t>
         </is>
       </c>
       <c r="J102" s="16" t="n">
-        <v>5069</v>
+        <v>4717</v>
       </c>
       <c r="K102" s="17" t="n">
-        <v>75.76383326003132</v>
+        <v>73.10104639937089</v>
       </c>
       <c r="L102" s="15" t="b">
         <v>1</v>
@@ -20754,7 +20869,7 @@
         <v>0</v>
       </c>
       <c r="AA102" s="5" t="n">
-        <v>16.72416625595531</v>
+        <v>22.50698209298505</v>
       </c>
       <c r="AB102" s="5" t="n">
         <v>3.400689995071464</v>
@@ -20786,14 +20901,14 @@
       </c>
       <c r="AJ102" s="18" t="inlineStr">
         <is>
-          <t>[32, 16, 12, 34, 31, 1, 23, 32]</t>
+          <t>[32, 16, 12, 34, 31, 23, 32]</t>
         </is>
       </c>
       <c r="AK102" s="19" t="n">
-        <v>6087</v>
+        <v>5679</v>
       </c>
       <c r="AL102" s="20" t="n">
-        <v>75.01421864387075</v>
+        <v>75.10551564821256</v>
       </c>
       <c r="AM102" s="18" t="b">
         <v>1</v>
@@ -20844,7 +20959,7 @@
         <v>0</v>
       </c>
       <c r="BA102" s="5" t="n">
-        <v>0</v>
+        <v>6.702809265648102</v>
       </c>
       <c r="BB102" s="5" t="n">
         <v>2.365697387875801</v>
@@ -21475,14 +21590,14 @@
       </c>
       <c r="I106" s="15" t="inlineStr">
         <is>
-          <t>[34, 32, 23, 1, 16, 12, 34]</t>
+          <t>[34, 16, 32, 23, 1, 12, 31, 34]</t>
         </is>
       </c>
       <c r="J106" s="16" t="n">
-        <v>5192</v>
+        <v>6039</v>
       </c>
       <c r="K106" s="17" t="n">
-        <v>74.0692681981388</v>
+        <v>75.11269845882315</v>
       </c>
       <c r="L106" s="15" t="b">
         <v>1</v>
@@ -21538,7 +21653,7 @@
         <v>0</v>
       </c>
       <c r="AA106" s="5" t="n">
-        <v>15.89178681354285</v>
+        <v>2.170743560667423</v>
       </c>
       <c r="AB106" s="5" t="n">
         <v>1.052972622711809</v>
@@ -21671,14 +21786,14 @@
       </c>
       <c r="I107" s="15" t="inlineStr">
         <is>
-          <t>[34, 23, 11, 13, 1, 12, 31, 34]</t>
+          <t>[34, 16, 31, 32, 1, 17, 34]</t>
         </is>
       </c>
       <c r="J107" s="16" t="n">
-        <v>5505</v>
+        <v>4996</v>
       </c>
       <c r="K107" s="17" t="n">
-        <v>74.42838266767468</v>
+        <v>72.80185862639158</v>
       </c>
       <c r="L107" s="15" t="b">
         <v>1</v>
@@ -21734,7 +21849,7 @@
         <v>0</v>
       </c>
       <c r="AA107" s="5" t="n">
-        <v>2.995594713656387</v>
+        <v>11.9647577092511</v>
       </c>
       <c r="AB107" s="5" t="n">
         <v>0.2819383259911895</v>
@@ -21867,14 +21982,14 @@
       </c>
       <c r="I108" s="15" t="inlineStr">
         <is>
-          <t>[34, 16, 11, 23, 17, 34]</t>
+          <t>[34, 23, 32, 16, 31, 12, 34]</t>
         </is>
       </c>
       <c r="J108" s="16" t="n">
-        <v>5028</v>
+        <v>5489</v>
       </c>
       <c r="K108" s="17" t="n">
-        <v>75.80977144016293</v>
+        <v>71.19715699148207</v>
       </c>
       <c r="L108" s="15" t="b">
         <v>1</v>
@@ -21930,7 +22045,7 @@
         <v>0</v>
       </c>
       <c r="AA108" s="5" t="n">
-        <v>17.50615258408532</v>
+        <v>9.942575881870386</v>
       </c>
       <c r="AB108" s="5" t="n">
         <v>0</v>
@@ -21962,14 +22077,14 @@
       </c>
       <c r="AJ108" s="18" t="inlineStr">
         <is>
-          <t>[34, 31, 16, 12, 32, 1, 17, 34]</t>
+          <t>[34, 16, 31, 1, 23, 17, 12, 34]</t>
         </is>
       </c>
       <c r="AK108" s="19" t="n">
-        <v>5445</v>
+        <v>5297</v>
       </c>
       <c r="AL108" s="20" t="n">
-        <v>74.5329364759455</v>
+        <v>76.0987958713573</v>
       </c>
       <c r="AM108" s="18" t="b">
         <v>1</v>
@@ -22020,7 +22135,7 @@
         <v>0</v>
       </c>
       <c r="BA108" s="5" t="n">
-        <v>10.66447908121411</v>
+        <v>13.09269893355209</v>
       </c>
       <c r="BB108" s="5" t="n">
         <v>9.942575881870386</v>
@@ -22127,19 +22242,19 @@
         <v>105</v>
       </c>
       <c r="D2" t="n">
-        <v>4408.571428571428</v>
+        <v>4417.114285714286</v>
       </c>
       <c r="E2" t="n">
-        <v>1439.446560695777</v>
+        <v>1440.056377864621</v>
       </c>
       <c r="F2" t="n">
         <v>3287</v>
       </c>
       <c r="G2" t="n">
-        <v>4946</v>
+        <v>4971</v>
       </c>
       <c r="H2" t="n">
-        <v>5406</v>
+        <v>5378</v>
       </c>
       <c r="I2" t="n">
         <v>555</v>
@@ -22316,19 +22431,19 @@
         <v>105</v>
       </c>
       <c r="C2" t="n">
-        <v>1655.47619047619</v>
+        <v>1664.019047619048</v>
       </c>
       <c r="D2" t="n">
-        <v>1540</v>
+        <v>1532</v>
       </c>
       <c r="E2" t="n">
-        <v>1055.819970224001</v>
+        <v>1066.989302997281</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>8.330397473485909e-18</v>
+        <v>5.696893031494331e-18</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -22344,19 +22459,19 @@
         <v>105</v>
       </c>
       <c r="C3" t="n">
-        <v>285.8571428571428</v>
+        <v>294.4</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="E3" t="n">
-        <v>519.0248517203166</v>
+        <v>522.8964561422786</v>
       </c>
       <c r="F3" t="n">
-        <v>347</v>
+        <v>324.5</v>
       </c>
       <c r="G3" t="n">
-        <v>2.676543543477171e-07</v>
+        <v>2.16396247952928e-07</v>
       </c>
       <c r="H3" t="b">
         <v>1</v>
@@ -22372,19 +22487,19 @@
         <v>105</v>
       </c>
       <c r="C4" t="n">
-        <v>322.8571428571428</v>
+        <v>331.4</v>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>74</v>
       </c>
       <c r="E4" t="n">
-        <v>614.2533840201613</v>
+        <v>579.9333781365953</v>
       </c>
       <c r="F4" t="n">
-        <v>349</v>
+        <v>215</v>
       </c>
       <c r="G4" t="n">
-        <v>1.020354055672476e-07</v>
+        <v>2.954302153547962e-09</v>
       </c>
       <c r="H4" t="b">
         <v>1</v>
@@ -22393,4 +22508,416 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>CHEQUEO DE CONVERGENCIA PPO  ·  35 nodos</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>CRITERIOS DE CONVERGENCIA  (evaluados sobre las últimas W = 50 PPO updates)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>Condición</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>Métrica observada</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>Cómo se mide</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="inlineStr">
+        <is>
+          <t>Umbral de aprobación</t>
+        </is>
+      </c>
+      <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>Nota de diseño</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>C1 — Reward aplanado</t>
+        </is>
+      </c>
+      <c r="B5" s="27" t="inlineStr">
+        <is>
+          <t>Pendiente relativa del reward de entrenamiento</t>
+        </is>
+      </c>
+      <c r="C5" s="27" t="inlineStr">
+        <is>
+          <t>Regresión lineal sobre la ventana → slope / |media reward|</t>
+        </is>
+      </c>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>&lt; 0.001  (adimensional)</t>
+        </is>
+      </c>
+      <c r="E5" s="27" t="inlineStr">
+        <is>
+          <t>Valor relativo para que sea comparable entre escalas de reward distintas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>C2 — Explained Variance estable</t>
+        </is>
+      </c>
+      <c r="B6" s="27" t="inlineStr">
+        <is>
+          <t>Media y pendiente relativa de explained_var del crítico</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>Media aritmética + regresión lineal sobre la ventana</t>
+        </is>
+      </c>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>Media ≥ 0.5  Y  |pendiente rel.| &lt; 0.001</t>
+        </is>
+      </c>
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>Umbral 0.5 coincide con la línea de referencia en PPO_Diagnostics_AM.png.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>C3 — KL divergence controlada</t>
+        </is>
+      </c>
+      <c r="B7" s="27" t="inlineStr">
+        <is>
+          <t>Fracción de updates en ventana con KL &gt; umbral KL</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>Proporción de filas donde kl_divergence &gt; kl_threshold</t>
+        </is>
+      </c>
+      <c r="D7" s="27" t="inlineStr">
+        <is>
+          <t>Fracción de violaciones ≤ 5%  (umbral KL = 0.02)</t>
+        </is>
+      </c>
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>Umbral KL 0.02 coincide con la línea de referencia en PPO_Diagnostics_AM.png.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>C4 — Entropía estabilizada</t>
+        </is>
+      </c>
+      <c r="B8" s="27" t="inlineStr">
+        <is>
+          <t>Pendiente ABSOLUTA de la entropía de la política</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>Regresión lineal sobre la ventana → |slope| en nats/update</t>
+        </is>
+      </c>
+      <c r="D8" s="27" t="inlineStr">
+        <is>
+          <t>&lt; 0.0005  nats/update</t>
+        </is>
+      </c>
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>Se usa pendiente absoluta (no relativa) porque la entropía puede pasar por 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1"/>
+    <row r="10" ht="40" customHeight="1"/>
+    <row r="11">
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>RESULTADOS DEL CHEQUEO</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="28" t="inlineStr">
+        <is>
+          <t>Identificación</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="n"/>
+      <c r="C12" s="29" t="n"/>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>C1 — Reward Aplanado</t>
+        </is>
+      </c>
+      <c r="E12" s="30" t="n"/>
+      <c r="F12" s="30" t="n"/>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>C2 — Explained Variance</t>
+        </is>
+      </c>
+      <c r="H12" s="31" t="n"/>
+      <c r="I12" s="31" t="n"/>
+      <c r="J12" s="31" t="n"/>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>C3 — KL Divergence</t>
+        </is>
+      </c>
+      <c r="L12" s="32" t="n"/>
+      <c r="M12" s="32" t="n"/>
+      <c r="N12" s="33" t="inlineStr">
+        <is>
+          <t>C4 — Entropía</t>
+        </is>
+      </c>
+      <c r="O12" s="34" t="n"/>
+      <c r="P12" s="34" t="n"/>
+      <c r="Q12" s="35" t="inlineStr">
+        <is>
+          <t>Veredicto Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t>Nodos</t>
+        </is>
+      </c>
+      <c r="B13" s="28" t="inlineStr">
+        <is>
+          <t>Total
+Updates</t>
+        </is>
+      </c>
+      <c r="C13" s="28" t="inlineStr">
+        <is>
+          <t>Ventana
+(W usado)</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Pendiente
+Reward Rel.
+(medido)</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>Umbral
+(&lt; 0.001)</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>C1
+Resultado</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>EV Media
+(medido)</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>EV Pendiente
+Rel. (medido)</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>Umbral
+Media ≥ 0.5</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>C2
+Resultado</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
+        <is>
+          <t>Fracc.
+Violaciones
+KL (medido)</t>
+        </is>
+      </c>
+      <c r="L13" s="9" t="inlineStr">
+        <is>
+          <t>Umbral
+(≤ 5%)</t>
+        </is>
+      </c>
+      <c r="M13" s="9" t="inlineStr">
+        <is>
+          <t>C3
+Resultado</t>
+        </is>
+      </c>
+      <c r="N13" s="33" t="inlineStr">
+        <is>
+          <t>Pendiente
+Entropía Abs.
+(medido)</t>
+        </is>
+      </c>
+      <c r="O13" s="33" t="inlineStr">
+        <is>
+          <t>Umbral
+(&lt; 0.0005)</t>
+        </is>
+      </c>
+      <c r="P13" s="33" t="inlineStr">
+        <is>
+          <t>C4
+Resultado</t>
+        </is>
+      </c>
+      <c r="Q13" s="35" t="inlineStr">
+        <is>
+          <t>CONVERGIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B14" s="37" t="n">
+        <v>500</v>
+      </c>
+      <c r="C14" s="37" t="n">
+        <v>50</v>
+      </c>
+      <c r="D14" s="38" t="n">
+        <v>0.000174</v>
+      </c>
+      <c r="E14" s="39" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="F14" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G14" s="41" t="n">
+        <v>0.8488</v>
+      </c>
+      <c r="H14" s="38" t="n">
+        <v>0.000132</v>
+      </c>
+      <c r="I14" s="42" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J14" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K14" s="41" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="L14" s="42" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M14" s="43" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="N14" s="38" t="n">
+        <v>0.000314</v>
+      </c>
+      <c r="O14" s="39" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="P14" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q14" s="44" t="inlineStr">
+        <is>
+          <t>NO — extender entrenamiento</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="K12:M12"/>
+    <mergeCell ref="G12:J12"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A11:Q11"/>
+    <mergeCell ref="N12:P12"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Resultados con 35 nodos, gap est 4% y det 6.3%
</commit_message>
<xml_diff>
--- a/results_35nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_35nodes/DRL_Routing_Summary_AM.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="0.000000"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,16 +62,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00C00000"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00C00000"/>
+      <color rgb="00548235"/>
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -148,11 +143,6 @@
         <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFE0E0"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -200,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -312,10 +302,7 @@
     <xf numFmtId="2" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -737,7 +724,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>35.26441483270555</v>
+        <v>35.47424134753999</v>
       </c>
     </row>
     <row r="4">
@@ -747,13 +734,13 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>4202.838095238095</v>
+        <v>4255.361904761905</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>7.366119880473141</v>
+        <v>6.303476736875134</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>566.8754305158342</v>
+        <v>572.0171201796759</v>
       </c>
     </row>
     <row r="5">
@@ -769,7 +756,7 @@
         <v>0.7830855557137725</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>13714.20839400519</v>
+        <v>12755.33604394822</v>
       </c>
     </row>
     <row r="6">
@@ -785,7 +772,7 @@
         <v>13.09578163496531</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>5.311296099708194</v>
+        <v>5.161812191917783</v>
       </c>
     </row>
     <row r="7">
@@ -801,7 +788,7 @@
         <v>52.95029311789443</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.5005405062720889</v>
+        <v>0.4802999042329335</v>
       </c>
     </row>
     <row r="9">
@@ -849,7 +836,7 @@
         <v>0</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>98.01252910069057</v>
+        <v>88.31757817949567</v>
       </c>
     </row>
     <row r="12">
@@ -859,13 +846,13 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>4417.114285714286</v>
+        <v>4368.409523809524</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>2.906151551462991</v>
+        <v>4.006824074793214</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>566.8754305158342</v>
+        <v>572.0171201796759</v>
       </c>
     </row>
     <row r="13">
@@ -881,7 +868,7 @@
         <v>11.87591998359568</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>13.8415881565639</v>
+        <v>12.74665423801967</v>
       </c>
     </row>
     <row r="14">
@@ -911,7 +898,7 @@
         <v>14.13950847586963</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>11.01879392351423</v>
+        <v>10.54941813151042</v>
       </c>
     </row>
     <row r="17">
@@ -941,7 +928,7 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>893.2330803871155</v>
+        <v>1201.365214109421</v>
       </c>
     </row>
     <row r="20">
@@ -951,7 +938,7 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>566.8754305158342</v>
+        <v>572.0171201796759</v>
       </c>
     </row>
     <row r="21">
@@ -961,7 +948,7 @@
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>13714.20839400519</v>
+        <v>12755.33604394822</v>
       </c>
     </row>
     <row r="22">
@@ -971,7 +958,7 @@
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>35.26441483270555</v>
+        <v>35.47424134753999</v>
       </c>
     </row>
     <row r="23">
@@ -981,7 +968,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>0.5005405062720889</v>
+        <v>0.4802999042329335</v>
       </c>
     </row>
     <row r="24">
@@ -991,7 +978,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>5.311296099708194</v>
+        <v>5.161812191917783</v>
       </c>
     </row>
     <row r="25">
@@ -1001,7 +988,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>13.8415881565639</v>
+        <v>12.74665423801967</v>
       </c>
     </row>
     <row r="26">
@@ -1011,7 +998,7 @@
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>11.01879392351423</v>
+        <v>10.54941813151042</v>
       </c>
     </row>
     <row r="27">
@@ -1021,7 +1008,7 @@
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>98.01252910069057</v>
+        <v>88.31757817949567</v>
       </c>
     </row>
   </sheetData>
@@ -1598,14 +1585,14 @@
       </c>
       <c r="I4" s="15" t="inlineStr">
         <is>
-          <t>[0, 27, 30, 15, 28, 6, 0]</t>
+          <t>[0, 32, 23, 1, 15, 30, 0]</t>
         </is>
       </c>
       <c r="J4" s="16" t="n">
-        <v>4378</v>
+        <v>4680</v>
       </c>
       <c r="K4" s="17" t="n">
-        <v>74.87284755753305</v>
+        <v>76.40911280206747</v>
       </c>
       <c r="L4" s="15" t="b">
         <v>1</v>
@@ -1661,7 +1648,7 @@
         <v>0</v>
       </c>
       <c r="AA4" s="5" t="n">
-        <v>12.97952693301531</v>
+        <v>6.976744186046512</v>
       </c>
       <c r="AB4" s="5" t="n">
         <v>0</v>
@@ -1794,14 +1781,14 @@
       </c>
       <c r="I5" s="15" t="inlineStr">
         <is>
-          <t>[0, 32, 28, 30, 27, 0]</t>
+          <t>[0, 32, 23, 11, 28, 15, 30, 0]</t>
         </is>
       </c>
       <c r="J5" s="16" t="n">
-        <v>4731</v>
+        <v>4915</v>
       </c>
       <c r="K5" s="17" t="n">
-        <v>71.2255389720694</v>
+        <v>72.3529809644612</v>
       </c>
       <c r="L5" s="15" t="b">
         <v>1</v>
@@ -1857,7 +1844,7 @@
         <v>0</v>
       </c>
       <c r="AA5" s="5" t="n">
-        <v>14.69527587450415</v>
+        <v>11.37756941940137</v>
       </c>
       <c r="AB5" s="5" t="n">
         <v>0</v>
@@ -1990,14 +1977,14 @@
       </c>
       <c r="I6" s="15" t="inlineStr">
         <is>
-          <t>[0, 32, 28, 30, 27, 0]</t>
+          <t>[0, 32, 23, 11, 28, 15, 30, 0]</t>
         </is>
       </c>
       <c r="J6" s="16" t="n">
-        <v>4632</v>
+        <v>5063</v>
       </c>
       <c r="K6" s="17" t="n">
-        <v>71.2255389720694</v>
+        <v>72.3529809644612</v>
       </c>
       <c r="L6" s="15" t="b">
         <v>1</v>
@@ -2053,7 +2040,7 @@
         <v>0</v>
       </c>
       <c r="AA6" s="5" t="n">
-        <v>9.584227991411282</v>
+        <v>1.171188756587937</v>
       </c>
       <c r="AB6" s="5" t="n">
         <v>1.737263322272106</v>
@@ -2085,14 +2072,14 @@
       </c>
       <c r="AJ6" s="18" t="inlineStr">
         <is>
-          <t>[0, 32, 23, 11, 28, 15, 30, 0]</t>
+          <t>[0, 27, 30, 32, 28, 15, 0]</t>
         </is>
       </c>
       <c r="AK6" s="19" t="n">
-        <v>5063</v>
+        <v>4709</v>
       </c>
       <c r="AL6" s="20" t="n">
-        <v>72.3529809644612</v>
+        <v>72.72308136763814</v>
       </c>
       <c r="AM6" s="18" t="b">
         <v>1</v>
@@ -2143,7 +2130,7 @@
         <v>0</v>
       </c>
       <c r="BA6" s="5" t="n">
-        <v>1.171188756587937</v>
+        <v>8.081202420456764</v>
       </c>
       <c r="BB6" s="5" t="n">
         <v>4.25531914893617</v>
@@ -2186,14 +2173,14 @@
       </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
-          <t>[1, 15, 32, 23, 1]</t>
+          <t>[1, 16, 32, 23, 13, 1]</t>
         </is>
       </c>
       <c r="J7" s="16" t="n">
-        <v>4341</v>
+        <v>4621</v>
       </c>
       <c r="K7" s="17" t="n">
-        <v>67.5733073091066</v>
+        <v>71.91926033151391</v>
       </c>
       <c r="L7" s="15" t="b">
         <v>1</v>
@@ -2249,7 +2236,7 @@
         <v>0</v>
       </c>
       <c r="AA7" s="5" t="n">
-        <v>28.68408082799408</v>
+        <v>24.08411368490225</v>
       </c>
       <c r="AB7" s="5" t="n">
         <v>0</v>
@@ -2281,14 +2268,14 @@
       </c>
       <c r="AJ7" s="18" t="inlineStr">
         <is>
-          <t>[1, 17, 23, 11, 28, 15, 1]</t>
+          <t>[1, 12, 34, 23, 11, 13, 1]</t>
         </is>
       </c>
       <c r="AK7" s="19" t="n">
-        <v>5074</v>
+        <v>4740</v>
       </c>
       <c r="AL7" s="20" t="n">
-        <v>74.01125865514462</v>
+        <v>67.88438089958805</v>
       </c>
       <c r="AM7" s="18" t="b">
         <v>1</v>
@@ -2339,7 +2326,7 @@
         <v>0</v>
       </c>
       <c r="BA7" s="5" t="n">
-        <v>16.64202398554296</v>
+        <v>22.12912764908822</v>
       </c>
       <c r="BB7" s="5" t="n">
         <v>27.40266140956136</v>
@@ -2477,14 +2464,14 @@
       </c>
       <c r="AJ8" s="18" t="inlineStr">
         <is>
-          <t>[1, 32, 23, 13, 17, 12, 34, 1]</t>
+          <t>[1, 32, 16, 12, 34, 31, 17, 1]</t>
         </is>
       </c>
       <c r="AK8" s="19" t="n">
-        <v>5723</v>
+        <v>5827</v>
       </c>
       <c r="AL8" s="20" t="n">
-        <v>76.75203292600122</v>
+        <v>72.61736662008917</v>
       </c>
       <c r="AM8" s="18" t="b">
         <v>1</v>
@@ -2535,7 +2522,7 @@
         <v>0</v>
       </c>
       <c r="BA8" s="5" t="n">
-        <v>5.232654412982282</v>
+        <v>3.510514985924822</v>
       </c>
       <c r="BB8" s="5" t="n">
         <v>13.92614671303196</v>
@@ -2578,14 +2565,14 @@
       </c>
       <c r="I9" s="15" t="inlineStr">
         <is>
-          <t>[1, 23, 32, 16, 34, 31, 12, 1]</t>
+          <t>[1, 23, 32, 16, 12, 34, 31, 1]</t>
         </is>
       </c>
       <c r="J9" s="16" t="n">
-        <v>6000</v>
+        <v>5976</v>
       </c>
       <c r="K9" s="17" t="n">
-        <v>75.05137961520434</v>
+        <v>75.01421864387075</v>
       </c>
       <c r="L9" s="15" t="b">
         <v>1</v>
@@ -2641,7 +2628,7 @@
         <v>0</v>
       </c>
       <c r="AA9" s="5" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="AB9" s="5" t="n">
         <v>2.833333333333333</v>
@@ -2869,14 +2856,14 @@
       </c>
       <c r="AJ10" s="18" t="inlineStr">
         <is>
-          <t>[2, 18, 17, 23, 11, 13, 2]</t>
+          <t>[2, 17, 23, 13, 8, 18, 2]</t>
         </is>
       </c>
       <c r="AK10" s="19" t="n">
-        <v>5227</v>
+        <v>4922</v>
       </c>
       <c r="AL10" s="20" t="n">
-        <v>75.43232651457264</v>
+        <v>74.42240734974001</v>
       </c>
       <c r="AM10" s="18" t="b">
         <v>1</v>
@@ -2927,7 +2914,7 @@
         <v>0</v>
       </c>
       <c r="BA10" s="5" t="n">
-        <v>0</v>
+        <v>5.835087048019897</v>
       </c>
       <c r="BB10" s="5" t="n">
         <v>10.94317964415535</v>
@@ -2970,14 +2957,14 @@
       </c>
       <c r="I11" s="15" t="inlineStr">
         <is>
-          <t>[2, 13, 23, 11, 8, 18, 2]</t>
+          <t>[2, 23, 11, 13, 8, 18, 2]</t>
         </is>
       </c>
       <c r="J11" s="16" t="n">
-        <v>5209</v>
+        <v>4965</v>
       </c>
       <c r="K11" s="17" t="n">
-        <v>76.11688487342525</v>
+        <v>74.84235419102524</v>
       </c>
       <c r="L11" s="15" t="b">
         <v>1</v>
@@ -3033,7 +3020,7 @@
         <v>0</v>
       </c>
       <c r="AA11" s="5" t="n">
-        <v>0</v>
+        <v>4.684200422345939</v>
       </c>
       <c r="AB11" s="5" t="n">
         <v>0</v>
@@ -3754,14 +3741,14 @@
       </c>
       <c r="I15" s="15" t="inlineStr">
         <is>
-          <t>[3, 4, 14, 33, 3]</t>
+          <t>[3, 4, 10, 33, 3]</t>
         </is>
       </c>
       <c r="J15" s="16" t="n">
-        <v>2105</v>
+        <v>2278</v>
       </c>
       <c r="K15" s="17" t="n">
-        <v>76.12162017812862</v>
+        <v>69.57524485498676</v>
       </c>
       <c r="L15" s="15" t="b">
         <v>1</v>
@@ -3817,7 +3804,7 @@
         <v>0</v>
       </c>
       <c r="AA15" s="5" t="n">
-        <v>7.594381035996488</v>
+        <v>0</v>
       </c>
       <c r="AB15" s="5" t="n">
         <v>0</v>
@@ -4045,14 +4032,14 @@
       </c>
       <c r="AJ16" s="18" t="inlineStr">
         <is>
-          <t>[4, 14, 33, 3, 4]</t>
+          <t>[4, 33, 3, 14, 4]</t>
         </is>
       </c>
       <c r="AK16" s="19" t="n">
-        <v>2386</v>
+        <v>2013</v>
       </c>
       <c r="AL16" s="20" t="n">
-        <v>76.12162017812862</v>
+        <v>66.1231493674095</v>
       </c>
       <c r="AM16" s="18" t="b">
         <v>1</v>
@@ -4103,7 +4090,7 @@
         <v>0</v>
       </c>
       <c r="BA16" s="5" t="n">
-        <v>0</v>
+        <v>15.63285834031853</v>
       </c>
       <c r="BB16" s="5" t="n">
         <v>0</v>
@@ -5221,14 +5208,14 @@
       </c>
       <c r="AJ22" s="18" t="inlineStr">
         <is>
-          <t>[6, 28, 32, 23, 11, 24, 6]</t>
+          <t>[6, 32, 23, 11, 24, 6]</t>
         </is>
       </c>
       <c r="AK22" s="19" t="n">
-        <v>5126</v>
+        <v>5248</v>
       </c>
       <c r="AL22" s="20" t="n">
-        <v>72.19802163182189</v>
+        <v>68.63913955482947</v>
       </c>
       <c r="AM22" s="18" t="b">
         <v>1</v>
@@ -5279,7 +5266,7 @@
         <v>0</v>
       </c>
       <c r="BA22" s="5" t="n">
-        <v>6.254572055596196</v>
+        <v>4.023408924652524</v>
       </c>
       <c r="BB22" s="5" t="n">
         <v>4.023408924652524</v>
@@ -5322,14 +5309,14 @@
       </c>
       <c r="I23" s="15" t="inlineStr">
         <is>
-          <t>[6, 32, 15, 28, 24, 6]</t>
+          <t>[6, 15, 32, 28, 24, 6]</t>
         </is>
       </c>
       <c r="J23" s="16" t="n">
-        <v>4466</v>
+        <v>4321</v>
       </c>
       <c r="K23" s="17" t="n">
-        <v>73.35659403721718</v>
+        <v>76.91467601944998</v>
       </c>
       <c r="L23" s="15" t="b">
         <v>1</v>
@@ -5385,7 +5372,7 @@
         <v>0</v>
       </c>
       <c r="AA23" s="5" t="n">
-        <v>23.57973990417522</v>
+        <v>26.06091718001369</v>
       </c>
       <c r="AB23" s="5" t="n">
         <v>0</v>
@@ -5417,14 +5404,14 @@
       </c>
       <c r="AJ23" s="18" t="inlineStr">
         <is>
-          <t>[6, 11, 23, 1, 32, 30, 15, 28, 6]</t>
+          <t>[6, 28, 15, 32, 23, 11, 6]</t>
         </is>
       </c>
       <c r="AK23" s="19" t="n">
-        <v>5393</v>
+        <v>4641</v>
       </c>
       <c r="AL23" s="20" t="n">
-        <v>75.83384333344556</v>
+        <v>68.80721202182097</v>
       </c>
       <c r="AM23" s="18" t="b">
         <v>1</v>
@@ -5475,7 +5462,7 @@
         <v>0</v>
       </c>
       <c r="BA23" s="5" t="n">
-        <v>7.717316906228611</v>
+        <v>20.58521560574949</v>
       </c>
       <c r="BB23" s="5" t="n">
         <v>23.57973990417522</v>
@@ -5518,14 +5505,14 @@
       </c>
       <c r="I24" s="15" t="inlineStr">
         <is>
-          <t>[6, 32, 23, 11, 28, 6]</t>
+          <t>[6, 15, 32, 28, 24, 6]</t>
         </is>
       </c>
       <c r="J24" s="16" t="n">
-        <v>4369</v>
+        <v>4692</v>
       </c>
       <c r="K24" s="17" t="n">
-        <v>73.6113709824498</v>
+        <v>76.91467601944998</v>
       </c>
       <c r="L24" s="15" t="b">
         <v>1</v>
@@ -5581,7 +5568,7 @@
         <v>0</v>
       </c>
       <c r="AA24" s="5" t="n">
-        <v>14.88408338203779</v>
+        <v>8.59146697837522</v>
       </c>
       <c r="AB24" s="5" t="n">
         <v>2.824858757062147</v>
@@ -5809,14 +5796,14 @@
       </c>
       <c r="AJ25" s="18" t="inlineStr">
         <is>
-          <t>[7, 28, 23, 11, 24, 7]</t>
+          <t>[7, 11, 23, 28, 6, 7]</t>
         </is>
       </c>
       <c r="AK25" s="19" t="n">
-        <v>4621</v>
+        <v>4408</v>
       </c>
       <c r="AL25" s="20" t="n">
-        <v>75.83608168317812</v>
+        <v>76.42419966683862</v>
       </c>
       <c r="AM25" s="18" t="b">
         <v>1</v>
@@ -5867,7 +5854,7 @@
         <v>0</v>
       </c>
       <c r="BA25" s="5" t="n">
-        <v>1.555176821474223</v>
+        <v>6.092884533446954</v>
       </c>
       <c r="BB25" s="5" t="n">
         <v>1.555176821474223</v>
@@ -5910,14 +5897,14 @@
       </c>
       <c r="I26" s="15" t="inlineStr">
         <is>
-          <t>[7, 28, 24, 11, 6, 7]</t>
+          <t>[7, 28, 23, 11, 24, 7]</t>
         </is>
       </c>
       <c r="J26" s="16" t="n">
-        <v>4005</v>
+        <v>4317</v>
       </c>
       <c r="K26" s="17" t="n">
-        <v>73.95218729374309</v>
+        <v>75.83608168317812</v>
       </c>
       <c r="L26" s="15" t="b">
         <v>1</v>
@@ -5973,7 +5960,7 @@
         <v>0</v>
       </c>
       <c r="AA26" s="5" t="n">
-        <v>9.634476534296029</v>
+        <v>2.594765342960289</v>
       </c>
       <c r="AB26" s="5" t="n">
         <v>0</v>
@@ -6106,14 +6093,14 @@
       </c>
       <c r="I27" s="15" t="inlineStr">
         <is>
-          <t>[7, 23, 11, 24, 6, 7]</t>
+          <t>[7, 24, 6, 11, 13, 7]</t>
         </is>
       </c>
       <c r="J27" s="16" t="n">
-        <v>3287</v>
+        <v>3367</v>
       </c>
       <c r="K27" s="17" t="n">
-        <v>72.87174262696787</v>
+        <v>70.93372623736701</v>
       </c>
       <c r="L27" s="15" t="b">
         <v>1</v>
@@ -6169,7 +6156,7 @@
         <v>0</v>
       </c>
       <c r="AA27" s="5" t="n">
-        <v>8.107352530053118</v>
+        <v>5.870841487279844</v>
       </c>
       <c r="AB27" s="5" t="n">
         <v>0</v>
@@ -6302,14 +6289,14 @@
       </c>
       <c r="I28" s="15" t="inlineStr">
         <is>
-          <t>[8, 18, 11, 23, 13, 8]</t>
+          <t>[8, 18, 2, 13, 23, 11, 8]</t>
         </is>
       </c>
       <c r="J28" s="16" t="n">
-        <v>4539</v>
+        <v>5207</v>
       </c>
       <c r="K28" s="17" t="n">
-        <v>75.35012256935434</v>
+        <v>76.11688487342524</v>
       </c>
       <c r="L28" s="15" t="b">
         <v>1</v>
@@ -6365,7 +6352,7 @@
         <v>0</v>
       </c>
       <c r="AA28" s="5" t="n">
-        <v>12.82888419435375</v>
+        <v>0</v>
       </c>
       <c r="AB28" s="5" t="n">
         <v>0</v>
@@ -6397,14 +6384,14 @@
       </c>
       <c r="AJ28" s="18" t="inlineStr">
         <is>
-          <t>[8, 18, 2, 13, 23, 11, 8]</t>
+          <t>[8, 18, 11, 23, 13, 8]</t>
         </is>
       </c>
       <c r="AK28" s="19" t="n">
-        <v>5207</v>
+        <v>4539</v>
       </c>
       <c r="AL28" s="20" t="n">
-        <v>76.11688487342524</v>
+        <v>75.35012256935434</v>
       </c>
       <c r="AM28" s="18" t="b">
         <v>1</v>
@@ -6455,7 +6442,7 @@
         <v>0</v>
       </c>
       <c r="BA28" s="5" t="n">
-        <v>0</v>
+        <v>12.82888419435375</v>
       </c>
       <c r="BB28" s="5" t="n">
         <v>12.82888419435375</v>
@@ -8357,14 +8344,14 @@
       </c>
       <c r="AJ38" s="18" t="inlineStr">
         <is>
-          <t>[11, 13, 23, 1, 15, 28, 6, 11]</t>
+          <t>[11, 13, 17, 34, 12, 31, 1, 23, 11]</t>
         </is>
       </c>
       <c r="AK38" s="19" t="n">
-        <v>5088</v>
+        <v>6198</v>
       </c>
       <c r="AL38" s="20" t="n">
-        <v>76.9634944961675</v>
+        <v>72.92391473027244</v>
       </c>
       <c r="AM38" s="18" t="b">
         <v>1</v>
@@ -8415,7 +8402,7 @@
         <v>0</v>
       </c>
       <c r="BA38" s="5" t="n">
-        <v>17.90900290416263</v>
+        <v>0</v>
       </c>
       <c r="BB38" s="5" t="n">
         <v>23.71732817037754</v>
@@ -9046,14 +9033,14 @@
       </c>
       <c r="I42" s="15" t="inlineStr">
         <is>
-          <t>[12, 34, 16, 31, 1, 23, 17, 12]</t>
+          <t>[12, 34, 16, 32, 23, 1, 31, 12]</t>
         </is>
       </c>
       <c r="J42" s="16" t="n">
-        <v>5371</v>
+        <v>5455</v>
       </c>
       <c r="K42" s="17" t="n">
-        <v>76.09879587135731</v>
+        <v>75.53118521626949</v>
       </c>
       <c r="L42" s="15" t="b">
         <v>1</v>
@@ -9109,7 +9096,7 @@
         <v>0</v>
       </c>
       <c r="AA42" s="5" t="n">
-        <v>6.802012840534443</v>
+        <v>5.34443866041992</v>
       </c>
       <c r="AB42" s="5" t="n">
         <v>0</v>
@@ -9242,14 +9229,14 @@
       </c>
       <c r="I43" s="15" t="inlineStr">
         <is>
-          <t>[13, 23, 32, 16, 12, 34, 13]</t>
+          <t>[13, 24, 7, 6, 11, 23, 13]</t>
         </is>
       </c>
       <c r="J43" s="16" t="n">
-        <v>5378</v>
+        <v>4658</v>
       </c>
       <c r="K43" s="17" t="n">
-        <v>76.53013715791758</v>
+        <v>74.21799739424517</v>
       </c>
       <c r="L43" s="15" t="b">
         <v>1</v>
@@ -9305,7 +9292,7 @@
         <v>0</v>
       </c>
       <c r="AA43" s="5" t="n">
-        <v>7.689667009955373</v>
+        <v>20.04806041881222</v>
       </c>
       <c r="AB43" s="5" t="n">
         <v>0</v>
@@ -9438,14 +9425,14 @@
       </c>
       <c r="I44" s="15" t="inlineStr">
         <is>
-          <t>[13, 6, 24, 7, 13]</t>
+          <t>[13, 1, 16, 34, 12, 23, 13]</t>
         </is>
       </c>
       <c r="J44" s="16" t="n">
-        <v>4227</v>
+        <v>5237</v>
       </c>
       <c r="K44" s="17" t="n">
-        <v>70.66009204763162</v>
+        <v>76.5606625994937</v>
       </c>
       <c r="L44" s="15" t="b">
         <v>1</v>
@@ -9501,7 +9488,7 @@
         <v>0</v>
       </c>
       <c r="AA44" s="5" t="n">
-        <v>26.15303983228511</v>
+        <v>8.508036338225017</v>
       </c>
       <c r="AB44" s="5" t="n">
         <v>0.628930817610063</v>
@@ -9533,14 +9520,14 @@
       </c>
       <c r="AJ44" s="18" t="inlineStr">
         <is>
-          <t>[13, 17, 34, 31, 12, 1, 23, 11, 13]</t>
+          <t>[13, 1, 34, 31, 12, 23, 11, 13]</t>
         </is>
       </c>
       <c r="AK44" s="19" t="n">
-        <v>5688</v>
+        <v>5669</v>
       </c>
       <c r="AL44" s="20" t="n">
-        <v>72.6154835462869</v>
+        <v>76.56785031046195</v>
       </c>
       <c r="AM44" s="18" t="b">
         <v>1</v>
@@ -9591,7 +9578,7 @@
         <v>0</v>
       </c>
       <c r="BA44" s="5" t="n">
-        <v>0.628930817610063</v>
+        <v>0.9608665269042628</v>
       </c>
       <c r="BB44" s="5" t="n">
         <v>32.25017470300489</v>
@@ -9634,14 +9621,14 @@
       </c>
       <c r="I45" s="15" t="inlineStr">
         <is>
-          <t>[13, 6, 15, 28, 11, 23, 13]</t>
+          <t>[13, 1, 16, 31, 12, 34, 13]</t>
         </is>
       </c>
       <c r="J45" s="16" t="n">
-        <v>4718</v>
+        <v>5038</v>
       </c>
       <c r="K45" s="17" t="n">
-        <v>72.63224967453041</v>
+        <v>73.88913350076947</v>
       </c>
       <c r="L45" s="15" t="b">
         <v>1</v>
@@ -9697,7 +9684,7 @@
         <v>0</v>
       </c>
       <c r="AA45" s="5" t="n">
-        <v>14.49800652410294</v>
+        <v>8.698803914461761</v>
       </c>
       <c r="AB45" s="5" t="n">
         <v>2.482783617252628</v>
@@ -9729,14 +9716,14 @@
       </c>
       <c r="AJ45" s="18" t="inlineStr">
         <is>
-          <t>[13, 23, 1, 34, 16, 12, 13]</t>
+          <t>[13, 23, 17, 34, 16, 12, 13]</t>
         </is>
       </c>
       <c r="AK45" s="19" t="n">
-        <v>5378</v>
+        <v>5505</v>
       </c>
       <c r="AL45" s="20" t="n">
-        <v>73.81274093424776</v>
+        <v>76.56177386696466</v>
       </c>
       <c r="AM45" s="18" t="b">
         <v>1</v>
@@ -9787,7 +9774,7 @@
         <v>0</v>
       </c>
       <c r="BA45" s="5" t="n">
-        <v>2.537151141718014</v>
+        <v>0.2355926060166727</v>
       </c>
       <c r="BB45" s="5" t="n">
         <v>5.799202609641174</v>
@@ -10614,14 +10601,14 @@
       </c>
       <c r="I50" s="15" t="inlineStr">
         <is>
-          <t>[15, 32, 23, 11, 28, 15]</t>
+          <t>[15, 32, 16, 12, 30, 15]</t>
         </is>
       </c>
       <c r="J50" s="16" t="n">
-        <v>4327</v>
+        <v>4392</v>
       </c>
       <c r="K50" s="17" t="n">
-        <v>63.51717547150033</v>
+        <v>76.77296658569027</v>
       </c>
       <c r="L50" s="15" t="b">
         <v>1</v>
@@ -10677,7 +10664,7 @@
         <v>0</v>
       </c>
       <c r="AA50" s="5" t="n">
-        <v>15.35602503912363</v>
+        <v>14.08450704225352</v>
       </c>
       <c r="AB50" s="5" t="n">
         <v>2.36697965571205</v>
@@ -10810,14 +10797,14 @@
       </c>
       <c r="I51" s="15" t="inlineStr">
         <is>
-          <t>[15, 26, 27, 0, 32, 15]</t>
+          <t>[15, 27, 0, 32, 28, 15]</t>
         </is>
       </c>
       <c r="J51" s="16" t="n">
-        <v>4332</v>
+        <v>4333</v>
       </c>
       <c r="K51" s="17" t="n">
-        <v>74.40492599202177</v>
+        <v>71.81491701587888</v>
       </c>
       <c r="L51" s="15" t="b">
         <v>1</v>
@@ -10873,7 +10860,7 @@
         <v>0</v>
       </c>
       <c r="AA51" s="5" t="n">
-        <v>16.11154144074361</v>
+        <v>16.09217660728118</v>
       </c>
       <c r="AB51" s="5" t="n">
         <v>0</v>
@@ -11006,14 +10993,14 @@
       </c>
       <c r="I52" s="15" t="inlineStr">
         <is>
-          <t>[16, 31, 32, 23, 1, 12, 16]</t>
+          <t>[16, 34, 31, 23, 1, 32, 16]</t>
         </is>
       </c>
       <c r="J52" s="16" t="n">
-        <v>4863</v>
+        <v>5208</v>
       </c>
       <c r="K52" s="17" t="n">
-        <v>75.34279720288458</v>
+        <v>76.12972937908032</v>
       </c>
       <c r="L52" s="15" t="b">
         <v>1</v>
@@ -11069,7 +11056,7 @@
         <v>0</v>
       </c>
       <c r="AA52" s="5" t="n">
-        <v>16.75795960287573</v>
+        <v>10.85244779185211</v>
       </c>
       <c r="AB52" s="5" t="n">
         <v>0</v>
@@ -11101,14 +11088,14 @@
       </c>
       <c r="AJ52" s="18" t="inlineStr">
         <is>
-          <t>[16, 31, 34, 12, 23, 32, 16]</t>
+          <t>[16, 34, 31, 17, 1, 32, 16]</t>
         </is>
       </c>
       <c r="AK52" s="19" t="n">
-        <v>5501</v>
+        <v>5387</v>
       </c>
       <c r="AL52" s="20" t="n">
-        <v>74.87587820600167</v>
+        <v>70.70303143161941</v>
       </c>
       <c r="AM52" s="18" t="b">
         <v>1</v>
@@ -11159,7 +11146,7 @@
         <v>0</v>
       </c>
       <c r="BA52" s="5" t="n">
-        <v>5.837042108866827</v>
+        <v>7.788428620335501</v>
       </c>
       <c r="BB52" s="5" t="n">
         <v>19.89044847654913</v>
@@ -11297,14 +11284,14 @@
       </c>
       <c r="AJ53" s="18" t="inlineStr">
         <is>
-          <t>[16, 12, 34, 31, 23, 32, 16]</t>
+          <t>[16, 34, 31, 12, 17, 1, 32, 16]</t>
         </is>
       </c>
       <c r="AK53" s="19" t="n">
-        <v>5311</v>
+        <v>5401</v>
       </c>
       <c r="AL53" s="20" t="n">
-        <v>75.10551564821257</v>
+        <v>72.5721514654558</v>
       </c>
       <c r="AM53" s="18" t="b">
         <v>1</v>
@@ -11355,7 +11342,7 @@
         <v>0</v>
       </c>
       <c r="BA53" s="5" t="n">
-        <v>4.957050823192556</v>
+        <v>3.346456692913386</v>
       </c>
       <c r="BB53" s="5" t="n">
         <v>5.368647100930565</v>
@@ -11398,14 +11385,14 @@
       </c>
       <c r="I54" s="15" t="inlineStr">
         <is>
-          <t>[16, 32, 23, 1, 31, 12, 34, 16]</t>
+          <t>[16, 32, 23, 1, 12, 31, 16]</t>
         </is>
       </c>
       <c r="J54" s="16" t="n">
-        <v>5895</v>
+        <v>6011</v>
       </c>
       <c r="K54" s="17" t="n">
-        <v>75.53118521626951</v>
+        <v>66.93947477981855</v>
       </c>
       <c r="L54" s="15" t="b">
         <v>1</v>
@@ -11461,7 +11448,7 @@
         <v>0</v>
       </c>
       <c r="AA54" s="5" t="n">
-        <v>3.186073246838561</v>
+        <v>1.280998521924782</v>
       </c>
       <c r="AB54" s="5" t="n">
         <v>0</v>
@@ -11493,14 +11480,14 @@
       </c>
       <c r="AJ54" s="18" t="inlineStr">
         <is>
-          <t>[16, 32, 23, 1, 12, 34, 31, 16]</t>
+          <t>[16, 32, 23, 17, 34, 12, 31, 16]</t>
         </is>
       </c>
       <c r="AK54" s="19" t="n">
-        <v>6089</v>
+        <v>6037</v>
       </c>
       <c r="AL54" s="20" t="n">
-        <v>75.08232804674387</v>
+        <v>76.04276339993501</v>
       </c>
       <c r="AM54" s="18" t="b">
         <v>1</v>
@@ -11551,7 +11538,7 @@
         <v>0</v>
       </c>
       <c r="BA54" s="5" t="n">
-        <v>0</v>
+        <v>0.8539990146165216</v>
       </c>
       <c r="BB54" s="5" t="n">
         <v>0</v>
@@ -11594,14 +11581,14 @@
       </c>
       <c r="I55" s="15" t="inlineStr">
         <is>
-          <t>[17, 16, 31, 1, 23, 13, 17]</t>
+          <t>[17, 34, 16, 11, 23, 17]</t>
         </is>
       </c>
       <c r="J55" s="16" t="n">
-        <v>5179</v>
+        <v>4793</v>
       </c>
       <c r="K55" s="17" t="n">
-        <v>76.71388319613814</v>
+        <v>75.80977144016293</v>
       </c>
       <c r="L55" s="15" t="b">
         <v>1</v>
@@ -11657,7 +11644,7 @@
         <v>0</v>
       </c>
       <c r="AA55" s="5" t="n">
-        <v>8.69181946403385</v>
+        <v>15.49717912552891</v>
       </c>
       <c r="AB55" s="5" t="n">
         <v>0</v>
@@ -11689,14 +11676,14 @@
       </c>
       <c r="AJ55" s="18" t="inlineStr">
         <is>
-          <t>[17, 16, 12, 34, 31, 1, 23, 17]</t>
+          <t>[17, 34, 16, 12, 13, 23, 17]</t>
         </is>
       </c>
       <c r="AK55" s="19" t="n">
-        <v>5472</v>
+        <v>5348</v>
       </c>
       <c r="AL55" s="20" t="n">
-        <v>76.65732371352398</v>
+        <v>76.56177386696466</v>
       </c>
       <c r="AM55" s="18" t="b">
         <v>1</v>
@@ -11747,7 +11734,7 @@
         <v>0</v>
       </c>
       <c r="BA55" s="5" t="n">
-        <v>3.526093088857546</v>
+        <v>5.712270803949225</v>
       </c>
       <c r="BB55" s="5" t="n">
         <v>12.09449929478138</v>
@@ -11790,14 +11777,14 @@
       </c>
       <c r="I56" s="15" t="inlineStr">
         <is>
-          <t>[17, 23, 1, 16, 31, 34, 12, 17]</t>
+          <t>[17, 23, 1, 31, 16, 34, 12, 17]</t>
         </is>
       </c>
       <c r="J56" s="16" t="n">
-        <v>6048</v>
+        <v>6242</v>
       </c>
       <c r="K56" s="17" t="n">
-        <v>73.14600940832835</v>
+        <v>76.66421294816206</v>
       </c>
       <c r="L56" s="15" t="b">
         <v>1</v>
@@ -11853,7 +11840,7 @@
         <v>0</v>
       </c>
       <c r="AA56" s="5" t="n">
-        <v>6.493506493506493</v>
+        <v>3.494124922696351</v>
       </c>
       <c r="AB56" s="5" t="n">
         <v>0</v>
@@ -11885,14 +11872,14 @@
       </c>
       <c r="AJ56" s="18" t="inlineStr">
         <is>
-          <t>[17, 23, 1, 12, 34, 16, 31, 17]</t>
+          <t>[17, 23, 1, 34, 16, 31, 12, 17]</t>
         </is>
       </c>
       <c r="AK56" s="19" t="n">
-        <v>6468</v>
+        <v>6394</v>
       </c>
       <c r="AL56" s="20" t="n">
-        <v>76.77412151089311</v>
+        <v>74.59471662141485</v>
       </c>
       <c r="AM56" s="18" t="b">
         <v>1</v>
@@ -11943,7 +11930,7 @@
         <v>0</v>
       </c>
       <c r="BA56" s="5" t="n">
-        <v>0</v>
+        <v>1.144094001236858</v>
       </c>
       <c r="BB56" s="5" t="n">
         <v>30.70500927643785</v>
@@ -11986,14 +11973,14 @@
       </c>
       <c r="I57" s="15" t="inlineStr">
         <is>
-          <t>[17, 16, 34, 31, 12, 1, 23, 17]</t>
+          <t>[17, 16, 34, 12, 32, 1, 17]</t>
         </is>
       </c>
       <c r="J57" s="16" t="n">
-        <v>5215</v>
+        <v>4532</v>
       </c>
       <c r="K57" s="17" t="n">
-        <v>76.69448468485756</v>
+        <v>74.71425149128011</v>
       </c>
       <c r="L57" s="15" t="b">
         <v>1</v>
@@ -12049,7 +12036,7 @@
         <v>0</v>
       </c>
       <c r="AA57" s="5" t="n">
-        <v>5.388243831640057</v>
+        <v>17.77939042089985</v>
       </c>
       <c r="AB57" s="5" t="n">
         <v>0</v>
@@ -12081,14 +12068,14 @@
       </c>
       <c r="AJ57" s="18" t="inlineStr">
         <is>
-          <t>[17, 34, 16, 31, 12, 1, 23, 17]</t>
+          <t>[17, 34, 16, 31, 12, 32, 1, 17]</t>
         </is>
       </c>
       <c r="AK57" s="19" t="n">
-        <v>5195</v>
+        <v>5169</v>
       </c>
       <c r="AL57" s="20" t="n">
-        <v>70.20300405918695</v>
+        <v>74.89144463759284</v>
       </c>
       <c r="AM57" s="18" t="b">
         <v>1</v>
@@ -12139,7 +12126,7 @@
         <v>0</v>
       </c>
       <c r="BA57" s="5" t="n">
-        <v>5.751088534107402</v>
+        <v>6.222786647314949</v>
       </c>
       <c r="BB57" s="5" t="n">
         <v>28.37445573294629</v>
@@ -12277,14 +12264,14 @@
       </c>
       <c r="AJ58" s="18" t="inlineStr">
         <is>
-          <t>[18, 2, 13, 23, 11, 8, 18]</t>
+          <t>[18, 2, 17, 34, 12, 31, 18]</t>
         </is>
       </c>
       <c r="AK58" s="19" t="n">
-        <v>5233</v>
+        <v>4328</v>
       </c>
       <c r="AL58" s="20" t="n">
-        <v>76.11688487342524</v>
+        <v>76.13471282007607</v>
       </c>
       <c r="AM58" s="18" t="b">
         <v>1</v>
@@ -12335,7 +12322,7 @@
         <v>0</v>
       </c>
       <c r="BA58" s="5" t="n">
-        <v>0</v>
+        <v>17.29409516529715</v>
       </c>
       <c r="BB58" s="5" t="n">
         <v>20.46627173705332</v>
@@ -12378,14 +12365,14 @@
       </c>
       <c r="I59" s="15" t="inlineStr">
         <is>
-          <t>[18, 1, 23, 13, 2, 18]</t>
+          <t>[18, 2, 13, 8, 29, 18]</t>
         </is>
       </c>
       <c r="J59" s="16" t="n">
-        <v>3888</v>
+        <v>3968</v>
       </c>
       <c r="K59" s="17" t="n">
-        <v>72.29713270193817</v>
+        <v>69.18855473644203</v>
       </c>
       <c r="L59" s="15" t="b">
         <v>1</v>
@@ -12441,7 +12428,7 @@
         <v>0</v>
       </c>
       <c r="AA59" s="5" t="n">
-        <v>21.54963680387409</v>
+        <v>19.93543179983858</v>
       </c>
       <c r="AB59" s="5" t="n">
         <v>10.49233252623083</v>
@@ -12865,14 +12852,14 @@
       </c>
       <c r="AJ61" s="18" t="inlineStr">
         <is>
-          <t>[19, 22, 17, 12, 19]</t>
+          <t>[19, 34, 31, 12, 19]</t>
         </is>
       </c>
       <c r="AK61" s="19" t="n">
-        <v>3182</v>
+        <v>2261</v>
       </c>
       <c r="AL61" s="20" t="n">
-        <v>75.68771422256441</v>
+        <v>76.09960509860163</v>
       </c>
       <c r="AM61" s="18" t="b">
         <v>1</v>
@@ -12923,7 +12910,7 @@
         <v>0</v>
       </c>
       <c r="BA61" s="5" t="n">
-        <v>0</v>
+        <v>28.94406033940918</v>
       </c>
       <c r="BB61" s="5" t="n">
         <v>0</v>
@@ -15122,14 +15109,14 @@
       </c>
       <c r="I73" s="15" t="inlineStr">
         <is>
-          <t>[23, 1, 28, 24, 6, 11, 23]</t>
+          <t>[23, 11, 13, 1, 12, 31, 34, 23]</t>
         </is>
       </c>
       <c r="J73" s="16" t="n">
-        <v>4915</v>
+        <v>4941</v>
       </c>
       <c r="K73" s="17" t="n">
-        <v>74.74858517898794</v>
+        <v>74.42838266767468</v>
       </c>
       <c r="L73" s="15" t="b">
         <v>1</v>
@@ -15185,7 +15172,7 @@
         <v>0</v>
       </c>
       <c r="AA73" s="5" t="n">
-        <v>15.17086641353124</v>
+        <v>14.72212633759061</v>
       </c>
       <c r="AB73" s="5" t="n">
         <v>0</v>
@@ -15217,14 +15204,14 @@
       </c>
       <c r="AJ73" s="18" t="inlineStr">
         <is>
-          <t>[23, 11, 13, 1, 34, 12, 31, 23]</t>
+          <t>[23, 1, 16, 12, 34, 32, 23]</t>
         </is>
       </c>
       <c r="AK73" s="19" t="n">
-        <v>5127</v>
+        <v>5274</v>
       </c>
       <c r="AL73" s="20" t="n">
-        <v>76.87628149444748</v>
+        <v>74.0692681981388</v>
       </c>
       <c r="AM73" s="18" t="b">
         <v>1</v>
@@ -15275,7 +15262,7 @@
         <v>0</v>
       </c>
       <c r="BA73" s="5" t="n">
-        <v>11.51190887124612</v>
+        <v>8.974801518812564</v>
       </c>
       <c r="BB73" s="5" t="n">
         <v>11.51190887124612</v>
@@ -15318,14 +15305,14 @@
       </c>
       <c r="I74" s="15" t="inlineStr">
         <is>
-          <t>[23, 1, 15, 28, 24, 11, 23]</t>
+          <t>[23, 1, 15, 28, 6, 11, 13, 23]</t>
         </is>
       </c>
       <c r="J74" s="16" t="n">
-        <v>5416</v>
+        <v>5839</v>
       </c>
       <c r="K74" s="17" t="n">
-        <v>75.65980089436411</v>
+        <v>76.9634944961675</v>
       </c>
       <c r="L74" s="15" t="b">
         <v>1</v>
@@ -15381,7 +15368,7 @@
         <v>0</v>
       </c>
       <c r="AA74" s="5" t="n">
-        <v>13.88138018762919</v>
+        <v>7.155350612179996</v>
       </c>
       <c r="AB74" s="5" t="n">
         <v>0</v>
@@ -15413,14 +15400,14 @@
       </c>
       <c r="AJ74" s="18" t="inlineStr">
         <is>
-          <t>[23, 1, 12, 31, 34, 16, 32, 23]</t>
+          <t>[23, 1, 34, 16, 12, 32, 23]</t>
         </is>
       </c>
       <c r="AK74" s="19" t="n">
-        <v>6289</v>
+        <v>5826</v>
       </c>
       <c r="AL74" s="20" t="n">
-        <v>75.11269845882313</v>
+        <v>75.02393738956991</v>
       </c>
       <c r="AM74" s="18" t="b">
         <v>1</v>
@@ -15471,7 +15458,7 @@
         <v>0</v>
       </c>
       <c r="BA74" s="5" t="n">
-        <v>0</v>
+        <v>7.362060740976307</v>
       </c>
       <c r="BB74" s="5" t="n">
         <v>7.362060740976307</v>
@@ -15609,14 +15596,14 @@
       </c>
       <c r="AJ75" s="18" t="inlineStr">
         <is>
-          <t>[23, 17, 34, 31, 12, 1, 32, 23]</t>
+          <t>[23, 13, 17, 34, 12, 31, 32, 23]</t>
         </is>
       </c>
       <c r="AK75" s="19" t="n">
-        <v>5318</v>
+        <v>5687</v>
       </c>
       <c r="AL75" s="20" t="n">
-        <v>69.36592006350338</v>
+        <v>76.58381500748465</v>
       </c>
       <c r="AM75" s="18" t="b">
         <v>1</v>
@@ -15667,7 +15654,7 @@
         <v>0</v>
       </c>
       <c r="BA75" s="5" t="n">
-        <v>7.865557865557865</v>
+        <v>1.472626472626473</v>
       </c>
       <c r="BB75" s="5" t="n">
         <v>13.79071379071379</v>
@@ -15906,14 +15893,14 @@
       </c>
       <c r="I77" s="15" t="inlineStr">
         <is>
-          <t>[24, 6, 7, 28, 11, 24]</t>
+          <t>[24, 7, 11, 6, 28, 24]</t>
         </is>
       </c>
       <c r="J77" s="16" t="n">
-        <v>4177</v>
+        <v>4209</v>
       </c>
       <c r="K77" s="17" t="n">
-        <v>67.77527243161661</v>
+        <v>71.76697859884823</v>
       </c>
       <c r="L77" s="15" t="b">
         <v>1</v>
@@ -15969,7 +15956,7 @@
         <v>0</v>
       </c>
       <c r="AA77" s="5" t="n">
-        <v>19.71939265808188</v>
+        <v>19.1043628675764</v>
       </c>
       <c r="AB77" s="5" t="n">
         <v>0</v>
@@ -16001,14 +15988,14 @@
       </c>
       <c r="AJ77" s="18" t="inlineStr">
         <is>
-          <t>[24, 11, 23, 13, 28, 24]</t>
+          <t>[24, 11, 13, 23, 28, 24]</t>
         </is>
       </c>
       <c r="AK77" s="19" t="n">
-        <v>4327</v>
+        <v>4487</v>
       </c>
       <c r="AL77" s="20" t="n">
-        <v>66.6828000597107</v>
+        <v>64.88962354143958</v>
       </c>
       <c r="AM77" s="18" t="b">
         <v>1</v>
@@ -16059,7 +16046,7 @@
         <v>0</v>
       </c>
       <c r="BA77" s="5" t="n">
-        <v>16.83644051508745</v>
+        <v>13.76129156256006</v>
       </c>
       <c r="BB77" s="5" t="n">
         <v>10.78224101479915</v>
@@ -16197,14 +16184,14 @@
       </c>
       <c r="AJ78" s="18" t="inlineStr">
         <is>
-          <t>[24, 6, 13, 1, 23, 11, 24]</t>
+          <t>[24, 6, 32, 23, 13, 24]</t>
         </is>
       </c>
       <c r="AK78" s="19" t="n">
-        <v>4920</v>
+        <v>5406</v>
       </c>
       <c r="AL78" s="20" t="n">
-        <v>72.39237672163087</v>
+        <v>76.09168411593276</v>
       </c>
       <c r="AM78" s="18" t="b">
         <v>1</v>
@@ -16255,7 +16242,7 @@
         <v>0</v>
       </c>
       <c r="BA78" s="5" t="n">
-        <v>8.990011098779133</v>
+        <v>0</v>
       </c>
       <c r="BB78" s="5" t="n">
         <v>0</v>
@@ -16886,14 +16873,14 @@
       </c>
       <c r="I82" s="15" t="inlineStr">
         <is>
-          <t>[26, 32, 27, 0, 30, 26]</t>
+          <t>[26, 27, 15, 32, 0, 26]</t>
         </is>
       </c>
       <c r="J82" s="16" t="n">
-        <v>4002</v>
+        <v>4288</v>
       </c>
       <c r="K82" s="17" t="n">
-        <v>76.92218514933194</v>
+        <v>74.68825977151276</v>
       </c>
       <c r="L82" s="15" t="b">
         <v>1</v>
@@ -16949,7 +16936,7 @@
         <v>0</v>
       </c>
       <c r="AA82" s="5" t="n">
-        <v>16.46837820914214</v>
+        <v>10.49885201419328</v>
       </c>
       <c r="AB82" s="5" t="n">
         <v>0</v>
@@ -17082,14 +17069,14 @@
       </c>
       <c r="I83" s="15" t="inlineStr">
         <is>
-          <t>[26, 32, 30, 27, 0, 26]</t>
+          <t>[26, 30, 32, 15, 0, 27, 26]</t>
         </is>
       </c>
       <c r="J83" s="16" t="n">
-        <v>4225</v>
+        <v>4454</v>
       </c>
       <c r="K83" s="17" t="n">
-        <v>74.68578731833023</v>
+        <v>75.319443211999</v>
       </c>
       <c r="L83" s="15" t="b">
         <v>1</v>
@@ -17145,7 +17132,7 @@
         <v>0</v>
       </c>
       <c r="AA83" s="5" t="n">
-        <v>14.31758264043805</v>
+        <v>9.673494220239302</v>
       </c>
       <c r="AB83" s="5" t="n">
         <v>0</v>
@@ -17278,14 +17265,14 @@
       </c>
       <c r="I84" s="15" t="inlineStr">
         <is>
-          <t>[26, 32, 27, 0, 30, 26]</t>
+          <t>[26, 27, 0, 15, 32, 30, 26]</t>
         </is>
       </c>
       <c r="J84" s="16" t="n">
-        <v>4029</v>
+        <v>4616</v>
       </c>
       <c r="K84" s="17" t="n">
-        <v>76.92218514933194</v>
+        <v>75.5383145684329</v>
       </c>
       <c r="L84" s="15" t="b">
         <v>1</v>
@@ -17341,7 +17328,7 @@
         <v>0</v>
       </c>
       <c r="AA84" s="5" t="n">
-        <v>13.07443365695793</v>
+        <v>0.4099244875943905</v>
       </c>
       <c r="AB84" s="5" t="n">
         <v>0</v>
@@ -17373,14 +17360,14 @@
       </c>
       <c r="AJ84" s="18" t="inlineStr">
         <is>
-          <t>[26, 27, 0, 15, 32, 30, 26]</t>
+          <t>[26, 27, 0, 32, 15, 30, 26]</t>
         </is>
       </c>
       <c r="AK84" s="19" t="n">
-        <v>4616</v>
+        <v>4635</v>
       </c>
       <c r="AL84" s="20" t="n">
-        <v>75.5383145684329</v>
+        <v>74.58649448949348</v>
       </c>
       <c r="AM84" s="18" t="b">
         <v>1</v>
@@ -17431,7 +17418,7 @@
         <v>0</v>
       </c>
       <c r="BA84" s="5" t="n">
-        <v>0.4099244875943905</v>
+        <v>0</v>
       </c>
       <c r="BB84" s="5" t="n">
         <v>4.681769147788565</v>
@@ -17670,14 +17657,14 @@
       </c>
       <c r="I86" s="15" t="inlineStr">
         <is>
-          <t>[27, 15, 26, 0, 27]</t>
+          <t>[27, 0, 26, 30, 15, 27]</t>
         </is>
       </c>
       <c r="J86" s="16" t="n">
-        <v>3245</v>
+        <v>3678</v>
       </c>
       <c r="K86" s="17" t="n">
-        <v>71.81044143013141</v>
+        <v>72.11445761460965</v>
       </c>
       <c r="L86" s="15" t="b">
         <v>1</v>
@@ -17733,7 +17720,7 @@
         <v>0</v>
       </c>
       <c r="AA86" s="5" t="n">
-        <v>33.12036273701566</v>
+        <v>24.1962077493817</v>
       </c>
       <c r="AB86" s="5" t="n">
         <v>0</v>
@@ -17765,14 +17752,14 @@
       </c>
       <c r="AJ86" s="18" t="inlineStr">
         <is>
-          <t>[27, 0, 32, 1, 15, 30, 27]</t>
+          <t>[27, 0, 32, 28, 15, 30, 27]</t>
         </is>
       </c>
       <c r="AK86" s="19" t="n">
-        <v>4852</v>
+        <v>4761</v>
       </c>
       <c r="AL86" s="20" t="n">
-        <v>76.98869770383878</v>
+        <v>71.99648707255528</v>
       </c>
       <c r="AM86" s="18" t="b">
         <v>1</v>
@@ -17823,7 +17810,7 @@
         <v>0</v>
       </c>
       <c r="BA86" s="5" t="n">
-        <v>0</v>
+        <v>1.875515251442704</v>
       </c>
       <c r="BB86" s="5" t="n">
         <v>0</v>
@@ -17866,14 +17853,14 @@
       </c>
       <c r="I87" s="15" t="inlineStr">
         <is>
-          <t>[27, 30, 32, 28, 15, 0, 27]</t>
+          <t>[27, 30, 32, 28, 27]</t>
         </is>
       </c>
       <c r="J87" s="16" t="n">
-        <v>4987</v>
+        <v>4340</v>
       </c>
       <c r="K87" s="17" t="n">
-        <v>72.72308136763816</v>
+        <v>72.87042754916699</v>
       </c>
       <c r="L87" s="15" t="b">
         <v>1</v>
@@ -17929,7 +17916,7 @@
         <v>0</v>
       </c>
       <c r="AA87" s="5" t="n">
-        <v>0</v>
+        <v>12.97373170242631</v>
       </c>
       <c r="AB87" s="5" t="n">
         <v>-0.08020854220974534</v>
@@ -18062,14 +18049,14 @@
       </c>
       <c r="I88" s="15" t="inlineStr">
         <is>
-          <t>[28, 6, 27, 0, 30, 15, 28]</t>
+          <t>[28, 27, 0, 15, 6, 28]</t>
         </is>
       </c>
       <c r="J88" s="16" t="n">
-        <v>4946</v>
+        <v>4707</v>
       </c>
       <c r="K88" s="17" t="n">
-        <v>74.8499243526344</v>
+        <v>74.48323704856701</v>
       </c>
       <c r="L88" s="15" t="b">
         <v>1</v>
@@ -18125,7 +18112,7 @@
         <v>0</v>
       </c>
       <c r="AA88" s="5" t="n">
-        <v>7.169669669669669</v>
+        <v>11.65540540540541</v>
       </c>
       <c r="AB88" s="5" t="n">
         <v>3.190690690690691</v>
@@ -18157,14 +18144,14 @@
       </c>
       <c r="AJ88" s="18" t="inlineStr">
         <is>
-          <t>[28, 15, 32, 23, 11, 6, 28]</t>
+          <t>[28, 27, 0, 30, 15, 6, 28]</t>
         </is>
       </c>
       <c r="AK88" s="19" t="n">
-        <v>5028</v>
+        <v>4881</v>
       </c>
       <c r="AL88" s="20" t="n">
-        <v>68.80721202182097</v>
+        <v>74.78725345578877</v>
       </c>
       <c r="AM88" s="18" t="b">
         <v>1</v>
@@ -18215,7 +18202,7 @@
         <v>0</v>
       </c>
       <c r="BA88" s="5" t="n">
-        <v>5.63063063063063</v>
+        <v>8.38963963963964</v>
       </c>
       <c r="BB88" s="5" t="n">
         <v>7.169669669669669</v>
@@ -18454,14 +18441,14 @@
       </c>
       <c r="I90" s="15" t="inlineStr">
         <is>
-          <t>[28, 32, 23, 11, 24, 6, 28]</t>
+          <t>[28, 30, 27, 0, 32, 15, 28]</t>
         </is>
       </c>
       <c r="J90" s="16" t="n">
-        <v>4468</v>
+        <v>4948</v>
       </c>
       <c r="K90" s="17" t="n">
-        <v>72.19802163182189</v>
+        <v>76.11262178500536</v>
       </c>
       <c r="L90" s="15" t="b">
         <v>1</v>
@@ -18517,7 +18504,7 @@
         <v>0</v>
       </c>
       <c r="AA90" s="5" t="n">
-        <v>12.32339089481947</v>
+        <v>2.904238618524333</v>
       </c>
       <c r="AB90" s="5" t="n">
         <v>0</v>
@@ -18549,14 +18536,14 @@
       </c>
       <c r="AJ90" s="18" t="inlineStr">
         <is>
-          <t>[28, 30, 27, 0, 32, 15, 28]</t>
+          <t>[28, 30, 26, 27, 0, 15, 28]</t>
         </is>
       </c>
       <c r="AK90" s="19" t="n">
-        <v>4948</v>
+        <v>4653</v>
       </c>
       <c r="AL90" s="20" t="n">
-        <v>76.11262178500536</v>
+        <v>67.88001534914439</v>
       </c>
       <c r="AM90" s="18" t="b">
         <v>1</v>
@@ -18607,7 +18594,7 @@
         <v>0</v>
       </c>
       <c r="BA90" s="5" t="n">
-        <v>2.904238618524333</v>
+        <v>8.69309262166405</v>
       </c>
       <c r="BB90" s="5" t="n">
         <v>12.32339089481947</v>
@@ -19042,14 +19029,14 @@
       </c>
       <c r="I93" s="15" t="inlineStr">
         <is>
-          <t>[29, 18, 2, 13, 8, 29]</t>
+          <t>[29, 11, 13, 8, 29]</t>
         </is>
       </c>
       <c r="J93" s="16" t="n">
-        <v>3377</v>
+        <v>3356</v>
       </c>
       <c r="K93" s="17" t="n">
-        <v>69.18855473644203</v>
+        <v>74.53326791831809</v>
       </c>
       <c r="L93" s="15" t="b">
         <v>1</v>
@@ -19105,7 +19092,7 @@
         <v>0</v>
       </c>
       <c r="AA93" s="5" t="n">
-        <v>18.35106382978723</v>
+        <v>18.85880077369439</v>
       </c>
       <c r="AB93" s="5" t="n">
         <v>0</v>
@@ -19137,14 +19124,14 @@
       </c>
       <c r="AJ93" s="18" t="inlineStr">
         <is>
-          <t>[29, 2, 13, 23, 29]</t>
+          <t>[29, 2, 18, 17, 8, 29]</t>
         </is>
       </c>
       <c r="AK93" s="19" t="n">
-        <v>3664</v>
+        <v>3401</v>
       </c>
       <c r="AL93" s="20" t="n">
-        <v>73.05730580690584</v>
+        <v>76.15648176800246</v>
       </c>
       <c r="AM93" s="18" t="b">
         <v>1</v>
@@ -19195,7 +19182,7 @@
         <v>0</v>
       </c>
       <c r="BA93" s="5" t="n">
-        <v>11.41199226305609</v>
+        <v>17.77079303675048</v>
       </c>
       <c r="BB93" s="5" t="n">
         <v>0</v>
@@ -19238,14 +19225,14 @@
       </c>
       <c r="I94" s="15" t="inlineStr">
         <is>
-          <t>[30, 32, 28, 0, 27, 30]</t>
+          <t>[30, 32, 16, 31, 12, 0, 30]</t>
         </is>
       </c>
       <c r="J94" s="16" t="n">
-        <v>4308</v>
+        <v>4620</v>
       </c>
       <c r="K94" s="17" t="n">
-        <v>73.12396826780835</v>
+        <v>75.39832271003269</v>
       </c>
       <c r="L94" s="15" t="b">
         <v>1</v>
@@ -19301,7 +19288,7 @@
         <v>0</v>
       </c>
       <c r="AA94" s="5" t="n">
-        <v>14.50684659654694</v>
+        <v>8.315141893232784</v>
       </c>
       <c r="AB94" s="5" t="n">
         <v>0</v>
@@ -19333,14 +19320,14 @@
       </c>
       <c r="AJ94" s="18" t="inlineStr">
         <is>
-          <t>[30, 32, 16, 31, 34, 1, 30]</t>
+          <t>[30, 27, 0, 32, 1, 15, 30]</t>
         </is>
       </c>
       <c r="AK94" s="19" t="n">
-        <v>4736</v>
+        <v>4813</v>
       </c>
       <c r="AL94" s="20" t="n">
-        <v>76.36835853210859</v>
+        <v>76.98869770383878</v>
       </c>
       <c r="AM94" s="18" t="b">
         <v>1</v>
@@ -19391,7 +19378,7 @@
         <v>0</v>
       </c>
       <c r="BA94" s="5" t="n">
-        <v>6.013097836872396</v>
+        <v>4.485016868426276</v>
       </c>
       <c r="BB94" s="5" t="n">
         <v>1.647152212740623</v>
@@ -19630,14 +19617,14 @@
       </c>
       <c r="I96" s="15" t="inlineStr">
         <is>
-          <t>[30, 27, 0, 15, 11, 28, 30]</t>
+          <t>[30, 32, 23, 11, 28, 15, 0, 30]</t>
         </is>
       </c>
       <c r="J96" s="16" t="n">
-        <v>4971</v>
+        <v>5274</v>
       </c>
       <c r="K96" s="17" t="n">
-        <v>76.91777059531171</v>
+        <v>73.08182586017075</v>
       </c>
       <c r="L96" s="15" t="b">
         <v>1</v>
@@ -19693,7 +19680,7 @@
         <v>0</v>
       </c>
       <c r="AA96" s="5" t="n">
-        <v>5.745164960182024</v>
+        <v>0</v>
       </c>
       <c r="AB96" s="5" t="n">
         <v>5.745164960182024</v>
@@ -19725,14 +19712,14 @@
       </c>
       <c r="AJ96" s="18" t="inlineStr">
         <is>
-          <t>[30, 27, 0, 15, 11, 28, 30]</t>
+          <t>[30, 32, 23, 11, 28, 15, 0, 30]</t>
         </is>
       </c>
       <c r="AK96" s="19" t="n">
-        <v>4971</v>
+        <v>5274</v>
       </c>
       <c r="AL96" s="20" t="n">
-        <v>76.91777059531171</v>
+        <v>73.08182586017075</v>
       </c>
       <c r="AM96" s="18" t="b">
         <v>1</v>
@@ -19783,7 +19770,7 @@
         <v>0</v>
       </c>
       <c r="BA96" s="5" t="n">
-        <v>5.745164960182024</v>
+        <v>0</v>
       </c>
       <c r="BB96" s="5" t="n">
         <v>9.878649981039061</v>
@@ -19826,14 +19813,14 @@
       </c>
       <c r="I97" s="15" t="inlineStr">
         <is>
-          <t>[31, 1, 23, 32, 16, 12, 34, 31]</t>
+          <t>[31, 16, 32, 23, 1, 12, 34, 31]</t>
         </is>
       </c>
       <c r="J97" s="16" t="n">
-        <v>6654</v>
+        <v>6177</v>
       </c>
       <c r="K97" s="17" t="n">
-        <v>75.01421864387075</v>
+        <v>75.08232804674387</v>
       </c>
       <c r="L97" s="15" t="b">
         <v>1</v>
@@ -19889,7 +19876,7 @@
         <v>0</v>
       </c>
       <c r="AA97" s="5" t="n">
-        <v>0</v>
+        <v>7.168620378719567</v>
       </c>
       <c r="AB97" s="5" t="n">
         <v>0</v>
@@ -20022,14 +20009,14 @@
       </c>
       <c r="I98" s="15" t="inlineStr">
         <is>
-          <t>[31, 23, 32, 16, 12, 34, 31]</t>
+          <t>[31, 23, 11, 13, 1, 34, 12, 31]</t>
         </is>
       </c>
       <c r="J98" s="16" t="n">
-        <v>5179</v>
+        <v>5476</v>
       </c>
       <c r="K98" s="17" t="n">
-        <v>75.10551564821257</v>
+        <v>76.87628149444748</v>
       </c>
       <c r="L98" s="15" t="b">
         <v>1</v>
@@ -20085,7 +20072,7 @@
         <v>0</v>
       </c>
       <c r="AA98" s="5" t="n">
-        <v>13.17686504610226</v>
+        <v>8.197820620284995</v>
       </c>
       <c r="AB98" s="5" t="n">
         <v>0.03352891869237217</v>
@@ -20117,14 +20104,14 @@
       </c>
       <c r="AJ98" s="18" t="inlineStr">
         <is>
-          <t>[31, 34, 16, 12, 1, 23, 17, 31]</t>
+          <t>[31, 34, 16, 32, 23, 1, 12, 31]</t>
         </is>
       </c>
       <c r="AK98" s="19" t="n">
-        <v>5965</v>
+        <v>5831</v>
       </c>
       <c r="AL98" s="20" t="n">
-        <v>76.58623801160354</v>
+        <v>75.11269845882315</v>
       </c>
       <c r="AM98" s="18" t="b">
         <v>1</v>
@@ -20175,7 +20162,7 @@
         <v>0</v>
       </c>
       <c r="BA98" s="5" t="n">
-        <v>0</v>
+        <v>2.246437552388935</v>
       </c>
       <c r="BB98" s="5" t="n">
         <v>13.17686504610226</v>
@@ -20218,14 +20205,14 @@
       </c>
       <c r="I99" s="15" t="inlineStr">
         <is>
-          <t>[31, 23, 1, 32, 16, 34, 31]</t>
+          <t>[31, 23, 1, 17, 16, 12, 31]</t>
         </is>
       </c>
       <c r="J99" s="16" t="n">
-        <v>5381</v>
+        <v>5545</v>
       </c>
       <c r="K99" s="17" t="n">
-        <v>76.1297293790803</v>
+        <v>76.55501627375277</v>
       </c>
       <c r="L99" s="15" t="b">
         <v>1</v>
@@ -20281,7 +20268,7 @@
         <v>0</v>
       </c>
       <c r="AA99" s="5" t="n">
-        <v>11.21927074740142</v>
+        <v>8.513446625969312</v>
       </c>
       <c r="AB99" s="5" t="n">
         <v>0</v>
@@ -20414,14 +20401,14 @@
       </c>
       <c r="I100" s="15" t="inlineStr">
         <is>
-          <t>[32, 16, 0, 27, 30, 32]</t>
+          <t>[32, 23, 11, 13, 17, 1, 32]</t>
         </is>
       </c>
       <c r="J100" s="16" t="n">
-        <v>4475</v>
+        <v>5057</v>
       </c>
       <c r="K100" s="17" t="n">
-        <v>76.30266589653552</v>
+        <v>72.25946588004804</v>
       </c>
       <c r="L100" s="15" t="b">
         <v>1</v>
@@ -20477,7 +20464,7 @@
         <v>0</v>
       </c>
       <c r="AA100" s="5" t="n">
-        <v>25.49117549117549</v>
+        <v>15.8008658008658</v>
       </c>
       <c r="AB100" s="5" t="n">
         <v>5.328005328005328</v>
@@ -20509,14 +20496,14 @@
       </c>
       <c r="AJ100" s="18" t="inlineStr">
         <is>
-          <t>[32, 16, 12, 34, 31, 1, 23, 32]</t>
+          <t>[32, 16, 34, 31, 12, 1, 23, 32]</t>
         </is>
       </c>
       <c r="AK100" s="19" t="n">
-        <v>5853</v>
+        <v>5575</v>
       </c>
       <c r="AL100" s="20" t="n">
-        <v>75.01421864387075</v>
+        <v>75.05137961520435</v>
       </c>
       <c r="AM100" s="18" t="b">
         <v>1</v>
@@ -20567,7 +20554,7 @@
         <v>0</v>
       </c>
       <c r="BA100" s="5" t="n">
-        <v>2.547452547452548</v>
+        <v>7.176157176157176</v>
       </c>
       <c r="BB100" s="5" t="n">
         <v>19.3972693972694</v>
@@ -20610,14 +20597,14 @@
       </c>
       <c r="I101" s="15" t="inlineStr">
         <is>
-          <t>[32, 23, 11, 6, 28, 15, 30, 32]</t>
+          <t>[32, 23, 11, 28, 15, 0, 30, 32]</t>
         </is>
       </c>
       <c r="J101" s="16" t="n">
-        <v>5249</v>
+        <v>5180</v>
       </c>
       <c r="K101" s="17" t="n">
-        <v>72.46790103387276</v>
+        <v>73.08182586017077</v>
       </c>
       <c r="L101" s="15" t="b">
         <v>1</v>
@@ -20673,7 +20660,7 @@
         <v>0</v>
       </c>
       <c r="AA101" s="5" t="n">
-        <v>5.847533632286996</v>
+        <v>7.085201793721973</v>
       </c>
       <c r="AB101" s="5" t="n">
         <v>1.991031390134529</v>
@@ -20901,14 +20888,14 @@
       </c>
       <c r="AJ102" s="18" t="inlineStr">
         <is>
-          <t>[32, 16, 12, 34, 31, 23, 32]</t>
+          <t>[32, 28, 27, 0, 30, 32]</t>
         </is>
       </c>
       <c r="AK102" s="19" t="n">
-        <v>5679</v>
+        <v>4717</v>
       </c>
       <c r="AL102" s="20" t="n">
-        <v>75.10551564821256</v>
+        <v>73.10104639937089</v>
       </c>
       <c r="AM102" s="18" t="b">
         <v>1</v>
@@ -20959,7 +20946,7 @@
         <v>0</v>
       </c>
       <c r="BA102" s="5" t="n">
-        <v>6.702809265648102</v>
+        <v>22.50698209298505</v>
       </c>
       <c r="BB102" s="5" t="n">
         <v>2.365697387875801</v>
@@ -21786,14 +21773,14 @@
       </c>
       <c r="I107" s="15" t="inlineStr">
         <is>
-          <t>[34, 16, 31, 32, 1, 17, 34]</t>
+          <t>[34, 23, 11, 13, 1, 12, 31, 34]</t>
         </is>
       </c>
       <c r="J107" s="16" t="n">
-        <v>4996</v>
+        <v>5505</v>
       </c>
       <c r="K107" s="17" t="n">
-        <v>72.80185862639158</v>
+        <v>74.42838266767468</v>
       </c>
       <c r="L107" s="15" t="b">
         <v>1</v>
@@ -21849,7 +21836,7 @@
         <v>0</v>
       </c>
       <c r="AA107" s="5" t="n">
-        <v>11.9647577092511</v>
+        <v>2.995594713656387</v>
       </c>
       <c r="AB107" s="5" t="n">
         <v>0.2819383259911895</v>
@@ -21982,14 +21969,14 @@
       </c>
       <c r="I108" s="15" t="inlineStr">
         <is>
-          <t>[34, 23, 32, 16, 31, 12, 34]</t>
+          <t>[34, 16, 11, 23, 17, 34]</t>
         </is>
       </c>
       <c r="J108" s="16" t="n">
-        <v>5489</v>
+        <v>5028</v>
       </c>
       <c r="K108" s="17" t="n">
-        <v>71.19715699148207</v>
+        <v>75.80977144016293</v>
       </c>
       <c r="L108" s="15" t="b">
         <v>1</v>
@@ -22045,7 +22032,7 @@
         <v>0</v>
       </c>
       <c r="AA108" s="5" t="n">
-        <v>9.942575881870386</v>
+        <v>17.50615258408532</v>
       </c>
       <c r="AB108" s="5" t="n">
         <v>0</v>
@@ -22077,14 +22064,14 @@
       </c>
       <c r="AJ108" s="18" t="inlineStr">
         <is>
-          <t>[34, 16, 31, 1, 23, 17, 12, 34]</t>
+          <t>[34, 31, 16, 12, 23, 17, 34]</t>
         </is>
       </c>
       <c r="AK108" s="19" t="n">
-        <v>5297</v>
+        <v>4936</v>
       </c>
       <c r="AL108" s="20" t="n">
-        <v>76.0987958713573</v>
+        <v>69.93579290188146</v>
       </c>
       <c r="AM108" s="18" t="b">
         <v>1</v>
@@ -22135,7 +22122,7 @@
         <v>0</v>
       </c>
       <c r="BA108" s="5" t="n">
-        <v>13.09269893355209</v>
+        <v>19.01558654634947</v>
       </c>
       <c r="BB108" s="5" t="n">
         <v>9.942575881870386</v>
@@ -22242,19 +22229,19 @@
         <v>105</v>
       </c>
       <c r="D2" t="n">
-        <v>4417.114285714286</v>
+        <v>4368.409523809524</v>
       </c>
       <c r="E2" t="n">
-        <v>1440.056377864621</v>
+        <v>1444.89232826984</v>
       </c>
       <c r="F2" t="n">
         <v>3287</v>
       </c>
       <c r="G2" t="n">
-        <v>4971</v>
+        <v>4807</v>
       </c>
       <c r="H2" t="n">
-        <v>5378</v>
+        <v>5401</v>
       </c>
       <c r="I2" t="n">
         <v>555</v>
@@ -22431,19 +22418,19 @@
         <v>105</v>
       </c>
       <c r="C2" t="n">
-        <v>1664.019047619048</v>
+        <v>1615.314285714286</v>
       </c>
       <c r="D2" t="n">
-        <v>1532</v>
+        <v>1446</v>
       </c>
       <c r="E2" t="n">
-        <v>1066.989302997281</v>
+        <v>1071.901637944719</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G2" t="n">
-        <v>5.696893031494331e-18</v>
+        <v>7.495318477697979e-18</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -22459,19 +22446,19 @@
         <v>105</v>
       </c>
       <c r="C3" t="n">
-        <v>294.4</v>
+        <v>245.6952380952381</v>
       </c>
       <c r="D3" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>522.8964561422786</v>
+        <v>554.8742602505947</v>
       </c>
       <c r="F3" t="n">
-        <v>324.5</v>
+        <v>504</v>
       </c>
       <c r="G3" t="n">
-        <v>2.16396247952928e-07</v>
+        <v>1.547226029143255e-05</v>
       </c>
       <c r="H3" t="b">
         <v>1</v>
@@ -22487,19 +22474,19 @@
         <v>105</v>
       </c>
       <c r="C4" t="n">
-        <v>331.4</v>
+        <v>282.6952380952381</v>
       </c>
       <c r="D4" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>579.9333781365953</v>
+        <v>608.5012186924388</v>
       </c>
       <c r="F4" t="n">
-        <v>215</v>
+        <v>420</v>
       </c>
       <c r="G4" t="n">
-        <v>2.954302153547962e-09</v>
+        <v>1.483612052518317e-06</v>
       </c>
       <c r="H4" t="b">
         <v>1</v>
@@ -22855,7 +22842,7 @@
         <v>50</v>
       </c>
       <c r="D14" s="38" t="n">
-        <v>0.000174</v>
+        <v>5.4e-05</v>
       </c>
       <c r="E14" s="39" t="n">
         <v>0.001</v>
@@ -22866,10 +22853,10 @@
         </is>
       </c>
       <c r="G14" s="41" t="n">
-        <v>0.8488</v>
+        <v>0.8683999999999999</v>
       </c>
       <c r="H14" s="38" t="n">
-        <v>0.000132</v>
+        <v>0.000245</v>
       </c>
       <c r="I14" s="42" t="n">
         <v>0.5</v>
@@ -22880,18 +22867,18 @@
         </is>
       </c>
       <c r="K14" s="41" t="n">
-        <v>0.26</v>
+        <v>0</v>
       </c>
       <c r="L14" s="42" t="n">
         <v>0.05</v>
       </c>
-      <c r="M14" s="43" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="M14" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="N14" s="38" t="n">
-        <v>0.000314</v>
+        <v>0.000471</v>
       </c>
       <c r="O14" s="39" t="n">
         <v>0.0005</v>
@@ -22901,9 +22888,9 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="Q14" s="44" t="inlineStr">
-        <is>
-          <t>NO — extender entrenamiento</t>
+      <c r="Q14" s="43" t="inlineStr">
+        <is>
+          <t>SÍ</t>
         </is>
       </c>
     </row>

</xml_diff>